<commit_message>
Actualización automática (Datos Provedores.xlsx): 26/08/06 09:04:30
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11654" uniqueCount="4911">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12043" uniqueCount="4912">
   <si>
     <t>Rut Proveedor</t>
   </si>
@@ -14752,6 +14752,9 @@
   </si>
   <si>
     <t>Fecha y Hora Actualización</t>
+  </si>
+  <si>
+    <t>26/08/06 09:04:30</t>
   </si>
 </sst>
 </file>
@@ -14816,14 +14819,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="22" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -14892,7 +14893,7 @@
         <name val="Calibri"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ h:mm"/>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="9" tint="0.79998168889431442"/>
@@ -16402,106 +16403,106 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="L1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="M1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="N1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="O1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="P1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="Q1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="7" t="s">
+      <c r="R1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="7" t="s">
+      <c r="S1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="T1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="7" t="s">
+      <c r="U1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="7" t="s">
+      <c r="V1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="7" t="s">
+      <c r="W1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="7" t="s">
+      <c r="X1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="7" t="s">
+      <c r="Y1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="7" t="s">
+      <c r="Z1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="7" t="s">
+      <c r="AA1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="7" t="s">
+      <c r="AB1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="7" t="s">
+      <c r="AC1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="7" t="s">
+      <c r="AD1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="7" t="s">
+      <c r="AE1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="7" t="s">
+      <c r="AF1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="7" t="s">
+      <c r="AG1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="7" t="s">
+      <c r="AH1" s="5" t="s">
         <v>4910</v>
       </c>
     </row>
@@ -16605,8 +16606,8 @@
       <c r="AG2" s="2">
         <v>13</v>
       </c>
-      <c r="AH2" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH2" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16709,8 +16710,8 @@
       <c r="AG3" s="4">
         <v>13</v>
       </c>
-      <c r="AH3" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH3" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16813,8 +16814,8 @@
       <c r="AG4" s="2">
         <v>13</v>
       </c>
-      <c r="AH4" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH4" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16917,8 +16918,8 @@
       <c r="AG5" s="4">
         <v>13</v>
       </c>
-      <c r="AH5" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH5" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17021,8 +17022,8 @@
       <c r="AG6" s="2">
         <v>13</v>
       </c>
-      <c r="AH6" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH6" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17125,8 +17126,8 @@
       <c r="AG7" s="4">
         <v>13</v>
       </c>
-      <c r="AH7" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH7" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17229,8 +17230,8 @@
       <c r="AG8" s="2">
         <v>13</v>
       </c>
-      <c r="AH8" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH8" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17333,8 +17334,8 @@
       <c r="AG9" s="4">
         <v>13</v>
       </c>
-      <c r="AH9" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH9" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17437,8 +17438,8 @@
       <c r="AG10" s="2">
         <v>13</v>
       </c>
-      <c r="AH10" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH10" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17541,8 +17542,8 @@
       <c r="AG11" s="4">
         <v>13</v>
       </c>
-      <c r="AH11" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH11" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17645,8 +17646,8 @@
       <c r="AG12" s="2">
         <v>13</v>
       </c>
-      <c r="AH12" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH12" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17749,8 +17750,8 @@
       <c r="AG13" s="4">
         <v>13</v>
       </c>
-      <c r="AH13" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH13" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17853,8 +17854,8 @@
       <c r="AG14" s="2">
         <v>13</v>
       </c>
-      <c r="AH14" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH14" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17957,8 +17958,8 @@
       <c r="AG15" s="4">
         <v>13</v>
       </c>
-      <c r="AH15" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH15" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18061,8 +18062,8 @@
       <c r="AG16" s="2">
         <v>13</v>
       </c>
-      <c r="AH16" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH16" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18165,8 +18166,8 @@
       <c r="AG17" s="4">
         <v>13</v>
       </c>
-      <c r="AH17" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH17" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18269,8 +18270,8 @@
       <c r="AG18" s="2">
         <v>13</v>
       </c>
-      <c r="AH18" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH18" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18373,8 +18374,8 @@
       <c r="AG19" s="4">
         <v>13</v>
       </c>
-      <c r="AH19" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH19" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18477,8 +18478,8 @@
       <c r="AG20" s="2">
         <v>13</v>
       </c>
-      <c r="AH20" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH20" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18581,8 +18582,8 @@
       <c r="AG21" s="4">
         <v>13</v>
       </c>
-      <c r="AH21" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH21" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18685,8 +18686,8 @@
       <c r="AG22" s="2">
         <v>13</v>
       </c>
-      <c r="AH22" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH22" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18789,8 +18790,8 @@
       <c r="AG23" s="4">
         <v>13</v>
       </c>
-      <c r="AH23" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH23" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18893,8 +18894,8 @@
       <c r="AG24" s="2">
         <v>13</v>
       </c>
-      <c r="AH24" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH24" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -18997,8 +18998,8 @@
       <c r="AG25" s="4">
         <v>13</v>
       </c>
-      <c r="AH25" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH25" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19101,8 +19102,8 @@
       <c r="AG26" s="2">
         <v>13</v>
       </c>
-      <c r="AH26" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH26" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19205,8 +19206,8 @@
       <c r="AG27" s="4">
         <v>13</v>
       </c>
-      <c r="AH27" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH27" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19309,8 +19310,8 @@
       <c r="AG28" s="2">
         <v>13</v>
       </c>
-      <c r="AH28" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH28" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19413,8 +19414,8 @@
       <c r="AG29" s="4">
         <v>5</v>
       </c>
-      <c r="AH29" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH29" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19517,8 +19518,8 @@
       <c r="AG30" s="2">
         <v>13</v>
       </c>
-      <c r="AH30" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH30" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19621,8 +19622,8 @@
       <c r="AG31" s="4">
         <v>13</v>
       </c>
-      <c r="AH31" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH31" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19725,8 +19726,8 @@
       <c r="AG32" s="2">
         <v>13</v>
       </c>
-      <c r="AH32" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH32" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19829,8 +19830,8 @@
       <c r="AG33" s="4">
         <v>13</v>
       </c>
-      <c r="AH33" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH33" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19933,8 +19934,8 @@
       <c r="AG34" s="2">
         <v>13</v>
       </c>
-      <c r="AH34" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH34" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20037,8 +20038,8 @@
       <c r="AG35" s="4">
         <v>13</v>
       </c>
-      <c r="AH35" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH35" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20141,8 +20142,8 @@
       <c r="AG36" s="2">
         <v>13</v>
       </c>
-      <c r="AH36" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH36" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20245,8 +20246,8 @@
       <c r="AG37" s="4">
         <v>13</v>
       </c>
-      <c r="AH37" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH37" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20349,8 +20350,8 @@
       <c r="AG38" s="2">
         <v>13</v>
       </c>
-      <c r="AH38" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH38" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20453,8 +20454,8 @@
       <c r="AG39" s="4">
         <v>13</v>
       </c>
-      <c r="AH39" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH39" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20557,8 +20558,8 @@
       <c r="AG40" s="2">
         <v>13</v>
       </c>
-      <c r="AH40" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH40" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20661,8 +20662,8 @@
       <c r="AG41" s="4">
         <v>13</v>
       </c>
-      <c r="AH41" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH41" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20765,8 +20766,8 @@
       <c r="AG42" s="2">
         <v>13</v>
       </c>
-      <c r="AH42" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH42" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20869,8 +20870,8 @@
       <c r="AG43" s="4">
         <v>13</v>
       </c>
-      <c r="AH43" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH43" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20973,8 +20974,8 @@
       <c r="AG44" s="2">
         <v>13</v>
       </c>
-      <c r="AH44" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH44" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21077,8 +21078,8 @@
       <c r="AG45" s="4">
         <v>13</v>
       </c>
-      <c r="AH45" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH45" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21181,8 +21182,8 @@
       <c r="AG46" s="2">
         <v>13</v>
       </c>
-      <c r="AH46" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH46" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21285,8 +21286,8 @@
       <c r="AG47" s="4">
         <v>13</v>
       </c>
-      <c r="AH47" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH47" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21389,8 +21390,8 @@
       <c r="AG48" s="2">
         <v>13</v>
       </c>
-      <c r="AH48" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH48" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21493,8 +21494,8 @@
       <c r="AG49" s="4">
         <v>13</v>
       </c>
-      <c r="AH49" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH49" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21597,8 +21598,8 @@
       <c r="AG50" s="2">
         <v>13</v>
       </c>
-      <c r="AH50" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH50" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21701,8 +21702,8 @@
       <c r="AG51" s="4">
         <v>6</v>
       </c>
-      <c r="AH51" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH51" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21805,8 +21806,8 @@
       <c r="AG52" s="2">
         <v>13</v>
       </c>
-      <c r="AH52" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH52" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21909,8 +21910,8 @@
       <c r="AG53" s="4">
         <v>13</v>
       </c>
-      <c r="AH53" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH53" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22013,8 +22014,8 @@
       <c r="AG54" s="2">
         <v>13</v>
       </c>
-      <c r="AH54" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH54" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22117,8 +22118,8 @@
       <c r="AG55" s="4">
         <v>13</v>
       </c>
-      <c r="AH55" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH55" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22221,8 +22222,8 @@
       <c r="AG56" s="2">
         <v>5</v>
       </c>
-      <c r="AH56" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH56" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22325,8 +22326,8 @@
       <c r="AG57" s="4">
         <v>13</v>
       </c>
-      <c r="AH57" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH57" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22429,8 +22430,8 @@
       <c r="AG58" s="2">
         <v>13</v>
       </c>
-      <c r="AH58" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH58" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22533,8 +22534,8 @@
       <c r="AG59" s="4">
         <v>13</v>
       </c>
-      <c r="AH59" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH59" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22637,8 +22638,8 @@
       <c r="AG60" s="2">
         <v>13</v>
       </c>
-      <c r="AH60" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH60" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22741,8 +22742,8 @@
       <c r="AG61" s="4">
         <v>13</v>
       </c>
-      <c r="AH61" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH61" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22845,8 +22846,8 @@
       <c r="AG62" s="2">
         <v>13</v>
       </c>
-      <c r="AH62" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH62" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22949,8 +22950,8 @@
       <c r="AG63" s="4">
         <v>13</v>
       </c>
-      <c r="AH63" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH63" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23053,8 +23054,8 @@
       <c r="AG64" s="2">
         <v>13</v>
       </c>
-      <c r="AH64" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH64" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23157,8 +23158,8 @@
       <c r="AG65" s="4">
         <v>13</v>
       </c>
-      <c r="AH65" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH65" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23261,8 +23262,8 @@
       <c r="AG66" s="2">
         <v>13</v>
       </c>
-      <c r="AH66" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH66" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23365,8 +23366,8 @@
       <c r="AG67" s="4">
         <v>13</v>
       </c>
-      <c r="AH67" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH67" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23469,8 +23470,8 @@
       <c r="AG68" s="2">
         <v>13</v>
       </c>
-      <c r="AH68" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH68" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23573,8 +23574,8 @@
       <c r="AG69" s="4">
         <v>13</v>
       </c>
-      <c r="AH69" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH69" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23677,8 +23678,8 @@
       <c r="AG70" s="2">
         <v>13</v>
       </c>
-      <c r="AH70" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH70" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23781,8 +23782,8 @@
       <c r="AG71" s="4">
         <v>13</v>
       </c>
-      <c r="AH71" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH71" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23885,8 +23886,8 @@
       <c r="AG72" s="2">
         <v>8</v>
       </c>
-      <c r="AH72" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH72" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23989,8 +23990,8 @@
       <c r="AG73" s="4">
         <v>5</v>
       </c>
-      <c r="AH73" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH73" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24093,8 +24094,8 @@
       <c r="AG74" s="2">
         <v>13</v>
       </c>
-      <c r="AH74" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH74" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24197,8 +24198,8 @@
       <c r="AG75" s="4">
         <v>5</v>
       </c>
-      <c r="AH75" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH75" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24301,8 +24302,8 @@
       <c r="AG76" s="2">
         <v>13</v>
       </c>
-      <c r="AH76" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH76" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24405,8 +24406,8 @@
       <c r="AG77" s="4">
         <v>13</v>
       </c>
-      <c r="AH77" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH77" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24509,8 +24510,8 @@
       <c r="AG78" s="2">
         <v>9</v>
       </c>
-      <c r="AH78" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH78" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24613,8 +24614,8 @@
       <c r="AG79" s="4">
         <v>13</v>
       </c>
-      <c r="AH79" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH79" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24717,8 +24718,8 @@
       <c r="AG80" s="2">
         <v>13</v>
       </c>
-      <c r="AH80" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH80" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24821,8 +24822,8 @@
       <c r="AG81" s="4">
         <v>13</v>
       </c>
-      <c r="AH81" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH81" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24925,8 +24926,8 @@
       <c r="AG82" s="2">
         <v>13</v>
       </c>
-      <c r="AH82" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH82" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25029,8 +25030,8 @@
       <c r="AG83" s="4">
         <v>13</v>
       </c>
-      <c r="AH83" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH83" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25133,8 +25134,8 @@
       <c r="AG84" s="2">
         <v>13</v>
       </c>
-      <c r="AH84" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH84" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25237,8 +25238,8 @@
       <c r="AG85" s="4">
         <v>13</v>
       </c>
-      <c r="AH85" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH85" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25341,8 +25342,8 @@
       <c r="AG86" s="2">
         <v>13</v>
       </c>
-      <c r="AH86" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH86" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25445,8 +25446,8 @@
       <c r="AG87" s="4">
         <v>13</v>
       </c>
-      <c r="AH87" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH87" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25549,8 +25550,8 @@
       <c r="AG88" s="2">
         <v>13</v>
       </c>
-      <c r="AH88" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH88" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25653,8 +25654,8 @@
       <c r="AG89" s="4">
         <v>13</v>
       </c>
-      <c r="AH89" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH89" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25757,8 +25758,8 @@
       <c r="AG90" s="2">
         <v>13</v>
       </c>
-      <c r="AH90" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH90" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25861,8 +25862,8 @@
       <c r="AG91" s="4">
         <v>13</v>
       </c>
-      <c r="AH91" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH91" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25965,8 +25966,8 @@
       <c r="AG92" s="2">
         <v>13</v>
       </c>
-      <c r="AH92" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH92" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26069,8 +26070,8 @@
       <c r="AG93" s="4">
         <v>13</v>
       </c>
-      <c r="AH93" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH93" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26173,8 +26174,8 @@
       <c r="AG94" s="2">
         <v>13</v>
       </c>
-      <c r="AH94" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH94" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26277,8 +26278,8 @@
       <c r="AG95" s="4">
         <v>13</v>
       </c>
-      <c r="AH95" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH95" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26381,8 +26382,8 @@
       <c r="AG96" s="2">
         <v>13</v>
       </c>
-      <c r="AH96" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH96" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26485,8 +26486,8 @@
       <c r="AG97" s="4">
         <v>13</v>
       </c>
-      <c r="AH97" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH97" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26589,8 +26590,8 @@
       <c r="AG98" s="2">
         <v>13</v>
       </c>
-      <c r="AH98" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH98" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26693,8 +26694,8 @@
       <c r="AG99" s="4">
         <v>13</v>
       </c>
-      <c r="AH99" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH99" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26797,8 +26798,8 @@
       <c r="AG100" s="2">
         <v>13</v>
       </c>
-      <c r="AH100" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH100" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26901,8 +26902,8 @@
       <c r="AG101" s="4">
         <v>13</v>
       </c>
-      <c r="AH101" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH101" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27005,8 +27006,8 @@
       <c r="AG102" s="2">
         <v>13</v>
       </c>
-      <c r="AH102" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH102" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27109,8 +27110,8 @@
       <c r="AG103" s="4">
         <v>13</v>
       </c>
-      <c r="AH103" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH103" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27213,8 +27214,8 @@
       <c r="AG104" s="2">
         <v>13</v>
       </c>
-      <c r="AH104" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH104" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27317,8 +27318,8 @@
       <c r="AG105" s="4">
         <v>13</v>
       </c>
-      <c r="AH105" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH105" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27421,8 +27422,8 @@
       <c r="AG106" s="2">
         <v>13</v>
       </c>
-      <c r="AH106" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH106" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27525,8 +27526,8 @@
       <c r="AG107" s="4">
         <v>13</v>
       </c>
-      <c r="AH107" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH107" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27629,8 +27630,8 @@
       <c r="AG108" s="2">
         <v>13</v>
       </c>
-      <c r="AH108" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH108" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27733,8 +27734,8 @@
       <c r="AG109" s="4">
         <v>13</v>
       </c>
-      <c r="AH109" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH109" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27837,8 +27838,8 @@
       <c r="AG110" s="2">
         <v>13</v>
       </c>
-      <c r="AH110" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH110" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27941,8 +27942,8 @@
       <c r="AG111" s="4">
         <v>13</v>
       </c>
-      <c r="AH111" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH111" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28045,8 +28046,8 @@
       <c r="AG112" s="2">
         <v>13</v>
       </c>
-      <c r="AH112" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH112" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28149,8 +28150,8 @@
       <c r="AG113" s="4">
         <v>13</v>
       </c>
-      <c r="AH113" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH113" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28253,8 +28254,8 @@
       <c r="AG114" s="2">
         <v>13</v>
       </c>
-      <c r="AH114" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH114" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28357,8 +28358,8 @@
       <c r="AG115" s="4">
         <v>13</v>
       </c>
-      <c r="AH115" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH115" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28461,8 +28462,8 @@
       <c r="AG116" s="2">
         <v>13</v>
       </c>
-      <c r="AH116" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH116" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28565,8 +28566,8 @@
       <c r="AG117" s="4">
         <v>5</v>
       </c>
-      <c r="AH117" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH117" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28669,8 +28670,8 @@
       <c r="AG118" s="2">
         <v>13</v>
       </c>
-      <c r="AH118" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH118" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28773,8 +28774,8 @@
       <c r="AG119" s="4">
         <v>13</v>
       </c>
-      <c r="AH119" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH119" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28877,8 +28878,8 @@
       <c r="AG120" s="2">
         <v>13</v>
       </c>
-      <c r="AH120" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH120" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28981,8 +28982,8 @@
       <c r="AG121" s="4">
         <v>13</v>
       </c>
-      <c r="AH121" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH121" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29085,8 +29086,8 @@
       <c r="AG122" s="2">
         <v>13</v>
       </c>
-      <c r="AH122" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH122" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29189,8 +29190,8 @@
       <c r="AG123" s="4">
         <v>13</v>
       </c>
-      <c r="AH123" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH123" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29293,8 +29294,8 @@
       <c r="AG124" s="2">
         <v>13</v>
       </c>
-      <c r="AH124" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH124" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29397,8 +29398,8 @@
       <c r="AG125" s="4">
         <v>13</v>
       </c>
-      <c r="AH125" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH125" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29501,8 +29502,8 @@
       <c r="AG126" s="2">
         <v>13</v>
       </c>
-      <c r="AH126" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH126" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29605,8 +29606,8 @@
       <c r="AG127" s="4">
         <v>13</v>
       </c>
-      <c r="AH127" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH127" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29709,8 +29710,8 @@
       <c r="AG128" s="2">
         <v>13</v>
       </c>
-      <c r="AH128" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH128" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29813,8 +29814,8 @@
       <c r="AG129" s="4">
         <v>13</v>
       </c>
-      <c r="AH129" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH129" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29917,8 +29918,8 @@
       <c r="AG130" s="2">
         <v>13</v>
       </c>
-      <c r="AH130" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH130" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30021,8 +30022,8 @@
       <c r="AG131" s="4">
         <v>5</v>
       </c>
-      <c r="AH131" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH131" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30125,8 +30126,8 @@
       <c r="AG132" s="2">
         <v>5</v>
       </c>
-      <c r="AH132" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH132" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30229,8 +30230,8 @@
       <c r="AG133" s="4">
         <v>13</v>
       </c>
-      <c r="AH133" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH133" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30333,8 +30334,8 @@
       <c r="AG134" s="2">
         <v>13</v>
       </c>
-      <c r="AH134" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH134" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30437,8 +30438,8 @@
       <c r="AG135" s="4">
         <v>13</v>
       </c>
-      <c r="AH135" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH135" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30541,8 +30542,8 @@
       <c r="AG136" s="2">
         <v>13</v>
       </c>
-      <c r="AH136" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH136" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30645,8 +30646,8 @@
       <c r="AG137" s="4">
         <v>13</v>
       </c>
-      <c r="AH137" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH137" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30749,8 +30750,8 @@
       <c r="AG138" s="2">
         <v>13</v>
       </c>
-      <c r="AH138" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH138" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30853,8 +30854,8 @@
       <c r="AG139" s="4">
         <v>13</v>
       </c>
-      <c r="AH139" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH139" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30957,8 +30958,8 @@
       <c r="AG140" s="2">
         <v>13</v>
       </c>
-      <c r="AH140" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH140" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31061,8 +31062,8 @@
       <c r="AG141" s="4">
         <v>13</v>
       </c>
-      <c r="AH141" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH141" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31165,8 +31166,8 @@
       <c r="AG142" s="2">
         <v>13</v>
       </c>
-      <c r="AH142" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH142" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31269,8 +31270,8 @@
       <c r="AG143" s="4">
         <v>13</v>
       </c>
-      <c r="AH143" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH143" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31373,8 +31374,8 @@
       <c r="AG144" s="2">
         <v>13</v>
       </c>
-      <c r="AH144" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH144" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31477,8 +31478,8 @@
       <c r="AG145" s="4">
         <v>13</v>
       </c>
-      <c r="AH145" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH145" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31581,8 +31582,8 @@
       <c r="AG146" s="2">
         <v>13</v>
       </c>
-      <c r="AH146" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH146" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31685,8 +31686,8 @@
       <c r="AG147" s="4">
         <v>13</v>
       </c>
-      <c r="AH147" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH147" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31789,8 +31790,8 @@
       <c r="AG148" s="2">
         <v>13</v>
       </c>
-      <c r="AH148" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH148" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31893,8 +31894,8 @@
       <c r="AG149" s="4">
         <v>13</v>
       </c>
-      <c r="AH149" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH149" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -31997,8 +31998,8 @@
       <c r="AG150" s="2">
         <v>13</v>
       </c>
-      <c r="AH150" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH150" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32101,8 +32102,8 @@
       <c r="AG151" s="4">
         <v>5</v>
       </c>
-      <c r="AH151" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH151" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32205,8 +32206,8 @@
       <c r="AG152" s="2">
         <v>13</v>
       </c>
-      <c r="AH152" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH152" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32309,8 +32310,8 @@
       <c r="AG153" s="4">
         <v>13</v>
       </c>
-      <c r="AH153" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH153" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32413,8 +32414,8 @@
       <c r="AG154" s="2">
         <v>13</v>
       </c>
-      <c r="AH154" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH154" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32517,8 +32518,8 @@
       <c r="AG155" s="4">
         <v>13</v>
       </c>
-      <c r="AH155" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH155" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32621,8 +32622,8 @@
       <c r="AG156" s="2">
         <v>13</v>
       </c>
-      <c r="AH156" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH156" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32725,8 +32726,8 @@
       <c r="AG157" s="4">
         <v>13</v>
       </c>
-      <c r="AH157" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH157" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32829,8 +32830,8 @@
       <c r="AG158" s="2">
         <v>13</v>
       </c>
-      <c r="AH158" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH158" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32933,8 +32934,8 @@
       <c r="AG159" s="4">
         <v>13</v>
       </c>
-      <c r="AH159" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH159" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33037,8 +33038,8 @@
       <c r="AG160" s="2">
         <v>13</v>
       </c>
-      <c r="AH160" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH160" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33141,8 +33142,8 @@
       <c r="AG161" s="4">
         <v>13</v>
       </c>
-      <c r="AH161" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH161" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33245,8 +33246,8 @@
       <c r="AG162" s="2">
         <v>13</v>
       </c>
-      <c r="AH162" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH162" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33349,8 +33350,8 @@
       <c r="AG163" s="4">
         <v>5</v>
       </c>
-      <c r="AH163" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH163" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33453,8 +33454,8 @@
       <c r="AG164" s="2">
         <v>13</v>
       </c>
-      <c r="AH164" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH164" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33557,8 +33558,8 @@
       <c r="AG165" s="4">
         <v>13</v>
       </c>
-      <c r="AH165" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH165" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33661,8 +33662,8 @@
       <c r="AG166" s="2">
         <v>13</v>
       </c>
-      <c r="AH166" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH166" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33765,8 +33766,8 @@
       <c r="AG167" s="4">
         <v>13</v>
       </c>
-      <c r="AH167" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH167" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33869,8 +33870,8 @@
       <c r="AG168" s="2">
         <v>13</v>
       </c>
-      <c r="AH168" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH168" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33973,8 +33974,8 @@
       <c r="AG169" s="4">
         <v>13</v>
       </c>
-      <c r="AH169" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH169" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34077,8 +34078,8 @@
       <c r="AG170" s="2">
         <v>13</v>
       </c>
-      <c r="AH170" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH170" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34181,8 +34182,8 @@
       <c r="AG171" s="4">
         <v>13</v>
       </c>
-      <c r="AH171" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH171" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34285,8 +34286,8 @@
       <c r="AG172" s="2">
         <v>13</v>
       </c>
-      <c r="AH172" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH172" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34389,8 +34390,8 @@
       <c r="AG173" s="4">
         <v>13</v>
       </c>
-      <c r="AH173" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH173" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34493,8 +34494,8 @@
       <c r="AG174" s="2">
         <v>13</v>
       </c>
-      <c r="AH174" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH174" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34597,8 +34598,8 @@
       <c r="AG175" s="4">
         <v>13</v>
       </c>
-      <c r="AH175" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH175" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34701,8 +34702,8 @@
       <c r="AG176" s="2">
         <v>13</v>
       </c>
-      <c r="AH176" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH176" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34805,8 +34806,8 @@
       <c r="AG177" s="4">
         <v>13</v>
       </c>
-      <c r="AH177" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH177" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34909,8 +34910,8 @@
       <c r="AG178" s="2">
         <v>13</v>
       </c>
-      <c r="AH178" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH178" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35013,8 +35014,8 @@
       <c r="AG179" s="4">
         <v>13</v>
       </c>
-      <c r="AH179" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH179" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35117,8 +35118,8 @@
       <c r="AG180" s="2">
         <v>13</v>
       </c>
-      <c r="AH180" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH180" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35221,8 +35222,8 @@
       <c r="AG181" s="4">
         <v>13</v>
       </c>
-      <c r="AH181" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH181" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35325,8 +35326,8 @@
       <c r="AG182" s="2">
         <v>6</v>
       </c>
-      <c r="AH182" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH182" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35429,8 +35430,8 @@
       <c r="AG183" s="4">
         <v>13</v>
       </c>
-      <c r="AH183" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH183" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35533,8 +35534,8 @@
       <c r="AG184" s="2">
         <v>13</v>
       </c>
-      <c r="AH184" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH184" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35637,8 +35638,8 @@
       <c r="AG185" s="4">
         <v>13</v>
       </c>
-      <c r="AH185" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH185" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35741,8 +35742,8 @@
       <c r="AG186" s="2">
         <v>13</v>
       </c>
-      <c r="AH186" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH186" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35845,8 +35846,8 @@
       <c r="AG187" s="4">
         <v>13</v>
       </c>
-      <c r="AH187" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH187" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35949,8 +35950,8 @@
       <c r="AG188" s="2">
         <v>5</v>
       </c>
-      <c r="AH188" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH188" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36053,8 +36054,8 @@
       <c r="AG189" s="4">
         <v>13</v>
       </c>
-      <c r="AH189" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH189" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36157,8 +36158,8 @@
       <c r="AG190" s="2">
         <v>13</v>
       </c>
-      <c r="AH190" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH190" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36261,8 +36262,8 @@
       <c r="AG191" s="4">
         <v>13</v>
       </c>
-      <c r="AH191" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH191" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36365,8 +36366,8 @@
       <c r="AG192" s="2">
         <v>7</v>
       </c>
-      <c r="AH192" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH192" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36469,8 +36470,8 @@
       <c r="AG193" s="4">
         <v>13</v>
       </c>
-      <c r="AH193" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH193" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36573,8 +36574,8 @@
       <c r="AG194" s="2">
         <v>13</v>
       </c>
-      <c r="AH194" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH194" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36677,8 +36678,8 @@
       <c r="AG195" s="4">
         <v>13</v>
       </c>
-      <c r="AH195" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH195" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36781,8 +36782,8 @@
       <c r="AG196" s="2">
         <v>13</v>
       </c>
-      <c r="AH196" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH196" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36885,8 +36886,8 @@
       <c r="AG197" s="4">
         <v>13</v>
       </c>
-      <c r="AH197" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH197" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36989,8 +36990,8 @@
       <c r="AG198" s="2">
         <v>13</v>
       </c>
-      <c r="AH198" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH198" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37093,8 +37094,8 @@
       <c r="AG199" s="4">
         <v>13</v>
       </c>
-      <c r="AH199" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH199" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37197,8 +37198,8 @@
       <c r="AG200" s="2">
         <v>13</v>
       </c>
-      <c r="AH200" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH200" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37301,8 +37302,8 @@
       <c r="AG201" s="4">
         <v>13</v>
       </c>
-      <c r="AH201" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH201" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37405,8 +37406,8 @@
       <c r="AG202" s="2">
         <v>5</v>
       </c>
-      <c r="AH202" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH202" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37509,8 +37510,8 @@
       <c r="AG203" s="4">
         <v>13</v>
       </c>
-      <c r="AH203" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH203" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37613,8 +37614,8 @@
       <c r="AG204" s="2">
         <v>13</v>
       </c>
-      <c r="AH204" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH204" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37717,8 +37718,8 @@
       <c r="AG205" s="4">
         <v>13</v>
       </c>
-      <c r="AH205" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH205" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37821,8 +37822,8 @@
       <c r="AG206" s="2">
         <v>13</v>
       </c>
-      <c r="AH206" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH206" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37925,8 +37926,8 @@
       <c r="AG207" s="4">
         <v>13</v>
       </c>
-      <c r="AH207" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH207" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38029,8 +38030,8 @@
       <c r="AG208" s="2">
         <v>13</v>
       </c>
-      <c r="AH208" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH208" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38133,8 +38134,8 @@
       <c r="AG209" s="4">
         <v>13</v>
       </c>
-      <c r="AH209" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH209" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38237,8 +38238,8 @@
       <c r="AG210" s="2">
         <v>10</v>
       </c>
-      <c r="AH210" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH210" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38341,8 +38342,8 @@
       <c r="AG211" s="4">
         <v>5</v>
       </c>
-      <c r="AH211" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH211" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38445,8 +38446,8 @@
       <c r="AG212" s="2">
         <v>13</v>
       </c>
-      <c r="AH212" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH212" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38549,8 +38550,8 @@
       <c r="AG213" s="4">
         <v>13</v>
       </c>
-      <c r="AH213" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH213" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38653,8 +38654,8 @@
       <c r="AG214" s="2">
         <v>13</v>
       </c>
-      <c r="AH214" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH214" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38757,8 +38758,8 @@
       <c r="AG215" s="4">
         <v>13</v>
       </c>
-      <c r="AH215" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH215" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38861,8 +38862,8 @@
       <c r="AG216" s="2">
         <v>13</v>
       </c>
-      <c r="AH216" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH216" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38965,8 +38966,8 @@
       <c r="AG217" s="4">
         <v>6</v>
       </c>
-      <c r="AH217" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH217" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39069,8 +39070,8 @@
       <c r="AG218" s="2">
         <v>13</v>
       </c>
-      <c r="AH218" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH218" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39173,8 +39174,8 @@
       <c r="AG219" s="4">
         <v>13</v>
       </c>
-      <c r="AH219" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH219" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39277,8 +39278,8 @@
       <c r="AG220" s="2">
         <v>5</v>
       </c>
-      <c r="AH220" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH220" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39381,8 +39382,8 @@
       <c r="AG221" s="4">
         <v>13</v>
       </c>
-      <c r="AH221" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH221" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39485,8 +39486,8 @@
       <c r="AG222" s="2">
         <v>13</v>
       </c>
-      <c r="AH222" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH222" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39589,8 +39590,8 @@
       <c r="AG223" s="4">
         <v>13</v>
       </c>
-      <c r="AH223" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH223" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39693,8 +39694,8 @@
       <c r="AG224" s="2">
         <v>13</v>
       </c>
-      <c r="AH224" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH224" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39797,8 +39798,8 @@
       <c r="AG225" s="4">
         <v>13</v>
       </c>
-      <c r="AH225" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH225" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39901,8 +39902,8 @@
       <c r="AG226" s="2">
         <v>13</v>
       </c>
-      <c r="AH226" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH226" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40005,8 +40006,8 @@
       <c r="AG227" s="4">
         <v>13</v>
       </c>
-      <c r="AH227" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH227" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40109,8 +40110,8 @@
       <c r="AG228" s="2">
         <v>13</v>
       </c>
-      <c r="AH228" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH228" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40213,8 +40214,8 @@
       <c r="AG229" s="4">
         <v>13</v>
       </c>
-      <c r="AH229" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH229" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40317,8 +40318,8 @@
       <c r="AG230" s="2">
         <v>13</v>
       </c>
-      <c r="AH230" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH230" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40421,8 +40422,8 @@
       <c r="AG231" s="4">
         <v>13</v>
       </c>
-      <c r="AH231" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH231" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40525,8 +40526,8 @@
       <c r="AG232" s="2">
         <v>13</v>
       </c>
-      <c r="AH232" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH232" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40629,8 +40630,8 @@
       <c r="AG233" s="4">
         <v>13</v>
       </c>
-      <c r="AH233" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH233" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40733,8 +40734,8 @@
       <c r="AG234" s="2">
         <v>13</v>
       </c>
-      <c r="AH234" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH234" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40837,8 +40838,8 @@
       <c r="AG235" s="4">
         <v>13</v>
       </c>
-      <c r="AH235" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH235" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40941,8 +40942,8 @@
       <c r="AG236" s="2">
         <v>13</v>
       </c>
-      <c r="AH236" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH236" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41045,8 +41046,8 @@
       <c r="AG237" s="4">
         <v>13</v>
       </c>
-      <c r="AH237" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH237" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41149,8 +41150,8 @@
       <c r="AG238" s="2">
         <v>13</v>
       </c>
-      <c r="AH238" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH238" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41253,8 +41254,8 @@
       <c r="AG239" s="4">
         <v>13</v>
       </c>
-      <c r="AH239" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH239" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41357,8 +41358,8 @@
       <c r="AG240" s="2">
         <v>13</v>
       </c>
-      <c r="AH240" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH240" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41461,8 +41462,8 @@
       <c r="AG241" s="4">
         <v>13</v>
       </c>
-      <c r="AH241" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH241" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41565,8 +41566,8 @@
       <c r="AG242" s="2">
         <v>5</v>
       </c>
-      <c r="AH242" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH242" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41669,8 +41670,8 @@
       <c r="AG243" s="4">
         <v>13</v>
       </c>
-      <c r="AH243" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH243" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41773,8 +41774,8 @@
       <c r="AG244" s="2">
         <v>13</v>
       </c>
-      <c r="AH244" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH244" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41877,8 +41878,8 @@
       <c r="AG245" s="4">
         <v>13</v>
       </c>
-      <c r="AH245" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH245" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41981,8 +41982,8 @@
       <c r="AG246" s="2">
         <v>13</v>
       </c>
-      <c r="AH246" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH246" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42085,8 +42086,8 @@
       <c r="AG247" s="4">
         <v>13</v>
       </c>
-      <c r="AH247" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH247" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42189,8 +42190,8 @@
       <c r="AG248" s="2">
         <v>13</v>
       </c>
-      <c r="AH248" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH248" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42293,8 +42294,8 @@
       <c r="AG249" s="4">
         <v>13</v>
       </c>
-      <c r="AH249" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH249" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42397,8 +42398,8 @@
       <c r="AG250" s="2">
         <v>13</v>
       </c>
-      <c r="AH250" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH250" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42501,8 +42502,8 @@
       <c r="AG251" s="4">
         <v>13</v>
       </c>
-      <c r="AH251" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH251" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42605,8 +42606,8 @@
       <c r="AG252" s="2">
         <v>13</v>
       </c>
-      <c r="AH252" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH252" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42709,8 +42710,8 @@
       <c r="AG253" s="4">
         <v>13</v>
       </c>
-      <c r="AH253" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH253" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42813,8 +42814,8 @@
       <c r="AG254" s="2">
         <v>13</v>
       </c>
-      <c r="AH254" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH254" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42917,8 +42918,8 @@
       <c r="AG255" s="4">
         <v>13</v>
       </c>
-      <c r="AH255" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH255" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43021,8 +43022,8 @@
       <c r="AG256" s="2">
         <v>13</v>
       </c>
-      <c r="AH256" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH256" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43125,8 +43126,8 @@
       <c r="AG257" s="4">
         <v>13</v>
       </c>
-      <c r="AH257" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH257" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43229,8 +43230,8 @@
       <c r="AG258" s="2">
         <v>13</v>
       </c>
-      <c r="AH258" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH258" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43333,8 +43334,8 @@
       <c r="AG259" s="4">
         <v>13</v>
       </c>
-      <c r="AH259" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH259" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43437,8 +43438,8 @@
       <c r="AG260" s="2">
         <v>13</v>
       </c>
-      <c r="AH260" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH260" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43541,8 +43542,8 @@
       <c r="AG261" s="4">
         <v>13</v>
       </c>
-      <c r="AH261" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH261" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43645,8 +43646,8 @@
       <c r="AG262" s="2">
         <v>13</v>
       </c>
-      <c r="AH262" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH262" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43749,8 +43750,8 @@
       <c r="AG263" s="4">
         <v>13</v>
       </c>
-      <c r="AH263" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH263" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43853,8 +43854,8 @@
       <c r="AG264" s="2">
         <v>13</v>
       </c>
-      <c r="AH264" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH264" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43957,8 +43958,8 @@
       <c r="AG265" s="4">
         <v>13</v>
       </c>
-      <c r="AH265" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH265" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44061,8 +44062,8 @@
       <c r="AG266" s="2">
         <v>13</v>
       </c>
-      <c r="AH266" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH266" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44165,8 +44166,8 @@
       <c r="AG267" s="4">
         <v>13</v>
       </c>
-      <c r="AH267" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH267" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44269,8 +44270,8 @@
       <c r="AG268" s="2">
         <v>13</v>
       </c>
-      <c r="AH268" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH268" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44373,8 +44374,8 @@
       <c r="AG269" s="4">
         <v>13</v>
       </c>
-      <c r="AH269" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH269" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44477,8 +44478,8 @@
       <c r="AG270" s="2">
         <v>13</v>
       </c>
-      <c r="AH270" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH270" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44581,8 +44582,8 @@
       <c r="AG271" s="4">
         <v>13</v>
       </c>
-      <c r="AH271" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH271" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44685,8 +44686,8 @@
       <c r="AG272" s="2">
         <v>13</v>
       </c>
-      <c r="AH272" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH272" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44789,8 +44790,8 @@
       <c r="AG273" s="4">
         <v>13</v>
       </c>
-      <c r="AH273" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH273" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44893,8 +44894,8 @@
       <c r="AG274" s="2">
         <v>13</v>
       </c>
-      <c r="AH274" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH274" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -44997,8 +44998,8 @@
       <c r="AG275" s="4">
         <v>13</v>
       </c>
-      <c r="AH275" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH275" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45101,8 +45102,8 @@
       <c r="AG276" s="2">
         <v>13</v>
       </c>
-      <c r="AH276" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH276" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45205,8 +45206,8 @@
       <c r="AG277" s="4">
         <v>13</v>
       </c>
-      <c r="AH277" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH277" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45309,8 +45310,8 @@
       <c r="AG278" s="2">
         <v>13</v>
       </c>
-      <c r="AH278" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH278" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45413,8 +45414,8 @@
       <c r="AG279" s="4">
         <v>13</v>
       </c>
-      <c r="AH279" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH279" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45517,8 +45518,8 @@
       <c r="AG280" s="2">
         <v>13</v>
       </c>
-      <c r="AH280" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH280" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45621,8 +45622,8 @@
       <c r="AG281" s="4">
         <v>13</v>
       </c>
-      <c r="AH281" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH281" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45725,8 +45726,8 @@
       <c r="AG282" s="2">
         <v>13</v>
       </c>
-      <c r="AH282" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH282" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45829,8 +45830,8 @@
       <c r="AG283" s="4">
         <v>5</v>
       </c>
-      <c r="AH283" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH283" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45933,8 +45934,8 @@
       <c r="AG284" s="2">
         <v>13</v>
       </c>
-      <c r="AH284" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH284" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46037,8 +46038,8 @@
       <c r="AG285" s="4">
         <v>13</v>
       </c>
-      <c r="AH285" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH285" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46141,8 +46142,8 @@
       <c r="AG286" s="2">
         <v>13</v>
       </c>
-      <c r="AH286" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH286" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46245,8 +46246,8 @@
       <c r="AG287" s="4">
         <v>13</v>
       </c>
-      <c r="AH287" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH287" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46349,8 +46350,8 @@
       <c r="AG288" s="2">
         <v>13</v>
       </c>
-      <c r="AH288" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH288" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46453,8 +46454,8 @@
       <c r="AG289" s="4">
         <v>13</v>
       </c>
-      <c r="AH289" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH289" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46557,8 +46558,8 @@
       <c r="AG290" s="2">
         <v>13</v>
       </c>
-      <c r="AH290" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH290" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46661,8 +46662,8 @@
       <c r="AG291" s="4">
         <v>13</v>
       </c>
-      <c r="AH291" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH291" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46765,8 +46766,8 @@
       <c r="AG292" s="2">
         <v>13</v>
       </c>
-      <c r="AH292" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH292" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46869,8 +46870,8 @@
       <c r="AG293" s="4">
         <v>13</v>
       </c>
-      <c r="AH293" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH293" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46973,8 +46974,8 @@
       <c r="AG294" s="2">
         <v>13</v>
       </c>
-      <c r="AH294" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH294" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47077,8 +47078,8 @@
       <c r="AG295" s="4">
         <v>13</v>
       </c>
-      <c r="AH295" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH295" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47181,8 +47182,8 @@
       <c r="AG296" s="2">
         <v>13</v>
       </c>
-      <c r="AH296" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH296" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47285,8 +47286,8 @@
       <c r="AG297" s="4">
         <v>13</v>
       </c>
-      <c r="AH297" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH297" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47389,8 +47390,8 @@
       <c r="AG298" s="2">
         <v>13</v>
       </c>
-      <c r="AH298" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH298" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47493,8 +47494,8 @@
       <c r="AG299" s="4">
         <v>13</v>
       </c>
-      <c r="AH299" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH299" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47597,8 +47598,8 @@
       <c r="AG300" s="2">
         <v>13</v>
       </c>
-      <c r="AH300" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH300" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47701,8 +47702,8 @@
       <c r="AG301" s="4">
         <v>13</v>
       </c>
-      <c r="AH301" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH301" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47805,8 +47806,8 @@
       <c r="AG302" s="2">
         <v>13</v>
       </c>
-      <c r="AH302" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH302" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47909,8 +47910,8 @@
       <c r="AG303" s="4">
         <v>13</v>
       </c>
-      <c r="AH303" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH303" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48013,8 +48014,8 @@
       <c r="AG304" s="2">
         <v>13</v>
       </c>
-      <c r="AH304" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH304" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48117,8 +48118,8 @@
       <c r="AG305" s="4">
         <v>13</v>
       </c>
-      <c r="AH305" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH305" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48221,8 +48222,8 @@
       <c r="AG306" s="2">
         <v>13</v>
       </c>
-      <c r="AH306" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH306" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48325,8 +48326,8 @@
       <c r="AG307" s="4">
         <v>13</v>
       </c>
-      <c r="AH307" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH307" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48429,8 +48430,8 @@
       <c r="AG308" s="2">
         <v>13</v>
       </c>
-      <c r="AH308" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH308" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48533,8 +48534,8 @@
       <c r="AG309" s="4">
         <v>13</v>
       </c>
-      <c r="AH309" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH309" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48637,8 +48638,8 @@
       <c r="AG310" s="2">
         <v>13</v>
       </c>
-      <c r="AH310" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH310" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48741,8 +48742,8 @@
       <c r="AG311" s="4">
         <v>13</v>
       </c>
-      <c r="AH311" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH311" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48845,8 +48846,8 @@
       <c r="AG312" s="2">
         <v>13</v>
       </c>
-      <c r="AH312" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH312" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48949,8 +48950,8 @@
       <c r="AG313" s="4">
         <v>13</v>
       </c>
-      <c r="AH313" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH313" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49053,8 +49054,8 @@
       <c r="AG314" s="2">
         <v>13</v>
       </c>
-      <c r="AH314" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH314" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49157,8 +49158,8 @@
       <c r="AG315" s="4">
         <v>13</v>
       </c>
-      <c r="AH315" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH315" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49261,8 +49262,8 @@
       <c r="AG316" s="2">
         <v>13</v>
       </c>
-      <c r="AH316" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH316" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49365,8 +49366,8 @@
       <c r="AG317" s="4">
         <v>8</v>
       </c>
-      <c r="AH317" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH317" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49469,8 +49470,8 @@
       <c r="AG318" s="2">
         <v>13</v>
       </c>
-      <c r="AH318" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH318" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49573,8 +49574,8 @@
       <c r="AG319" s="4">
         <v>13</v>
       </c>
-      <c r="AH319" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH319" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49677,8 +49678,8 @@
       <c r="AG320" s="2">
         <v>13</v>
       </c>
-      <c r="AH320" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH320" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49781,8 +49782,8 @@
       <c r="AG321" s="4">
         <v>13</v>
       </c>
-      <c r="AH321" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH321" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49885,8 +49886,8 @@
       <c r="AG322" s="2">
         <v>8</v>
       </c>
-      <c r="AH322" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH322" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49989,8 +49990,8 @@
       <c r="AG323" s="4">
         <v>13</v>
       </c>
-      <c r="AH323" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH323" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50093,8 +50094,8 @@
       <c r="AG324" s="2">
         <v>5</v>
       </c>
-      <c r="AH324" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH324" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50197,8 +50198,8 @@
       <c r="AG325" s="4">
         <v>13</v>
       </c>
-      <c r="AH325" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH325" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50301,8 +50302,8 @@
       <c r="AG326" s="2">
         <v>13</v>
       </c>
-      <c r="AH326" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH326" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50405,8 +50406,8 @@
       <c r="AG327" s="4">
         <v>13</v>
       </c>
-      <c r="AH327" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH327" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50509,8 +50510,8 @@
       <c r="AG328" s="2">
         <v>13</v>
       </c>
-      <c r="AH328" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH328" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50613,8 +50614,8 @@
       <c r="AG329" s="4">
         <v>13</v>
       </c>
-      <c r="AH329" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH329" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50717,8 +50718,8 @@
       <c r="AG330" s="2">
         <v>13</v>
       </c>
-      <c r="AH330" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH330" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50821,8 +50822,8 @@
       <c r="AG331" s="4">
         <v>13</v>
       </c>
-      <c r="AH331" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH331" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50925,8 +50926,8 @@
       <c r="AG332" s="2">
         <v>13</v>
       </c>
-      <c r="AH332" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH332" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51029,8 +51030,8 @@
       <c r="AG333" s="4">
         <v>13</v>
       </c>
-      <c r="AH333" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH333" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51133,8 +51134,8 @@
       <c r="AG334" s="2">
         <v>13</v>
       </c>
-      <c r="AH334" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH334" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51237,8 +51238,8 @@
       <c r="AG335" s="4">
         <v>13</v>
       </c>
-      <c r="AH335" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH335" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51341,8 +51342,8 @@
       <c r="AG336" s="2">
         <v>10</v>
       </c>
-      <c r="AH336" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH336" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51445,8 +51446,8 @@
       <c r="AG337" s="4">
         <v>13</v>
       </c>
-      <c r="AH337" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH337" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51549,8 +51550,8 @@
       <c r="AG338" s="2">
         <v>13</v>
       </c>
-      <c r="AH338" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH338" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51653,8 +51654,8 @@
       <c r="AG339" s="4">
         <v>13</v>
       </c>
-      <c r="AH339" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH339" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51757,8 +51758,8 @@
       <c r="AG340" s="2">
         <v>5</v>
       </c>
-      <c r="AH340" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH340" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51861,8 +51862,8 @@
       <c r="AG341" s="4">
         <v>13</v>
       </c>
-      <c r="AH341" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH341" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51965,8 +51966,8 @@
       <c r="AG342" s="2">
         <v>13</v>
       </c>
-      <c r="AH342" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH342" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52069,8 +52070,8 @@
       <c r="AG343" s="4">
         <v>13</v>
       </c>
-      <c r="AH343" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH343" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52173,8 +52174,8 @@
       <c r="AG344" s="2">
         <v>13</v>
       </c>
-      <c r="AH344" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH344" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52277,8 +52278,8 @@
       <c r="AG345" s="4">
         <v>13</v>
       </c>
-      <c r="AH345" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH345" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52381,8 +52382,8 @@
       <c r="AG346" s="2">
         <v>13</v>
       </c>
-      <c r="AH346" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH346" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52485,8 +52486,8 @@
       <c r="AG347" s="4">
         <v>13</v>
       </c>
-      <c r="AH347" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH347" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52589,8 +52590,8 @@
       <c r="AG348" s="2">
         <v>13</v>
       </c>
-      <c r="AH348" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH348" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52693,8 +52694,8 @@
       <c r="AG349" s="4">
         <v>13</v>
       </c>
-      <c r="AH349" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH349" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52797,8 +52798,8 @@
       <c r="AG350" s="2">
         <v>13</v>
       </c>
-      <c r="AH350" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH350" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52901,8 +52902,8 @@
       <c r="AG351" s="4">
         <v>13</v>
       </c>
-      <c r="AH351" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH351" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53005,8 +53006,8 @@
       <c r="AG352" s="2">
         <v>13</v>
       </c>
-      <c r="AH352" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH352" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53109,8 +53110,8 @@
       <c r="AG353" s="4">
         <v>13</v>
       </c>
-      <c r="AH353" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH353" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53213,8 +53214,8 @@
       <c r="AG354" s="2">
         <v>13</v>
       </c>
-      <c r="AH354" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH354" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53317,8 +53318,8 @@
       <c r="AG355" s="4">
         <v>13</v>
       </c>
-      <c r="AH355" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH355" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53421,8 +53422,8 @@
       <c r="AG356" s="2">
         <v>13</v>
       </c>
-      <c r="AH356" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH356" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53525,8 +53526,8 @@
       <c r="AG357" s="4">
         <v>13</v>
       </c>
-      <c r="AH357" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH357" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53579,8 +53580,8 @@
       <c r="AG358" s="2">
         <v>13</v>
       </c>
-      <c r="AH358" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH358" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53683,8 +53684,8 @@
       <c r="AG359" s="4">
         <v>13</v>
       </c>
-      <c r="AH359" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH359" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53787,8 +53788,8 @@
       <c r="AG360" s="2">
         <v>13</v>
       </c>
-      <c r="AH360" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH360" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53891,8 +53892,8 @@
       <c r="AG361" s="4">
         <v>13</v>
       </c>
-      <c r="AH361" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH361" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -53995,8 +53996,8 @@
       <c r="AG362" s="2">
         <v>13</v>
       </c>
-      <c r="AH362" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH362" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54099,8 +54100,8 @@
       <c r="AG363" s="4">
         <v>13</v>
       </c>
-      <c r="AH363" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH363" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54203,8 +54204,8 @@
       <c r="AG364" s="2">
         <v>13</v>
       </c>
-      <c r="AH364" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH364" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54307,8 +54308,8 @@
       <c r="AG365" s="4">
         <v>13</v>
       </c>
-      <c r="AH365" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH365" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54411,8 +54412,8 @@
       <c r="AG366" s="2">
         <v>13</v>
       </c>
-      <c r="AH366" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH366" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54515,8 +54516,8 @@
       <c r="AG367" s="4">
         <v>13</v>
       </c>
-      <c r="AH367" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH367" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54619,8 +54620,8 @@
       <c r="AG368" s="2">
         <v>13</v>
       </c>
-      <c r="AH368" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH368" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54723,8 +54724,8 @@
       <c r="AG369" s="4">
         <v>13</v>
       </c>
-      <c r="AH369" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH369" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54827,8 +54828,8 @@
       <c r="AG370" s="2">
         <v>13</v>
       </c>
-      <c r="AH370" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH370" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54931,8 +54932,8 @@
       <c r="AG371" s="4">
         <v>5</v>
       </c>
-      <c r="AH371" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH371" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55035,8 +55036,8 @@
       <c r="AG372" s="2">
         <v>13</v>
       </c>
-      <c r="AH372" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH372" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55139,8 +55140,8 @@
       <c r="AG373" s="4">
         <v>13</v>
       </c>
-      <c r="AH373" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH373" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55243,8 +55244,8 @@
       <c r="AG374" s="2">
         <v>13</v>
       </c>
-      <c r="AH374" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH374" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55347,8 +55348,8 @@
       <c r="AG375" s="4">
         <v>13</v>
       </c>
-      <c r="AH375" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH375" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55451,8 +55452,8 @@
       <c r="AG376" s="2">
         <v>13</v>
       </c>
-      <c r="AH376" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH376" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55555,8 +55556,8 @@
       <c r="AG377" s="4">
         <v>13</v>
       </c>
-      <c r="AH377" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH377" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55659,8 +55660,8 @@
       <c r="AG378" s="2">
         <v>13</v>
       </c>
-      <c r="AH378" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH378" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55763,8 +55764,8 @@
       <c r="AG379" s="4">
         <v>5</v>
       </c>
-      <c r="AH379" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH379" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55867,8 +55868,8 @@
       <c r="AG380" s="2">
         <v>13</v>
       </c>
-      <c r="AH380" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH380" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55971,8 +55972,8 @@
       <c r="AG381" s="4">
         <v>13</v>
       </c>
-      <c r="AH381" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH381" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56075,8 +56076,8 @@
       <c r="AG382" s="2">
         <v>13</v>
       </c>
-      <c r="AH382" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH382" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56179,8 +56180,8 @@
       <c r="AG383" s="4">
         <v>13</v>
       </c>
-      <c r="AH383" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH383" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56283,8 +56284,8 @@
       <c r="AG384" s="2">
         <v>13</v>
       </c>
-      <c r="AH384" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH384" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56337,8 +56338,8 @@
       <c r="AG385" s="4">
         <v>13</v>
       </c>
-      <c r="AH385" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH385" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56441,8 +56442,8 @@
       <c r="AG386" s="2">
         <v>13</v>
       </c>
-      <c r="AH386" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH386" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56545,8 +56546,8 @@
       <c r="AG387" s="4">
         <v>13</v>
       </c>
-      <c r="AH387" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH387" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56649,8 +56650,8 @@
       <c r="AG388" s="2">
         <v>13</v>
       </c>
-      <c r="AH388" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH388" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56753,8 +56754,8 @@
       <c r="AG389" s="4">
         <v>13</v>
       </c>
-      <c r="AH389" s="6">
-        <v>46181.350868055553</v>
+      <c r="AH389" s="3" t="s">
+        <v>4911</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56857,8 +56858,8 @@
       <c r="AG390" s="2">
         <v>13</v>
       </c>
-      <c r="AH390" s="5">
-        <v>46181.350868055553</v>
+      <c r="AH390" s="1" t="s">
+        <v>4911</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-06 09:09:23
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12043" uniqueCount="4912">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11654" uniqueCount="4911">
   <si>
     <t>Rut Proveedor</t>
   </si>
@@ -14752,9 +14752,6 @@
   </si>
   <si>
     <t>Fecha y Hora Actualización</t>
-  </si>
-  <si>
-    <t>26/08/06 09:04:30</t>
   </si>
 </sst>
 </file>
@@ -14819,12 +14816,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -14893,7 +14892,7 @@
         <name val="Calibri"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ h:mm"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="9" tint="0.79998168889431442"/>
@@ -16403,106 +16402,106 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="O1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="Q1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="R1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="S1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="T1" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="U1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="V1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="5" t="s">
+      <c r="W1" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="X1" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="5" t="s">
+      <c r="Y1" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="5" t="s">
+      <c r="Z1" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="5" t="s">
+      <c r="AA1" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="5" t="s">
+      <c r="AB1" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="AC1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="5" t="s">
+      <c r="AD1" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="5" t="s">
+      <c r="AE1" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="5" t="s">
+      <c r="AF1" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="5" t="s">
+      <c r="AG1" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="5" t="s">
+      <c r="AH1" s="7" t="s">
         <v>4910</v>
       </c>
     </row>
@@ -16606,8 +16605,8 @@
       <c r="AG2" s="2">
         <v>13</v>
       </c>
-      <c r="AH2" s="1" t="s">
-        <v>4911</v>
+      <c r="AH2" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16710,8 +16709,8 @@
       <c r="AG3" s="4">
         <v>13</v>
       </c>
-      <c r="AH3" s="3" t="s">
-        <v>4911</v>
+      <c r="AH3" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16814,8 +16813,8 @@
       <c r="AG4" s="2">
         <v>13</v>
       </c>
-      <c r="AH4" s="1" t="s">
-        <v>4911</v>
+      <c r="AH4" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16918,8 +16917,8 @@
       <c r="AG5" s="4">
         <v>13</v>
       </c>
-      <c r="AH5" s="3" t="s">
-        <v>4911</v>
+      <c r="AH5" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17022,8 +17021,8 @@
       <c r="AG6" s="2">
         <v>13</v>
       </c>
-      <c r="AH6" s="1" t="s">
-        <v>4911</v>
+      <c r="AH6" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17126,8 +17125,8 @@
       <c r="AG7" s="4">
         <v>13</v>
       </c>
-      <c r="AH7" s="3" t="s">
-        <v>4911</v>
+      <c r="AH7" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17230,8 +17229,8 @@
       <c r="AG8" s="2">
         <v>13</v>
       </c>
-      <c r="AH8" s="1" t="s">
-        <v>4911</v>
+      <c r="AH8" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17334,8 +17333,8 @@
       <c r="AG9" s="4">
         <v>13</v>
       </c>
-      <c r="AH9" s="3" t="s">
-        <v>4911</v>
+      <c r="AH9" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17438,8 +17437,8 @@
       <c r="AG10" s="2">
         <v>13</v>
       </c>
-      <c r="AH10" s="1" t="s">
-        <v>4911</v>
+      <c r="AH10" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17542,8 +17541,8 @@
       <c r="AG11" s="4">
         <v>13</v>
       </c>
-      <c r="AH11" s="3" t="s">
-        <v>4911</v>
+      <c r="AH11" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17646,8 +17645,8 @@
       <c r="AG12" s="2">
         <v>13</v>
       </c>
-      <c r="AH12" s="1" t="s">
-        <v>4911</v>
+      <c r="AH12" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17750,8 +17749,8 @@
       <c r="AG13" s="4">
         <v>13</v>
       </c>
-      <c r="AH13" s="3" t="s">
-        <v>4911</v>
+      <c r="AH13" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17854,8 +17853,8 @@
       <c r="AG14" s="2">
         <v>13</v>
       </c>
-      <c r="AH14" s="1" t="s">
-        <v>4911</v>
+      <c r="AH14" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17958,8 +17957,8 @@
       <c r="AG15" s="4">
         <v>13</v>
       </c>
-      <c r="AH15" s="3" t="s">
-        <v>4911</v>
+      <c r="AH15" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18062,8 +18061,8 @@
       <c r="AG16" s="2">
         <v>13</v>
       </c>
-      <c r="AH16" s="1" t="s">
-        <v>4911</v>
+      <c r="AH16" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18166,8 +18165,8 @@
       <c r="AG17" s="4">
         <v>13</v>
       </c>
-      <c r="AH17" s="3" t="s">
-        <v>4911</v>
+      <c r="AH17" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18270,8 +18269,8 @@
       <c r="AG18" s="2">
         <v>13</v>
       </c>
-      <c r="AH18" s="1" t="s">
-        <v>4911</v>
+      <c r="AH18" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18374,8 +18373,8 @@
       <c r="AG19" s="4">
         <v>13</v>
       </c>
-      <c r="AH19" s="3" t="s">
-        <v>4911</v>
+      <c r="AH19" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18478,8 +18477,8 @@
       <c r="AG20" s="2">
         <v>13</v>
       </c>
-      <c r="AH20" s="1" t="s">
-        <v>4911</v>
+      <c r="AH20" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18582,8 +18581,8 @@
       <c r="AG21" s="4">
         <v>13</v>
       </c>
-      <c r="AH21" s="3" t="s">
-        <v>4911</v>
+      <c r="AH21" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18686,8 +18685,8 @@
       <c r="AG22" s="2">
         <v>13</v>
       </c>
-      <c r="AH22" s="1" t="s">
-        <v>4911</v>
+      <c r="AH22" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18790,8 +18789,8 @@
       <c r="AG23" s="4">
         <v>13</v>
       </c>
-      <c r="AH23" s="3" t="s">
-        <v>4911</v>
+      <c r="AH23" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18894,8 +18893,8 @@
       <c r="AG24" s="2">
         <v>13</v>
       </c>
-      <c r="AH24" s="1" t="s">
-        <v>4911</v>
+      <c r="AH24" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -18998,8 +18997,8 @@
       <c r="AG25" s="4">
         <v>13</v>
       </c>
-      <c r="AH25" s="3" t="s">
-        <v>4911</v>
+      <c r="AH25" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19102,8 +19101,8 @@
       <c r="AG26" s="2">
         <v>13</v>
       </c>
-      <c r="AH26" s="1" t="s">
-        <v>4911</v>
+      <c r="AH26" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19206,8 +19205,8 @@
       <c r="AG27" s="4">
         <v>13</v>
       </c>
-      <c r="AH27" s="3" t="s">
-        <v>4911</v>
+      <c r="AH27" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19310,8 +19309,8 @@
       <c r="AG28" s="2">
         <v>13</v>
       </c>
-      <c r="AH28" s="1" t="s">
-        <v>4911</v>
+      <c r="AH28" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19414,8 +19413,8 @@
       <c r="AG29" s="4">
         <v>5</v>
       </c>
-      <c r="AH29" s="3" t="s">
-        <v>4911</v>
+      <c r="AH29" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19518,8 +19517,8 @@
       <c r="AG30" s="2">
         <v>13</v>
       </c>
-      <c r="AH30" s="1" t="s">
-        <v>4911</v>
+      <c r="AH30" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19622,8 +19621,8 @@
       <c r="AG31" s="4">
         <v>13</v>
       </c>
-      <c r="AH31" s="3" t="s">
-        <v>4911</v>
+      <c r="AH31" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19726,8 +19725,8 @@
       <c r="AG32" s="2">
         <v>13</v>
       </c>
-      <c r="AH32" s="1" t="s">
-        <v>4911</v>
+      <c r="AH32" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19830,8 +19829,8 @@
       <c r="AG33" s="4">
         <v>13</v>
       </c>
-      <c r="AH33" s="3" t="s">
-        <v>4911</v>
+      <c r="AH33" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19934,8 +19933,8 @@
       <c r="AG34" s="2">
         <v>13</v>
       </c>
-      <c r="AH34" s="1" t="s">
-        <v>4911</v>
+      <c r="AH34" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20038,8 +20037,8 @@
       <c r="AG35" s="4">
         <v>13</v>
       </c>
-      <c r="AH35" s="3" t="s">
-        <v>4911</v>
+      <c r="AH35" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20142,8 +20141,8 @@
       <c r="AG36" s="2">
         <v>13</v>
       </c>
-      <c r="AH36" s="1" t="s">
-        <v>4911</v>
+      <c r="AH36" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20246,8 +20245,8 @@
       <c r="AG37" s="4">
         <v>13</v>
       </c>
-      <c r="AH37" s="3" t="s">
-        <v>4911</v>
+      <c r="AH37" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20350,8 +20349,8 @@
       <c r="AG38" s="2">
         <v>13</v>
       </c>
-      <c r="AH38" s="1" t="s">
-        <v>4911</v>
+      <c r="AH38" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20454,8 +20453,8 @@
       <c r="AG39" s="4">
         <v>13</v>
       </c>
-      <c r="AH39" s="3" t="s">
-        <v>4911</v>
+      <c r="AH39" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20558,8 +20557,8 @@
       <c r="AG40" s="2">
         <v>13</v>
       </c>
-      <c r="AH40" s="1" t="s">
-        <v>4911</v>
+      <c r="AH40" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20662,8 +20661,8 @@
       <c r="AG41" s="4">
         <v>13</v>
       </c>
-      <c r="AH41" s="3" t="s">
-        <v>4911</v>
+      <c r="AH41" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20766,8 +20765,8 @@
       <c r="AG42" s="2">
         <v>13</v>
       </c>
-      <c r="AH42" s="1" t="s">
-        <v>4911</v>
+      <c r="AH42" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20870,8 +20869,8 @@
       <c r="AG43" s="4">
         <v>13</v>
       </c>
-      <c r="AH43" s="3" t="s">
-        <v>4911</v>
+      <c r="AH43" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20974,8 +20973,8 @@
       <c r="AG44" s="2">
         <v>13</v>
       </c>
-      <c r="AH44" s="1" t="s">
-        <v>4911</v>
+      <c r="AH44" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21078,8 +21077,8 @@
       <c r="AG45" s="4">
         <v>13</v>
       </c>
-      <c r="AH45" s="3" t="s">
-        <v>4911</v>
+      <c r="AH45" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21182,8 +21181,8 @@
       <c r="AG46" s="2">
         <v>13</v>
       </c>
-      <c r="AH46" s="1" t="s">
-        <v>4911</v>
+      <c r="AH46" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21286,8 +21285,8 @@
       <c r="AG47" s="4">
         <v>13</v>
       </c>
-      <c r="AH47" s="3" t="s">
-        <v>4911</v>
+      <c r="AH47" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21390,8 +21389,8 @@
       <c r="AG48" s="2">
         <v>13</v>
       </c>
-      <c r="AH48" s="1" t="s">
-        <v>4911</v>
+      <c r="AH48" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21494,8 +21493,8 @@
       <c r="AG49" s="4">
         <v>13</v>
       </c>
-      <c r="AH49" s="3" t="s">
-        <v>4911</v>
+      <c r="AH49" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21598,8 +21597,8 @@
       <c r="AG50" s="2">
         <v>13</v>
       </c>
-      <c r="AH50" s="1" t="s">
-        <v>4911</v>
+      <c r="AH50" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21702,8 +21701,8 @@
       <c r="AG51" s="4">
         <v>6</v>
       </c>
-      <c r="AH51" s="3" t="s">
-        <v>4911</v>
+      <c r="AH51" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21806,8 +21805,8 @@
       <c r="AG52" s="2">
         <v>13</v>
       </c>
-      <c r="AH52" s="1" t="s">
-        <v>4911</v>
+      <c r="AH52" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21910,8 +21909,8 @@
       <c r="AG53" s="4">
         <v>13</v>
       </c>
-      <c r="AH53" s="3" t="s">
-        <v>4911</v>
+      <c r="AH53" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22014,8 +22013,8 @@
       <c r="AG54" s="2">
         <v>13</v>
       </c>
-      <c r="AH54" s="1" t="s">
-        <v>4911</v>
+      <c r="AH54" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22118,8 +22117,8 @@
       <c r="AG55" s="4">
         <v>13</v>
       </c>
-      <c r="AH55" s="3" t="s">
-        <v>4911</v>
+      <c r="AH55" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22222,8 +22221,8 @@
       <c r="AG56" s="2">
         <v>5</v>
       </c>
-      <c r="AH56" s="1" t="s">
-        <v>4911</v>
+      <c r="AH56" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22326,8 +22325,8 @@
       <c r="AG57" s="4">
         <v>13</v>
       </c>
-      <c r="AH57" s="3" t="s">
-        <v>4911</v>
+      <c r="AH57" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22430,8 +22429,8 @@
       <c r="AG58" s="2">
         <v>13</v>
       </c>
-      <c r="AH58" s="1" t="s">
-        <v>4911</v>
+      <c r="AH58" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22534,8 +22533,8 @@
       <c r="AG59" s="4">
         <v>13</v>
       </c>
-      <c r="AH59" s="3" t="s">
-        <v>4911</v>
+      <c r="AH59" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22638,8 +22637,8 @@
       <c r="AG60" s="2">
         <v>13</v>
       </c>
-      <c r="AH60" s="1" t="s">
-        <v>4911</v>
+      <c r="AH60" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22742,8 +22741,8 @@
       <c r="AG61" s="4">
         <v>13</v>
       </c>
-      <c r="AH61" s="3" t="s">
-        <v>4911</v>
+      <c r="AH61" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22846,8 +22845,8 @@
       <c r="AG62" s="2">
         <v>13</v>
       </c>
-      <c r="AH62" s="1" t="s">
-        <v>4911</v>
+      <c r="AH62" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22950,8 +22949,8 @@
       <c r="AG63" s="4">
         <v>13</v>
       </c>
-      <c r="AH63" s="3" t="s">
-        <v>4911</v>
+      <c r="AH63" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23054,8 +23053,8 @@
       <c r="AG64" s="2">
         <v>13</v>
       </c>
-      <c r="AH64" s="1" t="s">
-        <v>4911</v>
+      <c r="AH64" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23158,8 +23157,8 @@
       <c r="AG65" s="4">
         <v>13</v>
       </c>
-      <c r="AH65" s="3" t="s">
-        <v>4911</v>
+      <c r="AH65" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23262,8 +23261,8 @@
       <c r="AG66" s="2">
         <v>13</v>
       </c>
-      <c r="AH66" s="1" t="s">
-        <v>4911</v>
+      <c r="AH66" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23366,8 +23365,8 @@
       <c r="AG67" s="4">
         <v>13</v>
       </c>
-      <c r="AH67" s="3" t="s">
-        <v>4911</v>
+      <c r="AH67" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23470,8 +23469,8 @@
       <c r="AG68" s="2">
         <v>13</v>
       </c>
-      <c r="AH68" s="1" t="s">
-        <v>4911</v>
+      <c r="AH68" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23574,8 +23573,8 @@
       <c r="AG69" s="4">
         <v>13</v>
       </c>
-      <c r="AH69" s="3" t="s">
-        <v>4911</v>
+      <c r="AH69" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23678,8 +23677,8 @@
       <c r="AG70" s="2">
         <v>13</v>
       </c>
-      <c r="AH70" s="1" t="s">
-        <v>4911</v>
+      <c r="AH70" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23782,8 +23781,8 @@
       <c r="AG71" s="4">
         <v>13</v>
       </c>
-      <c r="AH71" s="3" t="s">
-        <v>4911</v>
+      <c r="AH71" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23886,8 +23885,8 @@
       <c r="AG72" s="2">
         <v>8</v>
       </c>
-      <c r="AH72" s="1" t="s">
-        <v>4911</v>
+      <c r="AH72" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23990,8 +23989,8 @@
       <c r="AG73" s="4">
         <v>5</v>
       </c>
-      <c r="AH73" s="3" t="s">
-        <v>4911</v>
+      <c r="AH73" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24094,8 +24093,8 @@
       <c r="AG74" s="2">
         <v>13</v>
       </c>
-      <c r="AH74" s="1" t="s">
-        <v>4911</v>
+      <c r="AH74" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24198,8 +24197,8 @@
       <c r="AG75" s="4">
         <v>5</v>
       </c>
-      <c r="AH75" s="3" t="s">
-        <v>4911</v>
+      <c r="AH75" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24302,8 +24301,8 @@
       <c r="AG76" s="2">
         <v>13</v>
       </c>
-      <c r="AH76" s="1" t="s">
-        <v>4911</v>
+      <c r="AH76" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24406,8 +24405,8 @@
       <c r="AG77" s="4">
         <v>13</v>
       </c>
-      <c r="AH77" s="3" t="s">
-        <v>4911</v>
+      <c r="AH77" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24510,8 +24509,8 @@
       <c r="AG78" s="2">
         <v>9</v>
       </c>
-      <c r="AH78" s="1" t="s">
-        <v>4911</v>
+      <c r="AH78" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24614,8 +24613,8 @@
       <c r="AG79" s="4">
         <v>13</v>
       </c>
-      <c r="AH79" s="3" t="s">
-        <v>4911</v>
+      <c r="AH79" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24718,8 +24717,8 @@
       <c r="AG80" s="2">
         <v>13</v>
       </c>
-      <c r="AH80" s="1" t="s">
-        <v>4911</v>
+      <c r="AH80" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24822,8 +24821,8 @@
       <c r="AG81" s="4">
         <v>13</v>
       </c>
-      <c r="AH81" s="3" t="s">
-        <v>4911</v>
+      <c r="AH81" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24926,8 +24925,8 @@
       <c r="AG82" s="2">
         <v>13</v>
       </c>
-      <c r="AH82" s="1" t="s">
-        <v>4911</v>
+      <c r="AH82" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25030,8 +25029,8 @@
       <c r="AG83" s="4">
         <v>13</v>
       </c>
-      <c r="AH83" s="3" t="s">
-        <v>4911</v>
+      <c r="AH83" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25134,8 +25133,8 @@
       <c r="AG84" s="2">
         <v>13</v>
       </c>
-      <c r="AH84" s="1" t="s">
-        <v>4911</v>
+      <c r="AH84" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25238,8 +25237,8 @@
       <c r="AG85" s="4">
         <v>13</v>
       </c>
-      <c r="AH85" s="3" t="s">
-        <v>4911</v>
+      <c r="AH85" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25342,8 +25341,8 @@
       <c r="AG86" s="2">
         <v>13</v>
       </c>
-      <c r="AH86" s="1" t="s">
-        <v>4911</v>
+      <c r="AH86" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25446,8 +25445,8 @@
       <c r="AG87" s="4">
         <v>13</v>
       </c>
-      <c r="AH87" s="3" t="s">
-        <v>4911</v>
+      <c r="AH87" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25550,8 +25549,8 @@
       <c r="AG88" s="2">
         <v>13</v>
       </c>
-      <c r="AH88" s="1" t="s">
-        <v>4911</v>
+      <c r="AH88" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25654,8 +25653,8 @@
       <c r="AG89" s="4">
         <v>13</v>
       </c>
-      <c r="AH89" s="3" t="s">
-        <v>4911</v>
+      <c r="AH89" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25758,8 +25757,8 @@
       <c r="AG90" s="2">
         <v>13</v>
       </c>
-      <c r="AH90" s="1" t="s">
-        <v>4911</v>
+      <c r="AH90" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25862,8 +25861,8 @@
       <c r="AG91" s="4">
         <v>13</v>
       </c>
-      <c r="AH91" s="3" t="s">
-        <v>4911</v>
+      <c r="AH91" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25966,8 +25965,8 @@
       <c r="AG92" s="2">
         <v>13</v>
       </c>
-      <c r="AH92" s="1" t="s">
-        <v>4911</v>
+      <c r="AH92" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26070,8 +26069,8 @@
       <c r="AG93" s="4">
         <v>13</v>
       </c>
-      <c r="AH93" s="3" t="s">
-        <v>4911</v>
+      <c r="AH93" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26174,8 +26173,8 @@
       <c r="AG94" s="2">
         <v>13</v>
       </c>
-      <c r="AH94" s="1" t="s">
-        <v>4911</v>
+      <c r="AH94" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26278,8 +26277,8 @@
       <c r="AG95" s="4">
         <v>13</v>
       </c>
-      <c r="AH95" s="3" t="s">
-        <v>4911</v>
+      <c r="AH95" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26382,8 +26381,8 @@
       <c r="AG96" s="2">
         <v>13</v>
       </c>
-      <c r="AH96" s="1" t="s">
-        <v>4911</v>
+      <c r="AH96" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26486,8 +26485,8 @@
       <c r="AG97" s="4">
         <v>13</v>
       </c>
-      <c r="AH97" s="3" t="s">
-        <v>4911</v>
+      <c r="AH97" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26590,8 +26589,8 @@
       <c r="AG98" s="2">
         <v>13</v>
       </c>
-      <c r="AH98" s="1" t="s">
-        <v>4911</v>
+      <c r="AH98" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26694,8 +26693,8 @@
       <c r="AG99" s="4">
         <v>13</v>
       </c>
-      <c r="AH99" s="3" t="s">
-        <v>4911</v>
+      <c r="AH99" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26798,8 +26797,8 @@
       <c r="AG100" s="2">
         <v>13</v>
       </c>
-      <c r="AH100" s="1" t="s">
-        <v>4911</v>
+      <c r="AH100" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26902,8 +26901,8 @@
       <c r="AG101" s="4">
         <v>13</v>
       </c>
-      <c r="AH101" s="3" t="s">
-        <v>4911</v>
+      <c r="AH101" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27006,8 +27005,8 @@
       <c r="AG102" s="2">
         <v>13</v>
       </c>
-      <c r="AH102" s="1" t="s">
-        <v>4911</v>
+      <c r="AH102" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27110,8 +27109,8 @@
       <c r="AG103" s="4">
         <v>13</v>
       </c>
-      <c r="AH103" s="3" t="s">
-        <v>4911</v>
+      <c r="AH103" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27214,8 +27213,8 @@
       <c r="AG104" s="2">
         <v>13</v>
       </c>
-      <c r="AH104" s="1" t="s">
-        <v>4911</v>
+      <c r="AH104" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27318,8 +27317,8 @@
       <c r="AG105" s="4">
         <v>13</v>
       </c>
-      <c r="AH105" s="3" t="s">
-        <v>4911</v>
+      <c r="AH105" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27422,8 +27421,8 @@
       <c r="AG106" s="2">
         <v>13</v>
       </c>
-      <c r="AH106" s="1" t="s">
-        <v>4911</v>
+      <c r="AH106" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27526,8 +27525,8 @@
       <c r="AG107" s="4">
         <v>13</v>
       </c>
-      <c r="AH107" s="3" t="s">
-        <v>4911</v>
+      <c r="AH107" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27630,8 +27629,8 @@
       <c r="AG108" s="2">
         <v>13</v>
       </c>
-      <c r="AH108" s="1" t="s">
-        <v>4911</v>
+      <c r="AH108" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27734,8 +27733,8 @@
       <c r="AG109" s="4">
         <v>13</v>
       </c>
-      <c r="AH109" s="3" t="s">
-        <v>4911</v>
+      <c r="AH109" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27838,8 +27837,8 @@
       <c r="AG110" s="2">
         <v>13</v>
       </c>
-      <c r="AH110" s="1" t="s">
-        <v>4911</v>
+      <c r="AH110" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27942,8 +27941,8 @@
       <c r="AG111" s="4">
         <v>13</v>
       </c>
-      <c r="AH111" s="3" t="s">
-        <v>4911</v>
+      <c r="AH111" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28046,8 +28045,8 @@
       <c r="AG112" s="2">
         <v>13</v>
       </c>
-      <c r="AH112" s="1" t="s">
-        <v>4911</v>
+      <c r="AH112" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28150,8 +28149,8 @@
       <c r="AG113" s="4">
         <v>13</v>
       </c>
-      <c r="AH113" s="3" t="s">
-        <v>4911</v>
+      <c r="AH113" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28254,8 +28253,8 @@
       <c r="AG114" s="2">
         <v>13</v>
       </c>
-      <c r="AH114" s="1" t="s">
-        <v>4911</v>
+      <c r="AH114" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28358,8 +28357,8 @@
       <c r="AG115" s="4">
         <v>13</v>
       </c>
-      <c r="AH115" s="3" t="s">
-        <v>4911</v>
+      <c r="AH115" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28462,8 +28461,8 @@
       <c r="AG116" s="2">
         <v>13</v>
       </c>
-      <c r="AH116" s="1" t="s">
-        <v>4911</v>
+      <c r="AH116" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28566,8 +28565,8 @@
       <c r="AG117" s="4">
         <v>5</v>
       </c>
-      <c r="AH117" s="3" t="s">
-        <v>4911</v>
+      <c r="AH117" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28670,8 +28669,8 @@
       <c r="AG118" s="2">
         <v>13</v>
       </c>
-      <c r="AH118" s="1" t="s">
-        <v>4911</v>
+      <c r="AH118" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28774,8 +28773,8 @@
       <c r="AG119" s="4">
         <v>13</v>
       </c>
-      <c r="AH119" s="3" t="s">
-        <v>4911</v>
+      <c r="AH119" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28878,8 +28877,8 @@
       <c r="AG120" s="2">
         <v>13</v>
       </c>
-      <c r="AH120" s="1" t="s">
-        <v>4911</v>
+      <c r="AH120" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28982,8 +28981,8 @@
       <c r="AG121" s="4">
         <v>13</v>
       </c>
-      <c r="AH121" s="3" t="s">
-        <v>4911</v>
+      <c r="AH121" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29086,8 +29085,8 @@
       <c r="AG122" s="2">
         <v>13</v>
       </c>
-      <c r="AH122" s="1" t="s">
-        <v>4911</v>
+      <c r="AH122" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29190,8 +29189,8 @@
       <c r="AG123" s="4">
         <v>13</v>
       </c>
-      <c r="AH123" s="3" t="s">
-        <v>4911</v>
+      <c r="AH123" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29294,8 +29293,8 @@
       <c r="AG124" s="2">
         <v>13</v>
       </c>
-      <c r="AH124" s="1" t="s">
-        <v>4911</v>
+      <c r="AH124" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29398,8 +29397,8 @@
       <c r="AG125" s="4">
         <v>13</v>
       </c>
-      <c r="AH125" s="3" t="s">
-        <v>4911</v>
+      <c r="AH125" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29502,8 +29501,8 @@
       <c r="AG126" s="2">
         <v>13</v>
       </c>
-      <c r="AH126" s="1" t="s">
-        <v>4911</v>
+      <c r="AH126" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29606,8 +29605,8 @@
       <c r="AG127" s="4">
         <v>13</v>
       </c>
-      <c r="AH127" s="3" t="s">
-        <v>4911</v>
+      <c r="AH127" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29710,8 +29709,8 @@
       <c r="AG128" s="2">
         <v>13</v>
       </c>
-      <c r="AH128" s="1" t="s">
-        <v>4911</v>
+      <c r="AH128" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29814,8 +29813,8 @@
       <c r="AG129" s="4">
         <v>13</v>
       </c>
-      <c r="AH129" s="3" t="s">
-        <v>4911</v>
+      <c r="AH129" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29918,8 +29917,8 @@
       <c r="AG130" s="2">
         <v>13</v>
       </c>
-      <c r="AH130" s="1" t="s">
-        <v>4911</v>
+      <c r="AH130" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30022,8 +30021,8 @@
       <c r="AG131" s="4">
         <v>5</v>
       </c>
-      <c r="AH131" s="3" t="s">
-        <v>4911</v>
+      <c r="AH131" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30126,8 +30125,8 @@
       <c r="AG132" s="2">
         <v>5</v>
       </c>
-      <c r="AH132" s="1" t="s">
-        <v>4911</v>
+      <c r="AH132" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30230,8 +30229,8 @@
       <c r="AG133" s="4">
         <v>13</v>
       </c>
-      <c r="AH133" s="3" t="s">
-        <v>4911</v>
+      <c r="AH133" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30334,8 +30333,8 @@
       <c r="AG134" s="2">
         <v>13</v>
       </c>
-      <c r="AH134" s="1" t="s">
-        <v>4911</v>
+      <c r="AH134" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30438,8 +30437,8 @@
       <c r="AG135" s="4">
         <v>13</v>
       </c>
-      <c r="AH135" s="3" t="s">
-        <v>4911</v>
+      <c r="AH135" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30542,8 +30541,8 @@
       <c r="AG136" s="2">
         <v>13</v>
       </c>
-      <c r="AH136" s="1" t="s">
-        <v>4911</v>
+      <c r="AH136" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30646,8 +30645,8 @@
       <c r="AG137" s="4">
         <v>13</v>
       </c>
-      <c r="AH137" s="3" t="s">
-        <v>4911</v>
+      <c r="AH137" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30750,8 +30749,8 @@
       <c r="AG138" s="2">
         <v>13</v>
       </c>
-      <c r="AH138" s="1" t="s">
-        <v>4911</v>
+      <c r="AH138" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30854,8 +30853,8 @@
       <c r="AG139" s="4">
         <v>13</v>
       </c>
-      <c r="AH139" s="3" t="s">
-        <v>4911</v>
+      <c r="AH139" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30958,8 +30957,8 @@
       <c r="AG140" s="2">
         <v>13</v>
       </c>
-      <c r="AH140" s="1" t="s">
-        <v>4911</v>
+      <c r="AH140" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31062,8 +31061,8 @@
       <c r="AG141" s="4">
         <v>13</v>
       </c>
-      <c r="AH141" s="3" t="s">
-        <v>4911</v>
+      <c r="AH141" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31166,8 +31165,8 @@
       <c r="AG142" s="2">
         <v>13</v>
       </c>
-      <c r="AH142" s="1" t="s">
-        <v>4911</v>
+      <c r="AH142" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31270,8 +31269,8 @@
       <c r="AG143" s="4">
         <v>13</v>
       </c>
-      <c r="AH143" s="3" t="s">
-        <v>4911</v>
+      <c r="AH143" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31374,8 +31373,8 @@
       <c r="AG144" s="2">
         <v>13</v>
       </c>
-      <c r="AH144" s="1" t="s">
-        <v>4911</v>
+      <c r="AH144" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31478,8 +31477,8 @@
       <c r="AG145" s="4">
         <v>13</v>
       </c>
-      <c r="AH145" s="3" t="s">
-        <v>4911</v>
+      <c r="AH145" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31582,8 +31581,8 @@
       <c r="AG146" s="2">
         <v>13</v>
       </c>
-      <c r="AH146" s="1" t="s">
-        <v>4911</v>
+      <c r="AH146" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31686,8 +31685,8 @@
       <c r="AG147" s="4">
         <v>13</v>
       </c>
-      <c r="AH147" s="3" t="s">
-        <v>4911</v>
+      <c r="AH147" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31790,8 +31789,8 @@
       <c r="AG148" s="2">
         <v>13</v>
       </c>
-      <c r="AH148" s="1" t="s">
-        <v>4911</v>
+      <c r="AH148" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31894,8 +31893,8 @@
       <c r="AG149" s="4">
         <v>13</v>
       </c>
-      <c r="AH149" s="3" t="s">
-        <v>4911</v>
+      <c r="AH149" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -31998,8 +31997,8 @@
       <c r="AG150" s="2">
         <v>13</v>
       </c>
-      <c r="AH150" s="1" t="s">
-        <v>4911</v>
+      <c r="AH150" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32102,8 +32101,8 @@
       <c r="AG151" s="4">
         <v>5</v>
       </c>
-      <c r="AH151" s="3" t="s">
-        <v>4911</v>
+      <c r="AH151" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32206,8 +32205,8 @@
       <c r="AG152" s="2">
         <v>13</v>
       </c>
-      <c r="AH152" s="1" t="s">
-        <v>4911</v>
+      <c r="AH152" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32310,8 +32309,8 @@
       <c r="AG153" s="4">
         <v>13</v>
       </c>
-      <c r="AH153" s="3" t="s">
-        <v>4911</v>
+      <c r="AH153" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32414,8 +32413,8 @@
       <c r="AG154" s="2">
         <v>13</v>
       </c>
-      <c r="AH154" s="1" t="s">
-        <v>4911</v>
+      <c r="AH154" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32518,8 +32517,8 @@
       <c r="AG155" s="4">
         <v>13</v>
       </c>
-      <c r="AH155" s="3" t="s">
-        <v>4911</v>
+      <c r="AH155" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32622,8 +32621,8 @@
       <c r="AG156" s="2">
         <v>13</v>
       </c>
-      <c r="AH156" s="1" t="s">
-        <v>4911</v>
+      <c r="AH156" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32726,8 +32725,8 @@
       <c r="AG157" s="4">
         <v>13</v>
       </c>
-      <c r="AH157" s="3" t="s">
-        <v>4911</v>
+      <c r="AH157" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32830,8 +32829,8 @@
       <c r="AG158" s="2">
         <v>13</v>
       </c>
-      <c r="AH158" s="1" t="s">
-        <v>4911</v>
+      <c r="AH158" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32934,8 +32933,8 @@
       <c r="AG159" s="4">
         <v>13</v>
       </c>
-      <c r="AH159" s="3" t="s">
-        <v>4911</v>
+      <c r="AH159" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33038,8 +33037,8 @@
       <c r="AG160" s="2">
         <v>13</v>
       </c>
-      <c r="AH160" s="1" t="s">
-        <v>4911</v>
+      <c r="AH160" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33142,8 +33141,8 @@
       <c r="AG161" s="4">
         <v>13</v>
       </c>
-      <c r="AH161" s="3" t="s">
-        <v>4911</v>
+      <c r="AH161" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33246,8 +33245,8 @@
       <c r="AG162" s="2">
         <v>13</v>
       </c>
-      <c r="AH162" s="1" t="s">
-        <v>4911</v>
+      <c r="AH162" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33350,8 +33349,8 @@
       <c r="AG163" s="4">
         <v>5</v>
       </c>
-      <c r="AH163" s="3" t="s">
-        <v>4911</v>
+      <c r="AH163" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33454,8 +33453,8 @@
       <c r="AG164" s="2">
         <v>13</v>
       </c>
-      <c r="AH164" s="1" t="s">
-        <v>4911</v>
+      <c r="AH164" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33558,8 +33557,8 @@
       <c r="AG165" s="4">
         <v>13</v>
       </c>
-      <c r="AH165" s="3" t="s">
-        <v>4911</v>
+      <c r="AH165" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33662,8 +33661,8 @@
       <c r="AG166" s="2">
         <v>13</v>
       </c>
-      <c r="AH166" s="1" t="s">
-        <v>4911</v>
+      <c r="AH166" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33766,8 +33765,8 @@
       <c r="AG167" s="4">
         <v>13</v>
       </c>
-      <c r="AH167" s="3" t="s">
-        <v>4911</v>
+      <c r="AH167" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33870,8 +33869,8 @@
       <c r="AG168" s="2">
         <v>13</v>
       </c>
-      <c r="AH168" s="1" t="s">
-        <v>4911</v>
+      <c r="AH168" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33974,8 +33973,8 @@
       <c r="AG169" s="4">
         <v>13</v>
       </c>
-      <c r="AH169" s="3" t="s">
-        <v>4911</v>
+      <c r="AH169" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34078,8 +34077,8 @@
       <c r="AG170" s="2">
         <v>13</v>
       </c>
-      <c r="AH170" s="1" t="s">
-        <v>4911</v>
+      <c r="AH170" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34182,8 +34181,8 @@
       <c r="AG171" s="4">
         <v>13</v>
       </c>
-      <c r="AH171" s="3" t="s">
-        <v>4911</v>
+      <c r="AH171" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34286,8 +34285,8 @@
       <c r="AG172" s="2">
         <v>13</v>
       </c>
-      <c r="AH172" s="1" t="s">
-        <v>4911</v>
+      <c r="AH172" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34390,8 +34389,8 @@
       <c r="AG173" s="4">
         <v>13</v>
       </c>
-      <c r="AH173" s="3" t="s">
-        <v>4911</v>
+      <c r="AH173" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34494,8 +34493,8 @@
       <c r="AG174" s="2">
         <v>13</v>
       </c>
-      <c r="AH174" s="1" t="s">
-        <v>4911</v>
+      <c r="AH174" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34598,8 +34597,8 @@
       <c r="AG175" s="4">
         <v>13</v>
       </c>
-      <c r="AH175" s="3" t="s">
-        <v>4911</v>
+      <c r="AH175" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34702,8 +34701,8 @@
       <c r="AG176" s="2">
         <v>13</v>
       </c>
-      <c r="AH176" s="1" t="s">
-        <v>4911</v>
+      <c r="AH176" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34806,8 +34805,8 @@
       <c r="AG177" s="4">
         <v>13</v>
       </c>
-      <c r="AH177" s="3" t="s">
-        <v>4911</v>
+      <c r="AH177" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34910,8 +34909,8 @@
       <c r="AG178" s="2">
         <v>13</v>
       </c>
-      <c r="AH178" s="1" t="s">
-        <v>4911</v>
+      <c r="AH178" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35014,8 +35013,8 @@
       <c r="AG179" s="4">
         <v>13</v>
       </c>
-      <c r="AH179" s="3" t="s">
-        <v>4911</v>
+      <c r="AH179" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35118,8 +35117,8 @@
       <c r="AG180" s="2">
         <v>13</v>
       </c>
-      <c r="AH180" s="1" t="s">
-        <v>4911</v>
+      <c r="AH180" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35222,8 +35221,8 @@
       <c r="AG181" s="4">
         <v>13</v>
       </c>
-      <c r="AH181" s="3" t="s">
-        <v>4911</v>
+      <c r="AH181" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35326,8 +35325,8 @@
       <c r="AG182" s="2">
         <v>6</v>
       </c>
-      <c r="AH182" s="1" t="s">
-        <v>4911</v>
+      <c r="AH182" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35430,8 +35429,8 @@
       <c r="AG183" s="4">
         <v>13</v>
       </c>
-      <c r="AH183" s="3" t="s">
-        <v>4911</v>
+      <c r="AH183" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35534,8 +35533,8 @@
       <c r="AG184" s="2">
         <v>13</v>
       </c>
-      <c r="AH184" s="1" t="s">
-        <v>4911</v>
+      <c r="AH184" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35638,8 +35637,8 @@
       <c r="AG185" s="4">
         <v>13</v>
       </c>
-      <c r="AH185" s="3" t="s">
-        <v>4911</v>
+      <c r="AH185" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35742,8 +35741,8 @@
       <c r="AG186" s="2">
         <v>13</v>
       </c>
-      <c r="AH186" s="1" t="s">
-        <v>4911</v>
+      <c r="AH186" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35846,8 +35845,8 @@
       <c r="AG187" s="4">
         <v>13</v>
       </c>
-      <c r="AH187" s="3" t="s">
-        <v>4911</v>
+      <c r="AH187" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35950,8 +35949,8 @@
       <c r="AG188" s="2">
         <v>5</v>
       </c>
-      <c r="AH188" s="1" t="s">
-        <v>4911</v>
+      <c r="AH188" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36054,8 +36053,8 @@
       <c r="AG189" s="4">
         <v>13</v>
       </c>
-      <c r="AH189" s="3" t="s">
-        <v>4911</v>
+      <c r="AH189" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36158,8 +36157,8 @@
       <c r="AG190" s="2">
         <v>13</v>
       </c>
-      <c r="AH190" s="1" t="s">
-        <v>4911</v>
+      <c r="AH190" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36262,8 +36261,8 @@
       <c r="AG191" s="4">
         <v>13</v>
       </c>
-      <c r="AH191" s="3" t="s">
-        <v>4911</v>
+      <c r="AH191" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36366,8 +36365,8 @@
       <c r="AG192" s="2">
         <v>7</v>
       </c>
-      <c r="AH192" s="1" t="s">
-        <v>4911</v>
+      <c r="AH192" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36470,8 +36469,8 @@
       <c r="AG193" s="4">
         <v>13</v>
       </c>
-      <c r="AH193" s="3" t="s">
-        <v>4911</v>
+      <c r="AH193" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36574,8 +36573,8 @@
       <c r="AG194" s="2">
         <v>13</v>
       </c>
-      <c r="AH194" s="1" t="s">
-        <v>4911</v>
+      <c r="AH194" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36678,8 +36677,8 @@
       <c r="AG195" s="4">
         <v>13</v>
       </c>
-      <c r="AH195" s="3" t="s">
-        <v>4911</v>
+      <c r="AH195" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36782,8 +36781,8 @@
       <c r="AG196" s="2">
         <v>13</v>
       </c>
-      <c r="AH196" s="1" t="s">
-        <v>4911</v>
+      <c r="AH196" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36886,8 +36885,8 @@
       <c r="AG197" s="4">
         <v>13</v>
       </c>
-      <c r="AH197" s="3" t="s">
-        <v>4911</v>
+      <c r="AH197" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36990,8 +36989,8 @@
       <c r="AG198" s="2">
         <v>13</v>
       </c>
-      <c r="AH198" s="1" t="s">
-        <v>4911</v>
+      <c r="AH198" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37094,8 +37093,8 @@
       <c r="AG199" s="4">
         <v>13</v>
       </c>
-      <c r="AH199" s="3" t="s">
-        <v>4911</v>
+      <c r="AH199" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37198,8 +37197,8 @@
       <c r="AG200" s="2">
         <v>13</v>
       </c>
-      <c r="AH200" s="1" t="s">
-        <v>4911</v>
+      <c r="AH200" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37302,8 +37301,8 @@
       <c r="AG201" s="4">
         <v>13</v>
       </c>
-      <c r="AH201" s="3" t="s">
-        <v>4911</v>
+      <c r="AH201" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37406,8 +37405,8 @@
       <c r="AG202" s="2">
         <v>5</v>
       </c>
-      <c r="AH202" s="1" t="s">
-        <v>4911</v>
+      <c r="AH202" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37510,8 +37509,8 @@
       <c r="AG203" s="4">
         <v>13</v>
       </c>
-      <c r="AH203" s="3" t="s">
-        <v>4911</v>
+      <c r="AH203" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37614,8 +37613,8 @@
       <c r="AG204" s="2">
         <v>13</v>
       </c>
-      <c r="AH204" s="1" t="s">
-        <v>4911</v>
+      <c r="AH204" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37718,8 +37717,8 @@
       <c r="AG205" s="4">
         <v>13</v>
       </c>
-      <c r="AH205" s="3" t="s">
-        <v>4911</v>
+      <c r="AH205" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37822,8 +37821,8 @@
       <c r="AG206" s="2">
         <v>13</v>
       </c>
-      <c r="AH206" s="1" t="s">
-        <v>4911</v>
+      <c r="AH206" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37926,8 +37925,8 @@
       <c r="AG207" s="4">
         <v>13</v>
       </c>
-      <c r="AH207" s="3" t="s">
-        <v>4911</v>
+      <c r="AH207" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38030,8 +38029,8 @@
       <c r="AG208" s="2">
         <v>13</v>
       </c>
-      <c r="AH208" s="1" t="s">
-        <v>4911</v>
+      <c r="AH208" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38134,8 +38133,8 @@
       <c r="AG209" s="4">
         <v>13</v>
       </c>
-      <c r="AH209" s="3" t="s">
-        <v>4911</v>
+      <c r="AH209" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38238,8 +38237,8 @@
       <c r="AG210" s="2">
         <v>10</v>
       </c>
-      <c r="AH210" s="1" t="s">
-        <v>4911</v>
+      <c r="AH210" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38342,8 +38341,8 @@
       <c r="AG211" s="4">
         <v>5</v>
       </c>
-      <c r="AH211" s="3" t="s">
-        <v>4911</v>
+      <c r="AH211" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38446,8 +38445,8 @@
       <c r="AG212" s="2">
         <v>13</v>
       </c>
-      <c r="AH212" s="1" t="s">
-        <v>4911</v>
+      <c r="AH212" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38550,8 +38549,8 @@
       <c r="AG213" s="4">
         <v>13</v>
       </c>
-      <c r="AH213" s="3" t="s">
-        <v>4911</v>
+      <c r="AH213" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38654,8 +38653,8 @@
       <c r="AG214" s="2">
         <v>13</v>
       </c>
-      <c r="AH214" s="1" t="s">
-        <v>4911</v>
+      <c r="AH214" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38758,8 +38757,8 @@
       <c r="AG215" s="4">
         <v>13</v>
       </c>
-      <c r="AH215" s="3" t="s">
-        <v>4911</v>
+      <c r="AH215" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38862,8 +38861,8 @@
       <c r="AG216" s="2">
         <v>13</v>
       </c>
-      <c r="AH216" s="1" t="s">
-        <v>4911</v>
+      <c r="AH216" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38966,8 +38965,8 @@
       <c r="AG217" s="4">
         <v>6</v>
       </c>
-      <c r="AH217" s="3" t="s">
-        <v>4911</v>
+      <c r="AH217" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39070,8 +39069,8 @@
       <c r="AG218" s="2">
         <v>13</v>
       </c>
-      <c r="AH218" s="1" t="s">
-        <v>4911</v>
+      <c r="AH218" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39174,8 +39173,8 @@
       <c r="AG219" s="4">
         <v>13</v>
       </c>
-      <c r="AH219" s="3" t="s">
-        <v>4911</v>
+      <c r="AH219" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39278,8 +39277,8 @@
       <c r="AG220" s="2">
         <v>5</v>
       </c>
-      <c r="AH220" s="1" t="s">
-        <v>4911</v>
+      <c r="AH220" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39382,8 +39381,8 @@
       <c r="AG221" s="4">
         <v>13</v>
       </c>
-      <c r="AH221" s="3" t="s">
-        <v>4911</v>
+      <c r="AH221" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39486,8 +39485,8 @@
       <c r="AG222" s="2">
         <v>13</v>
       </c>
-      <c r="AH222" s="1" t="s">
-        <v>4911</v>
+      <c r="AH222" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39590,8 +39589,8 @@
       <c r="AG223" s="4">
         <v>13</v>
       </c>
-      <c r="AH223" s="3" t="s">
-        <v>4911</v>
+      <c r="AH223" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39694,8 +39693,8 @@
       <c r="AG224" s="2">
         <v>13</v>
       </c>
-      <c r="AH224" s="1" t="s">
-        <v>4911</v>
+      <c r="AH224" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39798,8 +39797,8 @@
       <c r="AG225" s="4">
         <v>13</v>
       </c>
-      <c r="AH225" s="3" t="s">
-        <v>4911</v>
+      <c r="AH225" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39902,8 +39901,8 @@
       <c r="AG226" s="2">
         <v>13</v>
       </c>
-      <c r="AH226" s="1" t="s">
-        <v>4911</v>
+      <c r="AH226" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40006,8 +40005,8 @@
       <c r="AG227" s="4">
         <v>13</v>
       </c>
-      <c r="AH227" s="3" t="s">
-        <v>4911</v>
+      <c r="AH227" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40110,8 +40109,8 @@
       <c r="AG228" s="2">
         <v>13</v>
       </c>
-      <c r="AH228" s="1" t="s">
-        <v>4911</v>
+      <c r="AH228" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40214,8 +40213,8 @@
       <c r="AG229" s="4">
         <v>13</v>
       </c>
-      <c r="AH229" s="3" t="s">
-        <v>4911</v>
+      <c r="AH229" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40318,8 +40317,8 @@
       <c r="AG230" s="2">
         <v>13</v>
       </c>
-      <c r="AH230" s="1" t="s">
-        <v>4911</v>
+      <c r="AH230" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40422,8 +40421,8 @@
       <c r="AG231" s="4">
         <v>13</v>
       </c>
-      <c r="AH231" s="3" t="s">
-        <v>4911</v>
+      <c r="AH231" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40526,8 +40525,8 @@
       <c r="AG232" s="2">
         <v>13</v>
       </c>
-      <c r="AH232" s="1" t="s">
-        <v>4911</v>
+      <c r="AH232" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40630,8 +40629,8 @@
       <c r="AG233" s="4">
         <v>13</v>
       </c>
-      <c r="AH233" s="3" t="s">
-        <v>4911</v>
+      <c r="AH233" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40734,8 +40733,8 @@
       <c r="AG234" s="2">
         <v>13</v>
       </c>
-      <c r="AH234" s="1" t="s">
-        <v>4911</v>
+      <c r="AH234" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40838,8 +40837,8 @@
       <c r="AG235" s="4">
         <v>13</v>
       </c>
-      <c r="AH235" s="3" t="s">
-        <v>4911</v>
+      <c r="AH235" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40942,8 +40941,8 @@
       <c r="AG236" s="2">
         <v>13</v>
       </c>
-      <c r="AH236" s="1" t="s">
-        <v>4911</v>
+      <c r="AH236" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41046,8 +41045,8 @@
       <c r="AG237" s="4">
         <v>13</v>
       </c>
-      <c r="AH237" s="3" t="s">
-        <v>4911</v>
+      <c r="AH237" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41150,8 +41149,8 @@
       <c r="AG238" s="2">
         <v>13</v>
       </c>
-      <c r="AH238" s="1" t="s">
-        <v>4911</v>
+      <c r="AH238" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41254,8 +41253,8 @@
       <c r="AG239" s="4">
         <v>13</v>
       </c>
-      <c r="AH239" s="3" t="s">
-        <v>4911</v>
+      <c r="AH239" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41358,8 +41357,8 @@
       <c r="AG240" s="2">
         <v>13</v>
       </c>
-      <c r="AH240" s="1" t="s">
-        <v>4911</v>
+      <c r="AH240" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41462,8 +41461,8 @@
       <c r="AG241" s="4">
         <v>13</v>
       </c>
-      <c r="AH241" s="3" t="s">
-        <v>4911</v>
+      <c r="AH241" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41566,8 +41565,8 @@
       <c r="AG242" s="2">
         <v>5</v>
       </c>
-      <c r="AH242" s="1" t="s">
-        <v>4911</v>
+      <c r="AH242" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41670,8 +41669,8 @@
       <c r="AG243" s="4">
         <v>13</v>
       </c>
-      <c r="AH243" s="3" t="s">
-        <v>4911</v>
+      <c r="AH243" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41774,8 +41773,8 @@
       <c r="AG244" s="2">
         <v>13</v>
       </c>
-      <c r="AH244" s="1" t="s">
-        <v>4911</v>
+      <c r="AH244" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41878,8 +41877,8 @@
       <c r="AG245" s="4">
         <v>13</v>
       </c>
-      <c r="AH245" s="3" t="s">
-        <v>4911</v>
+      <c r="AH245" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41982,8 +41981,8 @@
       <c r="AG246" s="2">
         <v>13</v>
       </c>
-      <c r="AH246" s="1" t="s">
-        <v>4911</v>
+      <c r="AH246" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42086,8 +42085,8 @@
       <c r="AG247" s="4">
         <v>13</v>
       </c>
-      <c r="AH247" s="3" t="s">
-        <v>4911</v>
+      <c r="AH247" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42190,8 +42189,8 @@
       <c r="AG248" s="2">
         <v>13</v>
       </c>
-      <c r="AH248" s="1" t="s">
-        <v>4911</v>
+      <c r="AH248" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42294,8 +42293,8 @@
       <c r="AG249" s="4">
         <v>13</v>
       </c>
-      <c r="AH249" s="3" t="s">
-        <v>4911</v>
+      <c r="AH249" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42398,8 +42397,8 @@
       <c r="AG250" s="2">
         <v>13</v>
       </c>
-      <c r="AH250" s="1" t="s">
-        <v>4911</v>
+      <c r="AH250" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42502,8 +42501,8 @@
       <c r="AG251" s="4">
         <v>13</v>
       </c>
-      <c r="AH251" s="3" t="s">
-        <v>4911</v>
+      <c r="AH251" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42606,8 +42605,8 @@
       <c r="AG252" s="2">
         <v>13</v>
       </c>
-      <c r="AH252" s="1" t="s">
-        <v>4911</v>
+      <c r="AH252" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42710,8 +42709,8 @@
       <c r="AG253" s="4">
         <v>13</v>
       </c>
-      <c r="AH253" s="3" t="s">
-        <v>4911</v>
+      <c r="AH253" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42814,8 +42813,8 @@
       <c r="AG254" s="2">
         <v>13</v>
       </c>
-      <c r="AH254" s="1" t="s">
-        <v>4911</v>
+      <c r="AH254" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42918,8 +42917,8 @@
       <c r="AG255" s="4">
         <v>13</v>
       </c>
-      <c r="AH255" s="3" t="s">
-        <v>4911</v>
+      <c r="AH255" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43022,8 +43021,8 @@
       <c r="AG256" s="2">
         <v>13</v>
       </c>
-      <c r="AH256" s="1" t="s">
-        <v>4911</v>
+      <c r="AH256" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43126,8 +43125,8 @@
       <c r="AG257" s="4">
         <v>13</v>
       </c>
-      <c r="AH257" s="3" t="s">
-        <v>4911</v>
+      <c r="AH257" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43230,8 +43229,8 @@
       <c r="AG258" s="2">
         <v>13</v>
       </c>
-      <c r="AH258" s="1" t="s">
-        <v>4911</v>
+      <c r="AH258" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43334,8 +43333,8 @@
       <c r="AG259" s="4">
         <v>13</v>
       </c>
-      <c r="AH259" s="3" t="s">
-        <v>4911</v>
+      <c r="AH259" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43438,8 +43437,8 @@
       <c r="AG260" s="2">
         <v>13</v>
       </c>
-      <c r="AH260" s="1" t="s">
-        <v>4911</v>
+      <c r="AH260" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43542,8 +43541,8 @@
       <c r="AG261" s="4">
         <v>13</v>
       </c>
-      <c r="AH261" s="3" t="s">
-        <v>4911</v>
+      <c r="AH261" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43646,8 +43645,8 @@
       <c r="AG262" s="2">
         <v>13</v>
       </c>
-      <c r="AH262" s="1" t="s">
-        <v>4911</v>
+      <c r="AH262" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43750,8 +43749,8 @@
       <c r="AG263" s="4">
         <v>13</v>
       </c>
-      <c r="AH263" s="3" t="s">
-        <v>4911</v>
+      <c r="AH263" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43854,8 +43853,8 @@
       <c r="AG264" s="2">
         <v>13</v>
       </c>
-      <c r="AH264" s="1" t="s">
-        <v>4911</v>
+      <c r="AH264" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43958,8 +43957,8 @@
       <c r="AG265" s="4">
         <v>13</v>
       </c>
-      <c r="AH265" s="3" t="s">
-        <v>4911</v>
+      <c r="AH265" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44062,8 +44061,8 @@
       <c r="AG266" s="2">
         <v>13</v>
       </c>
-      <c r="AH266" s="1" t="s">
-        <v>4911</v>
+      <c r="AH266" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44166,8 +44165,8 @@
       <c r="AG267" s="4">
         <v>13</v>
       </c>
-      <c r="AH267" s="3" t="s">
-        <v>4911</v>
+      <c r="AH267" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44270,8 +44269,8 @@
       <c r="AG268" s="2">
         <v>13</v>
       </c>
-      <c r="AH268" s="1" t="s">
-        <v>4911</v>
+      <c r="AH268" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44374,8 +44373,8 @@
       <c r="AG269" s="4">
         <v>13</v>
       </c>
-      <c r="AH269" s="3" t="s">
-        <v>4911</v>
+      <c r="AH269" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44478,8 +44477,8 @@
       <c r="AG270" s="2">
         <v>13</v>
       </c>
-      <c r="AH270" s="1" t="s">
-        <v>4911</v>
+      <c r="AH270" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44582,8 +44581,8 @@
       <c r="AG271" s="4">
         <v>13</v>
       </c>
-      <c r="AH271" s="3" t="s">
-        <v>4911</v>
+      <c r="AH271" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44686,8 +44685,8 @@
       <c r="AG272" s="2">
         <v>13</v>
       </c>
-      <c r="AH272" s="1" t="s">
-        <v>4911</v>
+      <c r="AH272" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44790,8 +44789,8 @@
       <c r="AG273" s="4">
         <v>13</v>
       </c>
-      <c r="AH273" s="3" t="s">
-        <v>4911</v>
+      <c r="AH273" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44894,8 +44893,8 @@
       <c r="AG274" s="2">
         <v>13</v>
       </c>
-      <c r="AH274" s="1" t="s">
-        <v>4911</v>
+      <c r="AH274" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -44998,8 +44997,8 @@
       <c r="AG275" s="4">
         <v>13</v>
       </c>
-      <c r="AH275" s="3" t="s">
-        <v>4911</v>
+      <c r="AH275" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45102,8 +45101,8 @@
       <c r="AG276" s="2">
         <v>13</v>
       </c>
-      <c r="AH276" s="1" t="s">
-        <v>4911</v>
+      <c r="AH276" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45206,8 +45205,8 @@
       <c r="AG277" s="4">
         <v>13</v>
       </c>
-      <c r="AH277" s="3" t="s">
-        <v>4911</v>
+      <c r="AH277" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45310,8 +45309,8 @@
       <c r="AG278" s="2">
         <v>13</v>
       </c>
-      <c r="AH278" s="1" t="s">
-        <v>4911</v>
+      <c r="AH278" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45414,8 +45413,8 @@
       <c r="AG279" s="4">
         <v>13</v>
       </c>
-      <c r="AH279" s="3" t="s">
-        <v>4911</v>
+      <c r="AH279" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45518,8 +45517,8 @@
       <c r="AG280" s="2">
         <v>13</v>
       </c>
-      <c r="AH280" s="1" t="s">
-        <v>4911</v>
+      <c r="AH280" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45622,8 +45621,8 @@
       <c r="AG281" s="4">
         <v>13</v>
       </c>
-      <c r="AH281" s="3" t="s">
-        <v>4911</v>
+      <c r="AH281" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45726,8 +45725,8 @@
       <c r="AG282" s="2">
         <v>13</v>
       </c>
-      <c r="AH282" s="1" t="s">
-        <v>4911</v>
+      <c r="AH282" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45830,8 +45829,8 @@
       <c r="AG283" s="4">
         <v>5</v>
       </c>
-      <c r="AH283" s="3" t="s">
-        <v>4911</v>
+      <c r="AH283" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45934,8 +45933,8 @@
       <c r="AG284" s="2">
         <v>13</v>
       </c>
-      <c r="AH284" s="1" t="s">
-        <v>4911</v>
+      <c r="AH284" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46038,8 +46037,8 @@
       <c r="AG285" s="4">
         <v>13</v>
       </c>
-      <c r="AH285" s="3" t="s">
-        <v>4911</v>
+      <c r="AH285" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46142,8 +46141,8 @@
       <c r="AG286" s="2">
         <v>13</v>
       </c>
-      <c r="AH286" s="1" t="s">
-        <v>4911</v>
+      <c r="AH286" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46246,8 +46245,8 @@
       <c r="AG287" s="4">
         <v>13</v>
       </c>
-      <c r="AH287" s="3" t="s">
-        <v>4911</v>
+      <c r="AH287" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46350,8 +46349,8 @@
       <c r="AG288" s="2">
         <v>13</v>
       </c>
-      <c r="AH288" s="1" t="s">
-        <v>4911</v>
+      <c r="AH288" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46454,8 +46453,8 @@
       <c r="AG289" s="4">
         <v>13</v>
       </c>
-      <c r="AH289" s="3" t="s">
-        <v>4911</v>
+      <c r="AH289" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46558,8 +46557,8 @@
       <c r="AG290" s="2">
         <v>13</v>
       </c>
-      <c r="AH290" s="1" t="s">
-        <v>4911</v>
+      <c r="AH290" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46662,8 +46661,8 @@
       <c r="AG291" s="4">
         <v>13</v>
       </c>
-      <c r="AH291" s="3" t="s">
-        <v>4911</v>
+      <c r="AH291" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46766,8 +46765,8 @@
       <c r="AG292" s="2">
         <v>13</v>
       </c>
-      <c r="AH292" s="1" t="s">
-        <v>4911</v>
+      <c r="AH292" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46870,8 +46869,8 @@
       <c r="AG293" s="4">
         <v>13</v>
       </c>
-      <c r="AH293" s="3" t="s">
-        <v>4911</v>
+      <c r="AH293" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46974,8 +46973,8 @@
       <c r="AG294" s="2">
         <v>13</v>
       </c>
-      <c r="AH294" s="1" t="s">
-        <v>4911</v>
+      <c r="AH294" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47078,8 +47077,8 @@
       <c r="AG295" s="4">
         <v>13</v>
       </c>
-      <c r="AH295" s="3" t="s">
-        <v>4911</v>
+      <c r="AH295" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47182,8 +47181,8 @@
       <c r="AG296" s="2">
         <v>13</v>
       </c>
-      <c r="AH296" s="1" t="s">
-        <v>4911</v>
+      <c r="AH296" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47286,8 +47285,8 @@
       <c r="AG297" s="4">
         <v>13</v>
       </c>
-      <c r="AH297" s="3" t="s">
-        <v>4911</v>
+      <c r="AH297" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47390,8 +47389,8 @@
       <c r="AG298" s="2">
         <v>13</v>
       </c>
-      <c r="AH298" s="1" t="s">
-        <v>4911</v>
+      <c r="AH298" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47494,8 +47493,8 @@
       <c r="AG299" s="4">
         <v>13</v>
       </c>
-      <c r="AH299" s="3" t="s">
-        <v>4911</v>
+      <c r="AH299" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47598,8 +47597,8 @@
       <c r="AG300" s="2">
         <v>13</v>
       </c>
-      <c r="AH300" s="1" t="s">
-        <v>4911</v>
+      <c r="AH300" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47702,8 +47701,8 @@
       <c r="AG301" s="4">
         <v>13</v>
       </c>
-      <c r="AH301" s="3" t="s">
-        <v>4911</v>
+      <c r="AH301" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47806,8 +47805,8 @@
       <c r="AG302" s="2">
         <v>13</v>
       </c>
-      <c r="AH302" s="1" t="s">
-        <v>4911</v>
+      <c r="AH302" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47910,8 +47909,8 @@
       <c r="AG303" s="4">
         <v>13</v>
       </c>
-      <c r="AH303" s="3" t="s">
-        <v>4911</v>
+      <c r="AH303" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48014,8 +48013,8 @@
       <c r="AG304" s="2">
         <v>13</v>
       </c>
-      <c r="AH304" s="1" t="s">
-        <v>4911</v>
+      <c r="AH304" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48118,8 +48117,8 @@
       <c r="AG305" s="4">
         <v>13</v>
       </c>
-      <c r="AH305" s="3" t="s">
-        <v>4911</v>
+      <c r="AH305" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48222,8 +48221,8 @@
       <c r="AG306" s="2">
         <v>13</v>
       </c>
-      <c r="AH306" s="1" t="s">
-        <v>4911</v>
+      <c r="AH306" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48326,8 +48325,8 @@
       <c r="AG307" s="4">
         <v>13</v>
       </c>
-      <c r="AH307" s="3" t="s">
-        <v>4911</v>
+      <c r="AH307" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48430,8 +48429,8 @@
       <c r="AG308" s="2">
         <v>13</v>
       </c>
-      <c r="AH308" s="1" t="s">
-        <v>4911</v>
+      <c r="AH308" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48534,8 +48533,8 @@
       <c r="AG309" s="4">
         <v>13</v>
       </c>
-      <c r="AH309" s="3" t="s">
-        <v>4911</v>
+      <c r="AH309" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48638,8 +48637,8 @@
       <c r="AG310" s="2">
         <v>13</v>
       </c>
-      <c r="AH310" s="1" t="s">
-        <v>4911</v>
+      <c r="AH310" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48742,8 +48741,8 @@
       <c r="AG311" s="4">
         <v>13</v>
       </c>
-      <c r="AH311" s="3" t="s">
-        <v>4911</v>
+      <c r="AH311" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48846,8 +48845,8 @@
       <c r="AG312" s="2">
         <v>13</v>
       </c>
-      <c r="AH312" s="1" t="s">
-        <v>4911</v>
+      <c r="AH312" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48950,8 +48949,8 @@
       <c r="AG313" s="4">
         <v>13</v>
       </c>
-      <c r="AH313" s="3" t="s">
-        <v>4911</v>
+      <c r="AH313" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49054,8 +49053,8 @@
       <c r="AG314" s="2">
         <v>13</v>
       </c>
-      <c r="AH314" s="1" t="s">
-        <v>4911</v>
+      <c r="AH314" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49158,8 +49157,8 @@
       <c r="AG315" s="4">
         <v>13</v>
       </c>
-      <c r="AH315" s="3" t="s">
-        <v>4911</v>
+      <c r="AH315" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49262,8 +49261,8 @@
       <c r="AG316" s="2">
         <v>13</v>
       </c>
-      <c r="AH316" s="1" t="s">
-        <v>4911</v>
+      <c r="AH316" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49366,8 +49365,8 @@
       <c r="AG317" s="4">
         <v>8</v>
       </c>
-      <c r="AH317" s="3" t="s">
-        <v>4911</v>
+      <c r="AH317" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49470,8 +49469,8 @@
       <c r="AG318" s="2">
         <v>13</v>
       </c>
-      <c r="AH318" s="1" t="s">
-        <v>4911</v>
+      <c r="AH318" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49574,8 +49573,8 @@
       <c r="AG319" s="4">
         <v>13</v>
       </c>
-      <c r="AH319" s="3" t="s">
-        <v>4911</v>
+      <c r="AH319" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49678,8 +49677,8 @@
       <c r="AG320" s="2">
         <v>13</v>
       </c>
-      <c r="AH320" s="1" t="s">
-        <v>4911</v>
+      <c r="AH320" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49782,8 +49781,8 @@
       <c r="AG321" s="4">
         <v>13</v>
       </c>
-      <c r="AH321" s="3" t="s">
-        <v>4911</v>
+      <c r="AH321" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49886,8 +49885,8 @@
       <c r="AG322" s="2">
         <v>8</v>
       </c>
-      <c r="AH322" s="1" t="s">
-        <v>4911</v>
+      <c r="AH322" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49990,8 +49989,8 @@
       <c r="AG323" s="4">
         <v>13</v>
       </c>
-      <c r="AH323" s="3" t="s">
-        <v>4911</v>
+      <c r="AH323" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50094,8 +50093,8 @@
       <c r="AG324" s="2">
         <v>5</v>
       </c>
-      <c r="AH324" s="1" t="s">
-        <v>4911</v>
+      <c r="AH324" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50198,8 +50197,8 @@
       <c r="AG325" s="4">
         <v>13</v>
       </c>
-      <c r="AH325" s="3" t="s">
-        <v>4911</v>
+      <c r="AH325" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50302,8 +50301,8 @@
       <c r="AG326" s="2">
         <v>13</v>
       </c>
-      <c r="AH326" s="1" t="s">
-        <v>4911</v>
+      <c r="AH326" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50406,8 +50405,8 @@
       <c r="AG327" s="4">
         <v>13</v>
       </c>
-      <c r="AH327" s="3" t="s">
-        <v>4911</v>
+      <c r="AH327" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50510,8 +50509,8 @@
       <c r="AG328" s="2">
         <v>13</v>
       </c>
-      <c r="AH328" s="1" t="s">
-        <v>4911</v>
+      <c r="AH328" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50614,8 +50613,8 @@
       <c r="AG329" s="4">
         <v>13</v>
       </c>
-      <c r="AH329" s="3" t="s">
-        <v>4911</v>
+      <c r="AH329" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50718,8 +50717,8 @@
       <c r="AG330" s="2">
         <v>13</v>
       </c>
-      <c r="AH330" s="1" t="s">
-        <v>4911</v>
+      <c r="AH330" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50822,8 +50821,8 @@
       <c r="AG331" s="4">
         <v>13</v>
       </c>
-      <c r="AH331" s="3" t="s">
-        <v>4911</v>
+      <c r="AH331" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50926,8 +50925,8 @@
       <c r="AG332" s="2">
         <v>13</v>
       </c>
-      <c r="AH332" s="1" t="s">
-        <v>4911</v>
+      <c r="AH332" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51030,8 +51029,8 @@
       <c r="AG333" s="4">
         <v>13</v>
       </c>
-      <c r="AH333" s="3" t="s">
-        <v>4911</v>
+      <c r="AH333" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51134,8 +51133,8 @@
       <c r="AG334" s="2">
         <v>13</v>
       </c>
-      <c r="AH334" s="1" t="s">
-        <v>4911</v>
+      <c r="AH334" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51238,8 +51237,8 @@
       <c r="AG335" s="4">
         <v>13</v>
       </c>
-      <c r="AH335" s="3" t="s">
-        <v>4911</v>
+      <c r="AH335" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51342,8 +51341,8 @@
       <c r="AG336" s="2">
         <v>10</v>
       </c>
-      <c r="AH336" s="1" t="s">
-        <v>4911</v>
+      <c r="AH336" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51446,8 +51445,8 @@
       <c r="AG337" s="4">
         <v>13</v>
       </c>
-      <c r="AH337" s="3" t="s">
-        <v>4911</v>
+      <c r="AH337" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51550,8 +51549,8 @@
       <c r="AG338" s="2">
         <v>13</v>
       </c>
-      <c r="AH338" s="1" t="s">
-        <v>4911</v>
+      <c r="AH338" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51654,8 +51653,8 @@
       <c r="AG339" s="4">
         <v>13</v>
       </c>
-      <c r="AH339" s="3" t="s">
-        <v>4911</v>
+      <c r="AH339" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51758,8 +51757,8 @@
       <c r="AG340" s="2">
         <v>5</v>
       </c>
-      <c r="AH340" s="1" t="s">
-        <v>4911</v>
+      <c r="AH340" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51862,8 +51861,8 @@
       <c r="AG341" s="4">
         <v>13</v>
       </c>
-      <c r="AH341" s="3" t="s">
-        <v>4911</v>
+      <c r="AH341" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51966,8 +51965,8 @@
       <c r="AG342" s="2">
         <v>13</v>
       </c>
-      <c r="AH342" s="1" t="s">
-        <v>4911</v>
+      <c r="AH342" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52070,8 +52069,8 @@
       <c r="AG343" s="4">
         <v>13</v>
       </c>
-      <c r="AH343" s="3" t="s">
-        <v>4911</v>
+      <c r="AH343" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52174,8 +52173,8 @@
       <c r="AG344" s="2">
         <v>13</v>
       </c>
-      <c r="AH344" s="1" t="s">
-        <v>4911</v>
+      <c r="AH344" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52278,8 +52277,8 @@
       <c r="AG345" s="4">
         <v>13</v>
       </c>
-      <c r="AH345" s="3" t="s">
-        <v>4911</v>
+      <c r="AH345" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52382,8 +52381,8 @@
       <c r="AG346" s="2">
         <v>13</v>
       </c>
-      <c r="AH346" s="1" t="s">
-        <v>4911</v>
+      <c r="AH346" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52486,8 +52485,8 @@
       <c r="AG347" s="4">
         <v>13</v>
       </c>
-      <c r="AH347" s="3" t="s">
-        <v>4911</v>
+      <c r="AH347" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52590,8 +52589,8 @@
       <c r="AG348" s="2">
         <v>13</v>
       </c>
-      <c r="AH348" s="1" t="s">
-        <v>4911</v>
+      <c r="AH348" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52694,8 +52693,8 @@
       <c r="AG349" s="4">
         <v>13</v>
       </c>
-      <c r="AH349" s="3" t="s">
-        <v>4911</v>
+      <c r="AH349" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52798,8 +52797,8 @@
       <c r="AG350" s="2">
         <v>13</v>
       </c>
-      <c r="AH350" s="1" t="s">
-        <v>4911</v>
+      <c r="AH350" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52902,8 +52901,8 @@
       <c r="AG351" s="4">
         <v>13</v>
       </c>
-      <c r="AH351" s="3" t="s">
-        <v>4911</v>
+      <c r="AH351" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53006,8 +53005,8 @@
       <c r="AG352" s="2">
         <v>13</v>
       </c>
-      <c r="AH352" s="1" t="s">
-        <v>4911</v>
+      <c r="AH352" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53110,8 +53109,8 @@
       <c r="AG353" s="4">
         <v>13</v>
       </c>
-      <c r="AH353" s="3" t="s">
-        <v>4911</v>
+      <c r="AH353" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53214,8 +53213,8 @@
       <c r="AG354" s="2">
         <v>13</v>
       </c>
-      <c r="AH354" s="1" t="s">
-        <v>4911</v>
+      <c r="AH354" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53318,8 +53317,8 @@
       <c r="AG355" s="4">
         <v>13</v>
       </c>
-      <c r="AH355" s="3" t="s">
-        <v>4911</v>
+      <c r="AH355" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53422,8 +53421,8 @@
       <c r="AG356" s="2">
         <v>13</v>
       </c>
-      <c r="AH356" s="1" t="s">
-        <v>4911</v>
+      <c r="AH356" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53526,8 +53525,8 @@
       <c r="AG357" s="4">
         <v>13</v>
       </c>
-      <c r="AH357" s="3" t="s">
-        <v>4911</v>
+      <c r="AH357" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53580,8 +53579,8 @@
       <c r="AG358" s="2">
         <v>13</v>
       </c>
-      <c r="AH358" s="1" t="s">
-        <v>4911</v>
+      <c r="AH358" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53684,8 +53683,8 @@
       <c r="AG359" s="4">
         <v>13</v>
       </c>
-      <c r="AH359" s="3" t="s">
-        <v>4911</v>
+      <c r="AH359" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53788,8 +53787,8 @@
       <c r="AG360" s="2">
         <v>13</v>
       </c>
-      <c r="AH360" s="1" t="s">
-        <v>4911</v>
+      <c r="AH360" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53892,8 +53891,8 @@
       <c r="AG361" s="4">
         <v>13</v>
       </c>
-      <c r="AH361" s="3" t="s">
-        <v>4911</v>
+      <c r="AH361" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -53996,8 +53995,8 @@
       <c r="AG362" s="2">
         <v>13</v>
       </c>
-      <c r="AH362" s="1" t="s">
-        <v>4911</v>
+      <c r="AH362" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54100,8 +54099,8 @@
       <c r="AG363" s="4">
         <v>13</v>
       </c>
-      <c r="AH363" s="3" t="s">
-        <v>4911</v>
+      <c r="AH363" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54204,8 +54203,8 @@
       <c r="AG364" s="2">
         <v>13</v>
       </c>
-      <c r="AH364" s="1" t="s">
-        <v>4911</v>
+      <c r="AH364" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54308,8 +54307,8 @@
       <c r="AG365" s="4">
         <v>13</v>
       </c>
-      <c r="AH365" s="3" t="s">
-        <v>4911</v>
+      <c r="AH365" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54412,8 +54411,8 @@
       <c r="AG366" s="2">
         <v>13</v>
       </c>
-      <c r="AH366" s="1" t="s">
-        <v>4911</v>
+      <c r="AH366" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54516,8 +54515,8 @@
       <c r="AG367" s="4">
         <v>13</v>
       </c>
-      <c r="AH367" s="3" t="s">
-        <v>4911</v>
+      <c r="AH367" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54620,8 +54619,8 @@
       <c r="AG368" s="2">
         <v>13</v>
       </c>
-      <c r="AH368" s="1" t="s">
-        <v>4911</v>
+      <c r="AH368" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54724,8 +54723,8 @@
       <c r="AG369" s="4">
         <v>13</v>
       </c>
-      <c r="AH369" s="3" t="s">
-        <v>4911</v>
+      <c r="AH369" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54828,8 +54827,8 @@
       <c r="AG370" s="2">
         <v>13</v>
       </c>
-      <c r="AH370" s="1" t="s">
-        <v>4911</v>
+      <c r="AH370" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54932,8 +54931,8 @@
       <c r="AG371" s="4">
         <v>5</v>
       </c>
-      <c r="AH371" s="3" t="s">
-        <v>4911</v>
+      <c r="AH371" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55036,8 +55035,8 @@
       <c r="AG372" s="2">
         <v>13</v>
       </c>
-      <c r="AH372" s="1" t="s">
-        <v>4911</v>
+      <c r="AH372" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55140,8 +55139,8 @@
       <c r="AG373" s="4">
         <v>13</v>
       </c>
-      <c r="AH373" s="3" t="s">
-        <v>4911</v>
+      <c r="AH373" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55244,8 +55243,8 @@
       <c r="AG374" s="2">
         <v>13</v>
       </c>
-      <c r="AH374" s="1" t="s">
-        <v>4911</v>
+      <c r="AH374" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55348,8 +55347,8 @@
       <c r="AG375" s="4">
         <v>13</v>
       </c>
-      <c r="AH375" s="3" t="s">
-        <v>4911</v>
+      <c r="AH375" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55452,8 +55451,8 @@
       <c r="AG376" s="2">
         <v>13</v>
       </c>
-      <c r="AH376" s="1" t="s">
-        <v>4911</v>
+      <c r="AH376" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55556,8 +55555,8 @@
       <c r="AG377" s="4">
         <v>13</v>
       </c>
-      <c r="AH377" s="3" t="s">
-        <v>4911</v>
+      <c r="AH377" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55660,8 +55659,8 @@
       <c r="AG378" s="2">
         <v>13</v>
       </c>
-      <c r="AH378" s="1" t="s">
-        <v>4911</v>
+      <c r="AH378" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55764,8 +55763,8 @@
       <c r="AG379" s="4">
         <v>5</v>
       </c>
-      <c r="AH379" s="3" t="s">
-        <v>4911</v>
+      <c r="AH379" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55868,8 +55867,8 @@
       <c r="AG380" s="2">
         <v>13</v>
       </c>
-      <c r="AH380" s="1" t="s">
-        <v>4911</v>
+      <c r="AH380" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55972,8 +55971,8 @@
       <c r="AG381" s="4">
         <v>13</v>
       </c>
-      <c r="AH381" s="3" t="s">
-        <v>4911</v>
+      <c r="AH381" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56076,8 +56075,8 @@
       <c r="AG382" s="2">
         <v>13</v>
       </c>
-      <c r="AH382" s="1" t="s">
-        <v>4911</v>
+      <c r="AH382" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56180,8 +56179,8 @@
       <c r="AG383" s="4">
         <v>13</v>
       </c>
-      <c r="AH383" s="3" t="s">
-        <v>4911</v>
+      <c r="AH383" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56284,8 +56283,8 @@
       <c r="AG384" s="2">
         <v>13</v>
       </c>
-      <c r="AH384" s="1" t="s">
-        <v>4911</v>
+      <c r="AH384" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56338,8 +56337,8 @@
       <c r="AG385" s="4">
         <v>13</v>
       </c>
-      <c r="AH385" s="3" t="s">
-        <v>4911</v>
+      <c r="AH385" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56442,8 +56441,8 @@
       <c r="AG386" s="2">
         <v>13</v>
       </c>
-      <c r="AH386" s="1" t="s">
-        <v>4911</v>
+      <c r="AH386" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56546,8 +56545,8 @@
       <c r="AG387" s="4">
         <v>13</v>
       </c>
-      <c r="AH387" s="3" t="s">
-        <v>4911</v>
+      <c r="AH387" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56650,8 +56649,8 @@
       <c r="AG388" s="2">
         <v>13</v>
       </c>
-      <c r="AH388" s="1" t="s">
-        <v>4911</v>
+      <c r="AH388" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56754,8 +56753,8 @@
       <c r="AG389" s="4">
         <v>13</v>
       </c>
-      <c r="AH389" s="3" t="s">
-        <v>4911</v>
+      <c r="AH389" s="6">
+        <v>46240.381516203706</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56858,8 +56857,8 @@
       <c r="AG390" s="2">
         <v>13</v>
       </c>
-      <c r="AH390" s="1" t="s">
-        <v>4911</v>
+      <c r="AH390" s="5">
+        <v>46240.381516203706</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-08 08:02:19
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16609,7 +16609,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16713,7 +16713,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16817,7 +16817,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16921,7 +16921,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17025,7 +17025,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17129,7 +17129,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17233,7 +17233,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17337,7 +17337,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17441,7 +17441,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17545,7 +17545,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17649,7 +17649,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17753,7 +17753,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17857,7 +17857,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17961,7 +17961,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18065,7 +18065,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18169,7 +18169,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18273,7 +18273,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18377,7 +18377,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18481,7 +18481,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18585,7 +18585,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18689,7 +18689,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18793,7 +18793,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18897,7 +18897,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19001,7 +19001,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19105,7 +19105,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19209,7 +19209,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19313,7 +19313,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19417,7 +19417,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19521,7 +19521,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19625,7 +19625,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19729,7 +19729,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19833,7 +19833,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19937,7 +19937,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20041,7 +20041,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20145,7 +20145,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20249,7 +20249,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20353,7 +20353,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20457,7 +20457,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20561,7 +20561,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20665,7 +20665,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20769,7 +20769,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20873,7 +20873,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20977,7 +20977,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21081,7 +21081,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21185,7 +21185,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21289,7 +21289,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21393,7 +21393,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21497,7 +21497,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21601,7 +21601,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21705,7 +21705,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21809,7 +21809,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21913,7 +21913,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22017,7 +22017,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22121,7 +22121,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22225,7 +22225,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22329,7 +22329,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22433,7 +22433,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22537,7 +22537,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22641,7 +22641,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22745,7 +22745,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22849,7 +22849,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22953,7 +22953,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23057,7 +23057,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23161,7 +23161,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23265,7 +23265,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23369,7 +23369,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23473,7 +23473,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23577,7 +23577,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23681,7 +23681,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23785,7 +23785,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23889,7 +23889,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23993,7 +23993,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24097,7 +24097,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24201,7 +24201,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24305,7 +24305,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24409,7 +24409,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24513,7 +24513,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24617,7 +24617,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24721,7 +24721,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24825,7 +24825,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24929,7 +24929,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25033,7 +25033,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25137,7 +25137,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25241,7 +25241,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25345,7 +25345,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25449,7 +25449,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25553,7 +25553,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25657,7 +25657,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25761,7 +25761,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25865,7 +25865,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25969,7 +25969,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26073,7 +26073,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26177,7 +26177,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26281,7 +26281,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26385,7 +26385,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26489,7 +26489,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26593,7 +26593,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26697,7 +26697,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26801,7 +26801,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26905,7 +26905,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27009,7 +27009,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27113,7 +27113,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27217,7 +27217,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27321,7 +27321,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27425,7 +27425,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27529,7 +27529,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27633,7 +27633,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27737,7 +27737,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27841,7 +27841,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27945,7 +27945,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28049,7 +28049,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28153,7 +28153,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28257,7 +28257,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28361,7 +28361,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28465,7 +28465,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28569,7 +28569,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28673,7 +28673,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28777,7 +28777,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28881,7 +28881,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28985,7 +28985,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29089,7 +29089,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29193,7 +29193,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29297,7 +29297,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29401,7 +29401,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29505,7 +29505,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29609,7 +29609,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29713,7 +29713,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29817,7 +29817,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29921,7 +29921,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30025,7 +30025,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30129,7 +30129,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30233,7 +30233,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30337,7 +30337,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30441,7 +30441,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30545,7 +30545,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30649,7 +30649,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30753,7 +30753,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30857,7 +30857,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30961,7 +30961,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31065,7 +31065,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31169,7 +31169,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31273,7 +31273,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31377,7 +31377,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31481,7 +31481,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31585,7 +31585,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31689,7 +31689,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31793,7 +31793,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31897,7 +31897,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32001,7 +32001,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32105,7 +32105,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32209,7 +32209,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32313,7 +32313,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32417,7 +32417,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32521,7 +32521,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32625,7 +32625,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32729,7 +32729,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32833,7 +32833,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32937,7 +32937,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33041,7 +33041,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33145,7 +33145,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33249,7 +33249,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33353,7 +33353,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33457,7 +33457,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33561,7 +33561,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33665,7 +33665,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33769,7 +33769,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33873,7 +33873,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33977,7 +33977,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34081,7 +34081,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34185,7 +34185,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34289,7 +34289,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34393,7 +34393,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34497,7 +34497,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34601,7 +34601,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34705,7 +34705,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34809,7 +34809,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34913,7 +34913,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35017,7 +35017,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35121,7 +35121,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35225,7 +35225,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35329,7 +35329,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35433,7 +35433,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35537,7 +35537,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35641,7 +35641,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35745,7 +35745,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35849,7 +35849,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35953,7 +35953,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36057,7 +36057,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36161,7 +36161,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36265,7 +36265,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36369,7 +36369,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36473,7 +36473,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36577,7 +36577,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36681,7 +36681,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36785,7 +36785,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36889,7 +36889,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36993,7 +36993,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37097,7 +37097,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37201,7 +37201,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37305,7 +37305,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37409,7 +37409,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37513,7 +37513,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37617,7 +37617,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37721,7 +37721,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37825,7 +37825,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37929,7 +37929,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38033,7 +38033,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38137,7 +38137,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38241,7 +38241,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38345,7 +38345,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38449,7 +38449,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38553,7 +38553,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38657,7 +38657,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38761,7 +38761,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38865,7 +38865,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38969,7 +38969,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39073,7 +39073,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39177,7 +39177,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39281,7 +39281,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39385,7 +39385,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39489,7 +39489,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39593,7 +39593,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39697,7 +39697,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39801,7 +39801,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39905,7 +39905,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40009,7 +40009,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40113,7 +40113,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40217,7 +40217,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40321,7 +40321,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40425,7 +40425,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40529,7 +40529,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40633,7 +40633,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40737,7 +40737,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40841,7 +40841,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40945,7 +40945,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41049,7 +41049,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41153,7 +41153,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41257,7 +41257,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41361,7 +41361,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41465,7 +41465,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41569,7 +41569,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41673,7 +41673,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41777,7 +41777,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41881,7 +41881,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41985,7 +41985,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42089,7 +42089,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42193,7 +42193,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42297,7 +42297,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42401,7 +42401,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42505,7 +42505,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42609,7 +42609,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42713,7 +42713,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42817,7 +42817,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42921,7 +42921,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43025,7 +43025,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43129,7 +43129,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43233,7 +43233,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43337,7 +43337,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43441,7 +43441,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43545,7 +43545,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43649,7 +43649,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43753,7 +43753,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43857,7 +43857,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43961,7 +43961,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44065,7 +44065,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44169,7 +44169,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44273,7 +44273,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44377,7 +44377,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44481,7 +44481,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44585,7 +44585,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44689,7 +44689,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44793,7 +44793,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44897,7 +44897,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45001,7 +45001,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45105,7 +45105,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45209,7 +45209,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45313,7 +45313,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45417,7 +45417,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45521,7 +45521,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45625,7 +45625,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45729,7 +45729,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45833,7 +45833,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45937,7 +45937,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46041,7 +46041,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46145,7 +46145,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46249,7 +46249,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46353,7 +46353,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46457,7 +46457,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46561,7 +46561,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46665,7 +46665,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46769,7 +46769,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46873,7 +46873,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46977,7 +46977,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47081,7 +47081,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47185,7 +47185,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47289,7 +47289,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47393,7 +47393,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47497,7 +47497,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47601,7 +47601,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47705,7 +47705,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47809,7 +47809,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47913,7 +47913,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48017,7 +48017,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48121,7 +48121,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48225,7 +48225,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48329,7 +48329,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48433,7 +48433,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48537,7 +48537,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48641,7 +48641,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48745,7 +48745,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48849,7 +48849,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48953,7 +48953,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49057,7 +49057,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49161,7 +49161,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49265,7 +49265,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49369,7 +49369,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49473,7 +49473,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49577,7 +49577,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49681,7 +49681,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49785,7 +49785,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49889,7 +49889,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49993,7 +49993,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50097,7 +50097,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50201,7 +50201,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50305,7 +50305,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50409,7 +50409,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50513,7 +50513,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50617,7 +50617,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50721,7 +50721,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50825,7 +50825,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50929,7 +50929,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51033,7 +51033,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51137,7 +51137,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51241,7 +51241,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51345,7 +51345,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51449,7 +51449,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51553,7 +51553,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51657,7 +51657,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51761,7 +51761,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51865,7 +51865,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51969,7 +51969,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52073,7 +52073,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52177,7 +52177,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52281,7 +52281,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52385,7 +52385,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52489,7 +52489,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52593,7 +52593,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52697,7 +52697,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52801,7 +52801,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52905,7 +52905,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53009,7 +53009,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53113,7 +53113,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53217,7 +53217,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53321,7 +53321,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53425,7 +53425,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53529,7 +53529,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53583,7 +53583,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53687,7 +53687,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53791,7 +53791,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53895,7 +53895,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -53999,7 +53999,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54103,7 +54103,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54207,7 +54207,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54311,7 +54311,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54415,7 +54415,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54519,7 +54519,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54623,7 +54623,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54727,7 +54727,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54831,7 +54831,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54935,7 +54935,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55039,7 +55039,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55143,7 +55143,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55247,7 +55247,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55351,7 +55351,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55455,7 +55455,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55559,7 +55559,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55663,7 +55663,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55767,7 +55767,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55871,7 +55871,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55975,7 +55975,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56079,7 +56079,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56183,7 +56183,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56287,7 +56287,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56341,7 +56341,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56445,7 +56445,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56549,7 +56549,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56653,7 +56653,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56757,7 +56757,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56861,7 +56861,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46241.491087962961</v>
+        <v>46242.33494212963</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-09 08:06:40
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16609,7 +16609,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16713,7 +16713,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16817,7 +16817,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16921,7 +16921,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17025,7 +17025,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17129,7 +17129,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17233,7 +17233,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17337,7 +17337,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17441,7 +17441,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17545,7 +17545,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17649,7 +17649,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17753,7 +17753,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17857,7 +17857,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17961,7 +17961,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18065,7 +18065,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18169,7 +18169,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18273,7 +18273,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18377,7 +18377,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18481,7 +18481,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18585,7 +18585,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18689,7 +18689,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18793,7 +18793,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18897,7 +18897,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19001,7 +19001,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19105,7 +19105,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19209,7 +19209,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19313,7 +19313,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19417,7 +19417,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19521,7 +19521,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19625,7 +19625,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19729,7 +19729,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19833,7 +19833,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19937,7 +19937,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20041,7 +20041,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20145,7 +20145,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20249,7 +20249,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20353,7 +20353,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20457,7 +20457,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20561,7 +20561,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20665,7 +20665,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20769,7 +20769,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20873,7 +20873,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20977,7 +20977,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21081,7 +21081,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21185,7 +21185,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21289,7 +21289,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21393,7 +21393,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21497,7 +21497,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21601,7 +21601,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21705,7 +21705,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21809,7 +21809,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21913,7 +21913,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22017,7 +22017,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22121,7 +22121,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22225,7 +22225,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22329,7 +22329,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22433,7 +22433,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22537,7 +22537,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22641,7 +22641,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22745,7 +22745,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22849,7 +22849,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22953,7 +22953,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23057,7 +23057,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23161,7 +23161,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23265,7 +23265,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23369,7 +23369,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23473,7 +23473,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23577,7 +23577,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23681,7 +23681,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23785,7 +23785,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23889,7 +23889,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23993,7 +23993,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24097,7 +24097,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24201,7 +24201,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24305,7 +24305,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24409,7 +24409,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24513,7 +24513,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24617,7 +24617,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24721,7 +24721,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24825,7 +24825,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24929,7 +24929,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25033,7 +25033,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25137,7 +25137,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25241,7 +25241,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25345,7 +25345,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25449,7 +25449,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25553,7 +25553,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25657,7 +25657,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25761,7 +25761,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25865,7 +25865,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25969,7 +25969,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26073,7 +26073,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26177,7 +26177,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26281,7 +26281,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26385,7 +26385,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26489,7 +26489,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26593,7 +26593,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26697,7 +26697,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26801,7 +26801,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26905,7 +26905,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27009,7 +27009,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27113,7 +27113,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27217,7 +27217,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27321,7 +27321,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27425,7 +27425,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27529,7 +27529,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27633,7 +27633,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27737,7 +27737,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27841,7 +27841,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27945,7 +27945,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28049,7 +28049,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28153,7 +28153,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28257,7 +28257,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28361,7 +28361,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28465,7 +28465,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28569,7 +28569,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28673,7 +28673,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28777,7 +28777,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28881,7 +28881,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28985,7 +28985,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29089,7 +29089,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29193,7 +29193,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29297,7 +29297,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29401,7 +29401,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29505,7 +29505,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29609,7 +29609,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29713,7 +29713,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29817,7 +29817,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29921,7 +29921,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30025,7 +30025,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30129,7 +30129,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30233,7 +30233,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30337,7 +30337,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30441,7 +30441,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30545,7 +30545,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30649,7 +30649,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30753,7 +30753,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30857,7 +30857,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30961,7 +30961,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31065,7 +31065,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31169,7 +31169,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31273,7 +31273,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31377,7 +31377,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31481,7 +31481,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31585,7 +31585,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31689,7 +31689,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31793,7 +31793,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31897,7 +31897,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32001,7 +32001,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32105,7 +32105,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32209,7 +32209,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32313,7 +32313,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32417,7 +32417,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32521,7 +32521,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32625,7 +32625,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32729,7 +32729,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32833,7 +32833,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32937,7 +32937,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33041,7 +33041,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33145,7 +33145,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33249,7 +33249,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33353,7 +33353,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33457,7 +33457,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33561,7 +33561,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33665,7 +33665,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33769,7 +33769,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33873,7 +33873,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33977,7 +33977,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34081,7 +34081,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34185,7 +34185,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34289,7 +34289,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34393,7 +34393,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34497,7 +34497,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34601,7 +34601,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34705,7 +34705,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34809,7 +34809,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34913,7 +34913,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35017,7 +35017,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35121,7 +35121,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35225,7 +35225,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35329,7 +35329,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35433,7 +35433,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35537,7 +35537,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35641,7 +35641,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35745,7 +35745,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35849,7 +35849,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35953,7 +35953,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36057,7 +36057,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36161,7 +36161,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36265,7 +36265,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36369,7 +36369,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36473,7 +36473,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36577,7 +36577,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36681,7 +36681,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36785,7 +36785,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36889,7 +36889,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36993,7 +36993,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37097,7 +37097,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37201,7 +37201,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37305,7 +37305,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37409,7 +37409,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37513,7 +37513,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37617,7 +37617,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37721,7 +37721,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37825,7 +37825,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37929,7 +37929,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38033,7 +38033,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38137,7 +38137,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38241,7 +38241,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38345,7 +38345,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38449,7 +38449,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38553,7 +38553,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38657,7 +38657,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38761,7 +38761,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38865,7 +38865,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38969,7 +38969,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39073,7 +39073,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39177,7 +39177,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39281,7 +39281,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39385,7 +39385,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39489,7 +39489,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39593,7 +39593,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39697,7 +39697,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39801,7 +39801,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39905,7 +39905,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40009,7 +40009,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40113,7 +40113,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40217,7 +40217,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40321,7 +40321,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40425,7 +40425,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40529,7 +40529,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40633,7 +40633,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40737,7 +40737,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40841,7 +40841,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40945,7 +40945,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41049,7 +41049,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41153,7 +41153,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41257,7 +41257,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41361,7 +41361,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41465,7 +41465,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41569,7 +41569,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41673,7 +41673,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41777,7 +41777,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41881,7 +41881,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41985,7 +41985,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42089,7 +42089,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42193,7 +42193,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42297,7 +42297,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42401,7 +42401,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42505,7 +42505,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42609,7 +42609,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42713,7 +42713,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42817,7 +42817,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42921,7 +42921,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43025,7 +43025,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43129,7 +43129,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43233,7 +43233,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43337,7 +43337,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43441,7 +43441,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43545,7 +43545,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43649,7 +43649,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43753,7 +43753,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43857,7 +43857,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43961,7 +43961,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44065,7 +44065,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44169,7 +44169,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44273,7 +44273,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44377,7 +44377,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44481,7 +44481,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44585,7 +44585,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44689,7 +44689,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44793,7 +44793,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44897,7 +44897,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45001,7 +45001,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45105,7 +45105,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45209,7 +45209,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45313,7 +45313,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45417,7 +45417,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45521,7 +45521,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45625,7 +45625,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45729,7 +45729,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45833,7 +45833,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45937,7 +45937,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46041,7 +46041,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46145,7 +46145,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46249,7 +46249,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46353,7 +46353,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46457,7 +46457,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46561,7 +46561,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46665,7 +46665,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46769,7 +46769,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46873,7 +46873,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46977,7 +46977,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47081,7 +47081,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47185,7 +47185,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47289,7 +47289,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47393,7 +47393,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47497,7 +47497,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47601,7 +47601,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47705,7 +47705,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47809,7 +47809,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47913,7 +47913,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48017,7 +48017,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48121,7 +48121,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48225,7 +48225,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48329,7 +48329,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48433,7 +48433,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48537,7 +48537,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48641,7 +48641,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48745,7 +48745,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48849,7 +48849,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48953,7 +48953,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49057,7 +49057,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49161,7 +49161,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49265,7 +49265,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49369,7 +49369,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49473,7 +49473,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49577,7 +49577,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49681,7 +49681,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49785,7 +49785,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49889,7 +49889,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49993,7 +49993,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50097,7 +50097,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50201,7 +50201,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50305,7 +50305,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50409,7 +50409,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50513,7 +50513,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50617,7 +50617,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50721,7 +50721,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50825,7 +50825,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50929,7 +50929,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51033,7 +51033,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51137,7 +51137,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51241,7 +51241,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51345,7 +51345,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51449,7 +51449,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51553,7 +51553,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51657,7 +51657,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51761,7 +51761,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51865,7 +51865,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51969,7 +51969,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52073,7 +52073,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52177,7 +52177,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52281,7 +52281,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52385,7 +52385,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52489,7 +52489,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52593,7 +52593,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52697,7 +52697,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52801,7 +52801,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52905,7 +52905,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53009,7 +53009,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53113,7 +53113,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53217,7 +53217,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53321,7 +53321,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53425,7 +53425,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53529,7 +53529,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53583,7 +53583,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53687,7 +53687,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53791,7 +53791,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53895,7 +53895,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -53999,7 +53999,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54103,7 +54103,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54207,7 +54207,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54311,7 +54311,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54415,7 +54415,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54519,7 +54519,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54623,7 +54623,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54727,7 +54727,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54831,7 +54831,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54935,7 +54935,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55039,7 +55039,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55143,7 +55143,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55247,7 +55247,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55351,7 +55351,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55455,7 +55455,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55559,7 +55559,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55663,7 +55663,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55767,7 +55767,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55871,7 +55871,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55975,7 +55975,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56079,7 +56079,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56183,7 +56183,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56287,7 +56287,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56341,7 +56341,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56445,7 +56445,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56549,7 +56549,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56653,7 +56653,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56757,7 +56757,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56861,7 +56861,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46242.33494212963</v>
+        <v>46243.337962962964</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-10 08:02:50
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16609,7 +16609,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16713,7 +16713,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16817,7 +16817,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16921,7 +16921,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17025,7 +17025,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17129,7 +17129,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17233,7 +17233,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17337,7 +17337,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17441,7 +17441,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17545,7 +17545,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17649,7 +17649,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17753,7 +17753,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17857,7 +17857,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17961,7 +17961,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18065,7 +18065,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18169,7 +18169,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18273,7 +18273,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18377,7 +18377,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18481,7 +18481,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18585,7 +18585,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18689,7 +18689,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18793,7 +18793,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18897,7 +18897,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19001,7 +19001,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19105,7 +19105,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19209,7 +19209,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19313,7 +19313,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19417,7 +19417,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19521,7 +19521,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19625,7 +19625,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19729,7 +19729,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19833,7 +19833,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19937,7 +19937,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20041,7 +20041,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20145,7 +20145,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20249,7 +20249,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20353,7 +20353,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20457,7 +20457,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20561,7 +20561,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20665,7 +20665,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20769,7 +20769,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20873,7 +20873,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20977,7 +20977,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21081,7 +21081,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21185,7 +21185,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21289,7 +21289,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21393,7 +21393,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21497,7 +21497,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21601,7 +21601,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21705,7 +21705,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21809,7 +21809,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21913,7 +21913,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22017,7 +22017,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22121,7 +22121,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22225,7 +22225,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22329,7 +22329,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22433,7 +22433,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22537,7 +22537,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22641,7 +22641,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22745,7 +22745,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22849,7 +22849,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22953,7 +22953,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23057,7 +23057,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23161,7 +23161,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23265,7 +23265,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23369,7 +23369,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23473,7 +23473,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23577,7 +23577,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23681,7 +23681,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23785,7 +23785,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23889,7 +23889,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23993,7 +23993,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24097,7 +24097,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24201,7 +24201,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24305,7 +24305,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24409,7 +24409,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24513,7 +24513,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24617,7 +24617,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24721,7 +24721,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24825,7 +24825,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24929,7 +24929,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25033,7 +25033,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25137,7 +25137,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25241,7 +25241,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25345,7 +25345,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25449,7 +25449,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25553,7 +25553,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25657,7 +25657,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25761,7 +25761,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25865,7 +25865,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25969,7 +25969,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26073,7 +26073,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26177,7 +26177,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26281,7 +26281,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26385,7 +26385,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26489,7 +26489,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26593,7 +26593,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26697,7 +26697,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26801,7 +26801,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26905,7 +26905,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27009,7 +27009,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27113,7 +27113,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27217,7 +27217,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27321,7 +27321,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27425,7 +27425,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27529,7 +27529,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27633,7 +27633,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27737,7 +27737,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27841,7 +27841,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27945,7 +27945,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28049,7 +28049,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28153,7 +28153,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28257,7 +28257,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28361,7 +28361,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28465,7 +28465,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28569,7 +28569,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28673,7 +28673,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28777,7 +28777,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28881,7 +28881,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28985,7 +28985,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29089,7 +29089,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29193,7 +29193,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29297,7 +29297,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29401,7 +29401,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29505,7 +29505,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29609,7 +29609,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29713,7 +29713,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29817,7 +29817,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29921,7 +29921,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30025,7 +30025,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30129,7 +30129,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30233,7 +30233,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30337,7 +30337,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30441,7 +30441,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30545,7 +30545,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30649,7 +30649,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30753,7 +30753,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30857,7 +30857,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30961,7 +30961,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31065,7 +31065,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31169,7 +31169,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31273,7 +31273,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31377,7 +31377,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31481,7 +31481,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31585,7 +31585,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31689,7 +31689,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31793,7 +31793,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31897,7 +31897,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32001,7 +32001,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32105,7 +32105,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32209,7 +32209,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32313,7 +32313,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32417,7 +32417,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32521,7 +32521,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32625,7 +32625,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32729,7 +32729,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32833,7 +32833,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32937,7 +32937,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33041,7 +33041,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33145,7 +33145,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33249,7 +33249,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33353,7 +33353,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33457,7 +33457,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33561,7 +33561,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33665,7 +33665,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33769,7 +33769,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33873,7 +33873,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33977,7 +33977,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34081,7 +34081,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34185,7 +34185,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34289,7 +34289,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34393,7 +34393,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34497,7 +34497,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34601,7 +34601,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34705,7 +34705,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34809,7 +34809,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34913,7 +34913,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35017,7 +35017,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35121,7 +35121,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35225,7 +35225,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35329,7 +35329,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35433,7 +35433,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35537,7 +35537,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35641,7 +35641,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35745,7 +35745,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35849,7 +35849,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35953,7 +35953,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36057,7 +36057,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36161,7 +36161,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36265,7 +36265,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36369,7 +36369,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36473,7 +36473,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36577,7 +36577,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36681,7 +36681,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36785,7 +36785,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36889,7 +36889,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36993,7 +36993,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37097,7 +37097,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37201,7 +37201,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37305,7 +37305,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37409,7 +37409,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37513,7 +37513,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37617,7 +37617,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37721,7 +37721,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37825,7 +37825,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37929,7 +37929,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38033,7 +38033,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38137,7 +38137,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38241,7 +38241,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38345,7 +38345,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38449,7 +38449,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38553,7 +38553,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38657,7 +38657,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38761,7 +38761,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38865,7 +38865,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38969,7 +38969,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39073,7 +39073,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39177,7 +39177,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39281,7 +39281,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39385,7 +39385,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39489,7 +39489,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39593,7 +39593,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39697,7 +39697,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39801,7 +39801,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39905,7 +39905,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40009,7 +40009,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40113,7 +40113,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40217,7 +40217,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40321,7 +40321,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40425,7 +40425,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40529,7 +40529,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40633,7 +40633,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40737,7 +40737,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40841,7 +40841,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40945,7 +40945,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41049,7 +41049,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41153,7 +41153,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41257,7 +41257,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41361,7 +41361,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41465,7 +41465,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41569,7 +41569,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41673,7 +41673,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41777,7 +41777,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41881,7 +41881,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41985,7 +41985,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42089,7 +42089,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42193,7 +42193,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42297,7 +42297,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42401,7 +42401,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42505,7 +42505,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42609,7 +42609,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42713,7 +42713,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42817,7 +42817,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42921,7 +42921,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43025,7 +43025,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43129,7 +43129,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43233,7 +43233,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43337,7 +43337,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43441,7 +43441,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43545,7 +43545,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43649,7 +43649,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43753,7 +43753,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43857,7 +43857,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43961,7 +43961,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44065,7 +44065,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44169,7 +44169,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44273,7 +44273,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44377,7 +44377,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44481,7 +44481,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44585,7 +44585,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44689,7 +44689,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44793,7 +44793,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44897,7 +44897,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45001,7 +45001,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45105,7 +45105,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45209,7 +45209,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45313,7 +45313,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45417,7 +45417,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45521,7 +45521,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45625,7 +45625,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45729,7 +45729,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45833,7 +45833,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45937,7 +45937,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46041,7 +46041,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46145,7 +46145,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46249,7 +46249,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46353,7 +46353,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46457,7 +46457,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46561,7 +46561,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46665,7 +46665,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46769,7 +46769,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46873,7 +46873,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46977,7 +46977,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47081,7 +47081,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47185,7 +47185,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47289,7 +47289,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47393,7 +47393,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47497,7 +47497,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47601,7 +47601,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47705,7 +47705,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47809,7 +47809,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47913,7 +47913,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48017,7 +48017,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48121,7 +48121,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48225,7 +48225,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48329,7 +48329,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48433,7 +48433,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48537,7 +48537,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48548,7 +48548,7 @@
         <v>3956</v>
       </c>
       <c r="C310" s="2">
-        <v>15536579</v>
+        <v>13897638</v>
       </c>
       <c r="D310" s="1" t="s">
         <v>3391</v>
@@ -48641,7 +48641,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48745,7 +48745,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48849,7 +48849,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48953,7 +48953,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49057,7 +49057,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49161,7 +49161,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49265,7 +49265,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49369,7 +49369,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49473,7 +49473,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49484,7 +49484,7 @@
         <v>4089</v>
       </c>
       <c r="C319" s="4">
-        <v>9170712</v>
+        <v>15345601</v>
       </c>
       <c r="D319" s="3" t="s">
         <v>4090</v>
@@ -49577,7 +49577,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49681,7 +49681,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49785,7 +49785,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49889,7 +49889,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49993,7 +49993,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50097,7 +50097,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50201,7 +50201,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50305,7 +50305,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50409,7 +50409,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50513,7 +50513,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50617,7 +50617,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50721,7 +50721,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50825,7 +50825,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50929,7 +50929,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51033,7 +51033,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51137,7 +51137,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51241,7 +51241,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51345,7 +51345,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51449,7 +51449,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51553,7 +51553,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51657,7 +51657,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51761,7 +51761,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51865,7 +51865,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51969,7 +51969,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52073,7 +52073,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52177,7 +52177,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52281,7 +52281,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52385,7 +52385,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52489,7 +52489,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52593,7 +52593,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52697,7 +52697,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52801,7 +52801,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52905,7 +52905,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53009,7 +53009,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53113,7 +53113,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53217,7 +53217,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53321,7 +53321,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53425,7 +53425,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53529,7 +53529,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53583,7 +53583,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53687,7 +53687,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53791,7 +53791,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53895,7 +53895,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -53999,7 +53999,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54103,7 +54103,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54207,7 +54207,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54311,7 +54311,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54415,7 +54415,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54519,7 +54519,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54623,7 +54623,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54727,7 +54727,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54831,7 +54831,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54935,7 +54935,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55039,7 +55039,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55143,7 +55143,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55247,7 +55247,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55351,7 +55351,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55455,7 +55455,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55559,7 +55559,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55663,7 +55663,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55767,7 +55767,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55871,7 +55871,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55975,7 +55975,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56079,7 +56079,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56183,7 +56183,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56287,7 +56287,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56341,7 +56341,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56445,7 +56445,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56549,7 +56549,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56653,7 +56653,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56757,7 +56757,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56861,7 +56861,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46243.337962962964</v>
+        <v>46244.335300925923</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-11 10:14:31
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16618,7 +16618,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16722,7 +16722,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16826,7 +16826,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16930,7 +16930,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17034,7 +17034,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17138,7 +17138,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17242,7 +17242,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17346,7 +17346,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17450,7 +17450,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17554,7 +17554,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17658,7 +17658,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17762,7 +17762,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17866,7 +17866,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17970,7 +17970,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18074,7 +18074,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18178,7 +18178,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18282,7 +18282,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18386,7 +18386,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18490,7 +18490,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18594,7 +18594,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18698,7 +18698,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18802,7 +18802,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18906,7 +18906,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19010,7 +19010,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19114,7 +19114,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19218,7 +19218,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19322,7 +19322,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19426,7 +19426,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19530,7 +19530,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19634,7 +19634,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19738,7 +19738,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19842,7 +19842,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19946,7 +19946,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20050,7 +20050,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20154,7 +20154,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20258,7 +20258,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20362,7 +20362,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20466,7 +20466,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20570,7 +20570,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20674,7 +20674,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20778,7 +20778,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20882,7 +20882,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20986,7 +20986,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21090,7 +21090,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21194,7 +21194,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21298,7 +21298,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21402,7 +21402,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21506,7 +21506,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21610,7 +21610,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21714,7 +21714,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21818,7 +21818,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21922,7 +21922,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22026,7 +22026,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22130,7 +22130,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22234,7 +22234,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22338,7 +22338,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22442,7 +22442,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22546,7 +22546,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22650,7 +22650,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22754,7 +22754,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22858,7 +22858,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22962,7 +22962,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23066,7 +23066,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23170,7 +23170,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23274,7 +23274,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23378,7 +23378,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23482,7 +23482,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23586,7 +23586,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23690,7 +23690,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23794,7 +23794,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23898,7 +23898,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -24002,7 +24002,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24106,7 +24106,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24210,7 +24210,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24221,7 +24221,7 @@
         <v>1157</v>
       </c>
       <c r="C76" s="2">
-        <v>26680705</v>
+        <v>26721632</v>
       </c>
       <c r="D76" s="1" t="s">
         <v>1158</v>
@@ -24314,7 +24314,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24418,7 +24418,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24522,7 +24522,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24626,7 +24626,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24730,7 +24730,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24834,7 +24834,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24938,7 +24938,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25042,7 +25042,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25146,7 +25146,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25250,7 +25250,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25354,7 +25354,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25458,7 +25458,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25562,7 +25562,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25666,7 +25666,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25770,7 +25770,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25874,7 +25874,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25978,7 +25978,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26082,7 +26082,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26186,7 +26186,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26290,7 +26290,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26394,7 +26394,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26498,7 +26498,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26602,7 +26602,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26706,7 +26706,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26810,7 +26810,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26914,7 +26914,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27018,7 +27018,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27122,7 +27122,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27226,7 +27226,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27330,7 +27330,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27434,7 +27434,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27538,7 +27538,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27642,7 +27642,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27746,7 +27746,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27850,7 +27850,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27954,7 +27954,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28058,7 +28058,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28162,7 +28162,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28266,7 +28266,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28370,7 +28370,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28474,7 +28474,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28578,7 +28578,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28682,7 +28682,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28786,7 +28786,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28890,7 +28890,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28994,7 +28994,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29098,7 +29098,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29202,7 +29202,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29306,7 +29306,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29410,7 +29410,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29514,7 +29514,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29618,7 +29618,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29722,7 +29722,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29826,7 +29826,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29930,7 +29930,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30034,7 +30034,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30138,7 +30138,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30242,7 +30242,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30346,7 +30346,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30450,7 +30450,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30554,7 +30554,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30658,7 +30658,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30762,7 +30762,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30866,7 +30866,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30970,7 +30970,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31074,7 +31074,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31178,7 +31178,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31282,7 +31282,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31386,7 +31386,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31490,7 +31490,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31594,7 +31594,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31698,7 +31698,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31802,7 +31802,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31906,7 +31906,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32010,7 +32010,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32114,7 +32114,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32218,7 +32218,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32322,7 +32322,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32426,7 +32426,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32530,7 +32530,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32634,7 +32634,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32738,7 +32738,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32842,7 +32842,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32946,7 +32946,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33050,7 +33050,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33154,7 +33154,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33258,7 +33258,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33362,7 +33362,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33466,7 +33466,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33570,7 +33570,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33674,7 +33674,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33778,7 +33778,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33882,7 +33882,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33986,7 +33986,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34090,7 +34090,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34194,7 +34194,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34298,7 +34298,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34402,7 +34402,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34506,7 +34506,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34610,7 +34610,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34714,7 +34714,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34818,7 +34818,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34922,7 +34922,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35026,7 +35026,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35130,7 +35130,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35234,7 +35234,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35338,7 +35338,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35442,7 +35442,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35546,7 +35546,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35650,7 +35650,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35754,7 +35754,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35858,7 +35858,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35962,7 +35962,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36066,7 +36066,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36170,7 +36170,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36274,7 +36274,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36378,7 +36378,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36482,7 +36482,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36586,7 +36586,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36690,7 +36690,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36794,7 +36794,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36898,7 +36898,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -37002,7 +37002,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37106,7 +37106,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37210,7 +37210,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37314,7 +37314,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37418,7 +37418,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37522,7 +37522,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37626,7 +37626,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37730,7 +37730,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37834,7 +37834,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37938,7 +37938,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38042,7 +38042,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38146,7 +38146,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38250,7 +38250,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38354,7 +38354,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38458,7 +38458,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38562,7 +38562,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38666,7 +38666,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38770,7 +38770,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38874,7 +38874,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38978,7 +38978,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39082,7 +39082,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39186,7 +39186,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39290,7 +39290,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39394,7 +39394,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39498,7 +39498,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39602,7 +39602,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39706,7 +39706,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39810,7 +39810,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39914,7 +39914,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40018,7 +40018,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40122,7 +40122,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40226,7 +40226,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40330,7 +40330,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40434,7 +40434,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40538,7 +40538,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40642,7 +40642,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40746,7 +40746,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40850,7 +40850,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40954,7 +40954,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41058,7 +41058,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41162,7 +41162,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41266,7 +41266,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41370,7 +41370,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41474,7 +41474,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41578,7 +41578,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41682,7 +41682,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41786,7 +41786,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41890,7 +41890,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41994,7 +41994,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42098,7 +42098,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42202,7 +42202,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42306,7 +42306,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42410,7 +42410,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42514,7 +42514,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42618,7 +42618,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42722,7 +42722,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42826,7 +42826,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42930,7 +42930,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43034,7 +43034,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43138,7 +43138,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43242,7 +43242,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43346,7 +43346,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43450,7 +43450,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43554,7 +43554,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43658,7 +43658,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43762,7 +43762,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43866,7 +43866,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43970,7 +43970,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44074,7 +44074,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44178,7 +44178,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44282,7 +44282,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44386,7 +44386,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44490,7 +44490,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44594,7 +44594,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44698,7 +44698,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44802,7 +44802,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44906,7 +44906,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45010,7 +45010,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45114,7 +45114,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45218,7 +45218,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45322,7 +45322,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45426,7 +45426,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45530,7 +45530,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45634,7 +45634,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45738,7 +45738,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45842,7 +45842,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45946,7 +45946,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46050,7 +46050,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46154,7 +46154,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46258,7 +46258,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46362,7 +46362,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46466,7 +46466,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46570,7 +46570,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46674,7 +46674,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46778,7 +46778,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46882,7 +46882,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46986,7 +46986,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47090,7 +47090,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47194,7 +47194,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47298,7 +47298,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47402,7 +47402,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47506,7 +47506,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47610,7 +47610,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47714,7 +47714,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47818,7 +47818,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47922,7 +47922,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48026,7 +48026,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48130,7 +48130,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48234,7 +48234,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48338,7 +48338,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48442,7 +48442,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48546,7 +48546,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48650,7 +48650,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48754,7 +48754,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48858,7 +48858,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48962,7 +48962,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49066,7 +49066,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49170,7 +49170,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49274,7 +49274,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49378,7 +49378,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49482,7 +49482,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49586,7 +49586,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49690,7 +49690,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49794,7 +49794,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49898,7 +49898,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -50002,7 +50002,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50106,7 +50106,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50210,7 +50210,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50314,7 +50314,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50418,7 +50418,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50522,7 +50522,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50626,7 +50626,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50730,7 +50730,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50834,7 +50834,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50938,7 +50938,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51042,7 +51042,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51146,7 +51146,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51250,7 +51250,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51354,7 +51354,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51458,7 +51458,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51562,7 +51562,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51666,7 +51666,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51770,7 +51770,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51874,7 +51874,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51978,7 +51978,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52082,7 +52082,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52186,7 +52186,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52290,7 +52290,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52394,7 +52394,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52498,7 +52498,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52602,7 +52602,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52706,7 +52706,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52810,7 +52810,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52914,7 +52914,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53018,7 +53018,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53122,7 +53122,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53226,7 +53226,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53330,7 +53330,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53434,7 +53434,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53538,7 +53538,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53592,7 +53592,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53696,7 +53696,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53800,7 +53800,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53904,7 +53904,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -54008,7 +54008,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54112,7 +54112,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54216,7 +54216,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54320,7 +54320,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54424,7 +54424,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54528,7 +54528,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54632,7 +54632,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54736,7 +54736,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54840,7 +54840,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54944,7 +54944,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55048,7 +55048,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55152,7 +55152,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55256,7 +55256,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55360,7 +55360,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55464,7 +55464,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55475,7 +55475,7 @@
         <v>4747</v>
       </c>
       <c r="C377" s="4">
-        <v>25952636</v>
+        <v>13957353</v>
       </c>
       <c r="D377" s="3" t="s">
         <v>4748</v>
@@ -55568,7 +55568,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55672,7 +55672,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55776,7 +55776,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55880,7 +55880,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55984,7 +55984,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56088,7 +56088,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56192,7 +56192,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56296,7 +56296,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56350,7 +56350,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56454,7 +56454,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56558,7 +56558,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56662,7 +56662,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56766,7 +56766,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56870,7 +56870,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46245.338877314818</v>
+        <v>46245.426747685182</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-11 12:31:59
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16618,7 +16618,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16722,7 +16722,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16826,7 +16826,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16930,7 +16930,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17034,7 +17034,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17138,7 +17138,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17242,7 +17242,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17346,7 +17346,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17450,7 +17450,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17554,7 +17554,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17658,7 +17658,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17762,7 +17762,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17866,7 +17866,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17970,7 +17970,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18074,7 +18074,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18178,7 +18178,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18282,7 +18282,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18386,7 +18386,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18490,7 +18490,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18594,7 +18594,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18698,7 +18698,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18802,7 +18802,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18906,7 +18906,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19010,7 +19010,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19114,7 +19114,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19218,7 +19218,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19322,7 +19322,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19426,7 +19426,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19530,7 +19530,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19634,7 +19634,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19738,7 +19738,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19842,7 +19842,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19946,7 +19946,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20050,7 +20050,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20154,7 +20154,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20258,7 +20258,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20362,7 +20362,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20466,7 +20466,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20570,7 +20570,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20674,7 +20674,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20778,7 +20778,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20882,7 +20882,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20986,7 +20986,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21090,7 +21090,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21194,7 +21194,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21298,7 +21298,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21402,7 +21402,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21506,7 +21506,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21610,7 +21610,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21714,7 +21714,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21818,7 +21818,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21922,7 +21922,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22026,7 +22026,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22130,7 +22130,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22234,7 +22234,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22338,7 +22338,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22442,7 +22442,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22546,7 +22546,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22650,7 +22650,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22754,7 +22754,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22858,7 +22858,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22962,7 +22962,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23066,7 +23066,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23170,7 +23170,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23274,7 +23274,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23378,7 +23378,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23482,7 +23482,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23586,7 +23586,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23690,7 +23690,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23794,7 +23794,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23898,7 +23898,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -24002,7 +24002,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24106,7 +24106,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24210,7 +24210,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24314,7 +24314,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24418,7 +24418,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24522,7 +24522,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24626,7 +24626,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24730,7 +24730,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24834,7 +24834,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24938,7 +24938,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25042,7 +25042,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25146,7 +25146,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25250,7 +25250,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25354,7 +25354,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25458,7 +25458,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25562,7 +25562,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25666,7 +25666,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25770,7 +25770,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25874,7 +25874,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25978,7 +25978,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26082,7 +26082,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26186,7 +26186,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26290,7 +26290,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26394,7 +26394,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26498,7 +26498,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26602,7 +26602,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26706,7 +26706,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26810,7 +26810,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26914,7 +26914,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27018,7 +27018,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27122,7 +27122,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27226,7 +27226,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27330,7 +27330,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27434,7 +27434,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27538,7 +27538,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27642,7 +27642,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27746,7 +27746,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27850,7 +27850,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27954,7 +27954,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28058,7 +28058,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28162,7 +28162,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28266,7 +28266,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28370,7 +28370,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28474,7 +28474,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28578,7 +28578,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28682,7 +28682,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28786,7 +28786,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28890,7 +28890,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28994,7 +28994,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29098,7 +29098,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29202,7 +29202,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29306,7 +29306,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29410,7 +29410,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29514,7 +29514,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29618,7 +29618,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29722,7 +29722,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29826,7 +29826,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29930,7 +29930,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30034,7 +30034,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30138,7 +30138,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30242,7 +30242,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30346,7 +30346,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30450,7 +30450,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30554,7 +30554,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30658,7 +30658,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30762,7 +30762,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30866,7 +30866,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30970,7 +30970,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31074,7 +31074,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31178,7 +31178,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31282,7 +31282,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31386,7 +31386,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31490,7 +31490,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31594,7 +31594,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31698,7 +31698,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31802,7 +31802,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31906,7 +31906,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32010,7 +32010,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32114,7 +32114,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32218,7 +32218,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32322,7 +32322,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32426,7 +32426,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32530,7 +32530,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32634,7 +32634,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32738,7 +32738,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32842,7 +32842,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32946,7 +32946,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33050,7 +33050,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33154,7 +33154,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33258,7 +33258,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33362,7 +33362,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33466,7 +33466,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33570,7 +33570,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33674,7 +33674,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33778,7 +33778,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33882,7 +33882,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33986,7 +33986,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34090,7 +34090,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34194,7 +34194,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34298,7 +34298,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34402,7 +34402,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34506,7 +34506,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34610,7 +34610,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34714,7 +34714,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34818,7 +34818,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34922,7 +34922,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35026,7 +35026,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35130,7 +35130,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35234,7 +35234,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35338,7 +35338,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35442,7 +35442,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35546,7 +35546,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35650,7 +35650,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35754,7 +35754,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35858,7 +35858,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35962,7 +35962,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36066,7 +36066,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36170,7 +36170,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36181,7 +36181,7 @@
         <v>2561</v>
       </c>
       <c r="C191" s="4">
-        <v>13687956</v>
+        <v>14162840</v>
       </c>
       <c r="D191" s="3" t="s">
         <v>2562</v>
@@ -36274,7 +36274,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36378,7 +36378,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36482,7 +36482,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36586,7 +36586,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36690,7 +36690,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36794,7 +36794,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36898,7 +36898,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -37002,7 +37002,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37106,7 +37106,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37210,7 +37210,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37314,7 +37314,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37418,7 +37418,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37522,7 +37522,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37626,7 +37626,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37730,7 +37730,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37834,7 +37834,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37938,7 +37938,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38042,7 +38042,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38146,7 +38146,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38250,7 +38250,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38354,7 +38354,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38365,7 +38365,7 @@
         <v>2807</v>
       </c>
       <c r="C212" s="2">
-        <v>13712995</v>
+        <v>20673543</v>
       </c>
       <c r="D212" s="1" t="s">
         <v>2808</v>
@@ -38458,7 +38458,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38562,7 +38562,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38666,7 +38666,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38770,7 +38770,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38874,7 +38874,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38978,7 +38978,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39082,7 +39082,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39186,7 +39186,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39290,7 +39290,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39394,7 +39394,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39498,7 +39498,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39602,7 +39602,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39706,7 +39706,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39810,7 +39810,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39914,7 +39914,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40018,7 +40018,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40122,7 +40122,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40226,7 +40226,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40330,7 +40330,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40434,7 +40434,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40538,7 +40538,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40642,7 +40642,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40746,7 +40746,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40850,7 +40850,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40954,7 +40954,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41058,7 +41058,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41162,7 +41162,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41266,7 +41266,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41370,7 +41370,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41474,7 +41474,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41578,7 +41578,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41682,7 +41682,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41786,7 +41786,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41890,7 +41890,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41994,7 +41994,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42098,7 +42098,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42202,7 +42202,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42306,7 +42306,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42410,7 +42410,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42514,7 +42514,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42618,7 +42618,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42722,7 +42722,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42826,7 +42826,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42930,7 +42930,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43034,7 +43034,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43138,7 +43138,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43242,7 +43242,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43346,7 +43346,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43450,7 +43450,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43554,7 +43554,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43658,7 +43658,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43762,7 +43762,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43866,7 +43866,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43970,7 +43970,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44074,7 +44074,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44178,7 +44178,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44282,7 +44282,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44386,7 +44386,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44490,7 +44490,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44594,7 +44594,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44698,7 +44698,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44802,7 +44802,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44906,7 +44906,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45010,7 +45010,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45114,7 +45114,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45218,7 +45218,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45322,7 +45322,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45426,7 +45426,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45530,7 +45530,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45634,7 +45634,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45738,7 +45738,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45842,7 +45842,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45946,7 +45946,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46050,7 +46050,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46154,7 +46154,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46258,7 +46258,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46362,7 +46362,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46466,7 +46466,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46570,7 +46570,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46674,7 +46674,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46778,7 +46778,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46882,7 +46882,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46986,7 +46986,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47090,7 +47090,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47194,7 +47194,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47298,7 +47298,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47402,7 +47402,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47506,7 +47506,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47610,7 +47610,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47714,7 +47714,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47818,7 +47818,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47922,7 +47922,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48026,7 +48026,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48130,7 +48130,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48234,7 +48234,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48338,7 +48338,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48442,7 +48442,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48546,7 +48546,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48650,7 +48650,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48754,7 +48754,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48858,7 +48858,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48962,7 +48962,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49066,7 +49066,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49170,7 +49170,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49274,7 +49274,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49378,7 +49378,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49482,7 +49482,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49586,7 +49586,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49690,7 +49690,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49794,7 +49794,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49898,7 +49898,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -50002,7 +50002,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50106,7 +50106,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50210,7 +50210,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50314,7 +50314,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50418,7 +50418,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50522,7 +50522,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50626,7 +50626,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50730,7 +50730,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50834,7 +50834,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50938,7 +50938,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51042,7 +51042,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51146,7 +51146,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51250,7 +51250,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51354,7 +51354,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51458,7 +51458,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51562,7 +51562,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51666,7 +51666,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51770,7 +51770,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51874,7 +51874,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51978,7 +51978,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52082,7 +52082,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52186,7 +52186,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52290,7 +52290,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52394,7 +52394,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52498,7 +52498,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52602,7 +52602,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52706,7 +52706,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52810,7 +52810,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52914,7 +52914,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53018,7 +53018,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53122,7 +53122,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53226,7 +53226,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53330,7 +53330,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53434,7 +53434,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53538,7 +53538,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53592,7 +53592,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53696,7 +53696,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53800,7 +53800,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53904,7 +53904,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -54008,7 +54008,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54112,7 +54112,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54216,7 +54216,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54320,7 +54320,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54424,7 +54424,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54528,7 +54528,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54632,7 +54632,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54736,7 +54736,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54840,7 +54840,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54944,7 +54944,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55048,7 +55048,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55152,7 +55152,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55256,7 +55256,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55360,7 +55360,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55464,7 +55464,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55568,7 +55568,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55672,7 +55672,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55776,7 +55776,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55880,7 +55880,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55984,7 +55984,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56088,7 +56088,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56192,7 +56192,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56296,7 +56296,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56350,7 +56350,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56454,7 +56454,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56558,7 +56558,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56662,7 +56662,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56766,7 +56766,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56870,7 +56870,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46245.426747685182</v>
+        <v>46245.522210648145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-12 07:37:17
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16618,7 +16618,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16722,7 +16722,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16826,7 +16826,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16930,7 +16930,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17034,7 +17034,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17138,7 +17138,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17242,7 +17242,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17346,7 +17346,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17450,7 +17450,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17554,7 +17554,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17658,7 +17658,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17762,7 +17762,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17866,7 +17866,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17970,7 +17970,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18074,7 +18074,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18178,7 +18178,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18282,7 +18282,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18386,7 +18386,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18490,7 +18490,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18594,7 +18594,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18698,7 +18698,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18802,7 +18802,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18906,7 +18906,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19010,7 +19010,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19114,7 +19114,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19218,7 +19218,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19322,7 +19322,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19426,7 +19426,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19530,7 +19530,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19634,7 +19634,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19738,7 +19738,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19842,7 +19842,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19946,7 +19946,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20050,7 +20050,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20154,7 +20154,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20258,7 +20258,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20362,7 +20362,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20466,7 +20466,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20570,7 +20570,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20674,7 +20674,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20778,7 +20778,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20882,7 +20882,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20986,7 +20986,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21090,7 +21090,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21194,7 +21194,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21298,7 +21298,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21402,7 +21402,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21506,7 +21506,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21610,7 +21610,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21714,7 +21714,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21818,7 +21818,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21922,7 +21922,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22026,7 +22026,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22130,7 +22130,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22234,7 +22234,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22338,7 +22338,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22442,7 +22442,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22546,7 +22546,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22650,7 +22650,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22754,7 +22754,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22858,7 +22858,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22962,7 +22962,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23066,7 +23066,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23170,7 +23170,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23274,7 +23274,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23378,7 +23378,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23482,7 +23482,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23586,7 +23586,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23690,7 +23690,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23794,7 +23794,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23898,7 +23898,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -24002,7 +24002,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24106,7 +24106,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24210,7 +24210,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24314,7 +24314,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24418,7 +24418,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24522,7 +24522,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24626,7 +24626,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24730,7 +24730,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24834,7 +24834,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24938,7 +24938,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25042,7 +25042,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25146,7 +25146,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25250,7 +25250,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25354,7 +25354,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25458,7 +25458,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25562,7 +25562,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25666,7 +25666,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25770,7 +25770,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25874,7 +25874,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25978,7 +25978,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26082,7 +26082,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26186,7 +26186,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26290,7 +26290,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26394,7 +26394,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26498,7 +26498,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26602,7 +26602,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26706,7 +26706,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26810,7 +26810,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26914,7 +26914,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27018,7 +27018,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27122,7 +27122,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27226,7 +27226,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27330,7 +27330,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27434,7 +27434,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27538,7 +27538,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27642,7 +27642,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27746,7 +27746,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27850,7 +27850,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27954,7 +27954,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28058,7 +28058,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28162,7 +28162,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28266,7 +28266,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28370,7 +28370,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28474,7 +28474,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28578,7 +28578,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28682,7 +28682,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28786,7 +28786,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28890,7 +28890,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28994,7 +28994,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29098,7 +29098,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29202,7 +29202,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29306,7 +29306,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29410,7 +29410,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29514,7 +29514,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29618,7 +29618,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29722,7 +29722,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29826,7 +29826,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29930,7 +29930,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30034,7 +30034,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30138,7 +30138,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30242,7 +30242,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30346,7 +30346,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30450,7 +30450,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30554,7 +30554,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30658,7 +30658,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30762,7 +30762,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30866,7 +30866,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30970,7 +30970,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31074,7 +31074,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31178,7 +31178,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31282,7 +31282,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31386,7 +31386,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31490,7 +31490,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31594,7 +31594,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31698,7 +31698,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31802,7 +31802,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31906,7 +31906,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32010,7 +32010,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32114,7 +32114,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32218,7 +32218,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32322,7 +32322,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32426,7 +32426,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32530,7 +32530,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32634,7 +32634,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32738,7 +32738,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32842,7 +32842,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32946,7 +32946,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33050,7 +33050,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33154,7 +33154,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33258,7 +33258,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33362,7 +33362,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33466,7 +33466,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33570,7 +33570,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33674,7 +33674,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33778,7 +33778,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33882,7 +33882,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33986,7 +33986,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34090,7 +34090,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34194,7 +34194,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34298,7 +34298,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34402,7 +34402,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34506,7 +34506,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34610,7 +34610,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34714,7 +34714,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34818,7 +34818,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34922,7 +34922,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35026,7 +35026,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35130,7 +35130,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35234,7 +35234,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35338,7 +35338,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35442,7 +35442,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35546,7 +35546,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35650,7 +35650,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35754,7 +35754,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35858,7 +35858,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35962,7 +35962,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36066,7 +36066,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36170,7 +36170,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36274,7 +36274,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36378,7 +36378,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36482,7 +36482,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36586,7 +36586,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36690,7 +36690,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36794,7 +36794,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36898,7 +36898,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -37002,7 +37002,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37106,7 +37106,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37210,7 +37210,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37314,7 +37314,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37418,7 +37418,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37522,7 +37522,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37626,7 +37626,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37730,7 +37730,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37834,7 +37834,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37938,7 +37938,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38042,7 +38042,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38146,7 +38146,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38250,7 +38250,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38354,7 +38354,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38458,7 +38458,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38562,7 +38562,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38666,7 +38666,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38770,7 +38770,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38781,7 +38781,7 @@
         <v>2868</v>
       </c>
       <c r="C216" s="2">
-        <v>16370456</v>
+        <v>18325333</v>
       </c>
       <c r="D216" s="1" t="s">
         <v>2869</v>
@@ -38874,7 +38874,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38978,7 +38978,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39082,7 +39082,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39186,7 +39186,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39290,7 +39290,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39394,7 +39394,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39498,7 +39498,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39602,7 +39602,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39706,7 +39706,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39810,7 +39810,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39914,7 +39914,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40018,7 +40018,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40122,7 +40122,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40226,7 +40226,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40330,7 +40330,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40434,7 +40434,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40538,7 +40538,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40642,7 +40642,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40746,7 +40746,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40850,7 +40850,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40954,7 +40954,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41058,7 +41058,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41162,7 +41162,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41266,7 +41266,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41370,7 +41370,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41474,7 +41474,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41578,7 +41578,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41682,7 +41682,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41786,7 +41786,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41890,7 +41890,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41994,7 +41994,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42098,7 +42098,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42202,7 +42202,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42306,7 +42306,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42410,7 +42410,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42514,7 +42514,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42618,7 +42618,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42722,7 +42722,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42826,7 +42826,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42930,7 +42930,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43034,7 +43034,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43138,7 +43138,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43242,7 +43242,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43346,7 +43346,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43450,7 +43450,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43554,7 +43554,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43658,7 +43658,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43762,7 +43762,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43866,7 +43866,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43970,7 +43970,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44074,7 +44074,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44178,7 +44178,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44282,7 +44282,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44386,7 +44386,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44490,7 +44490,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44594,7 +44594,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44698,7 +44698,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44802,7 +44802,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44906,7 +44906,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45010,7 +45010,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45114,7 +45114,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45218,7 +45218,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45322,7 +45322,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45426,7 +45426,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45530,7 +45530,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45634,7 +45634,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45738,7 +45738,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45842,7 +45842,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45946,7 +45946,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46050,7 +46050,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46154,7 +46154,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46258,7 +46258,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46362,7 +46362,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46466,7 +46466,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46477,7 +46477,7 @@
         <v>3724</v>
       </c>
       <c r="C290" s="2">
-        <v>18064834</v>
+        <v>9669134</v>
       </c>
       <c r="D290" s="1" t="s">
         <v>2407</v>
@@ -46570,7 +46570,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46674,7 +46674,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46778,7 +46778,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46882,7 +46882,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46986,7 +46986,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47090,7 +47090,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47194,7 +47194,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47298,7 +47298,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47402,7 +47402,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47506,7 +47506,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47610,7 +47610,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47714,7 +47714,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47818,7 +47818,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47922,7 +47922,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48026,7 +48026,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48130,7 +48130,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48234,7 +48234,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48338,7 +48338,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48442,7 +48442,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48546,7 +48546,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48650,7 +48650,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48754,7 +48754,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48858,7 +48858,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48962,7 +48962,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49066,7 +49066,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49170,7 +49170,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49274,7 +49274,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49378,7 +49378,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49482,7 +49482,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49586,7 +49586,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49690,7 +49690,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49794,7 +49794,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49898,7 +49898,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -50002,7 +50002,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50106,7 +50106,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50210,7 +50210,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50314,7 +50314,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50418,7 +50418,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50522,7 +50522,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50626,7 +50626,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50730,7 +50730,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50834,7 +50834,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50938,7 +50938,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51042,7 +51042,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51146,7 +51146,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51250,7 +51250,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51354,7 +51354,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51458,7 +51458,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51562,7 +51562,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51666,7 +51666,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51770,7 +51770,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51874,7 +51874,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51885,7 +51885,7 @@
         <v>4365</v>
       </c>
       <c r="C342" s="2">
-        <v>15664265</v>
+        <v>15670492</v>
       </c>
       <c r="D342" s="1" t="s">
         <v>4366</v>
@@ -51978,7 +51978,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52082,7 +52082,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52186,7 +52186,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52290,7 +52290,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52394,7 +52394,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52498,7 +52498,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52602,7 +52602,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52706,7 +52706,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52810,7 +52810,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52914,7 +52914,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53018,7 +53018,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53122,7 +53122,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53226,7 +53226,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53330,7 +53330,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53434,7 +53434,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53538,7 +53538,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53592,7 +53592,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53696,7 +53696,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53800,7 +53800,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53904,7 +53904,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -54008,7 +54008,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54112,7 +54112,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54216,7 +54216,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54320,7 +54320,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54424,7 +54424,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54528,7 +54528,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54632,7 +54632,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54736,7 +54736,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54840,7 +54840,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54944,7 +54944,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55048,7 +55048,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55152,7 +55152,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55256,7 +55256,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55360,7 +55360,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55464,7 +55464,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55568,7 +55568,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55672,7 +55672,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55776,7 +55776,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55880,7 +55880,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55984,7 +55984,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56088,7 +56088,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56192,7 +56192,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56296,7 +56296,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56350,7 +56350,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56454,7 +56454,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56558,7 +56558,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56662,7 +56662,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56766,7 +56766,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56870,7 +56870,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46245.522210648145</v>
+        <v>46246.317557870374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-17 17:05:01
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16600,7 +16600,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16704,7 +16704,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16808,7 +16808,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16912,7 +16912,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17016,7 +17016,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17120,7 +17120,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17224,7 +17224,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17328,7 +17328,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17432,7 +17432,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17536,7 +17536,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17640,7 +17640,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17744,7 +17744,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17848,7 +17848,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17952,7 +17952,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18056,7 +18056,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18160,7 +18160,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18264,7 +18264,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18368,7 +18368,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18472,7 +18472,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18576,7 +18576,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18680,7 +18680,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18784,7 +18784,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18888,7 +18888,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -18992,7 +18992,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19096,7 +19096,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19200,7 +19200,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19304,7 +19304,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19408,7 +19408,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19512,7 +19512,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19616,7 +19616,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19720,7 +19720,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19824,7 +19824,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19928,7 +19928,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20032,7 +20032,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20136,7 +20136,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20240,7 +20240,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20344,7 +20344,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20448,7 +20448,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20552,7 +20552,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20656,7 +20656,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20760,7 +20760,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20864,7 +20864,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20968,7 +20968,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21072,7 +21072,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21176,7 +21176,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21280,7 +21280,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21384,7 +21384,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21488,7 +21488,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21592,7 +21592,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21696,7 +21696,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21707,7 +21707,7 @@
         <v>857</v>
       </c>
       <c r="C52" s="2">
-        <v>13078195</v>
+        <v>14255919</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>858</v>
@@ -21800,7 +21800,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21904,7 +21904,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22008,7 +22008,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22112,7 +22112,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22216,7 +22216,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22320,7 +22320,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22424,7 +22424,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22528,7 +22528,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22632,7 +22632,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22736,7 +22736,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22840,7 +22840,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22944,7 +22944,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23048,7 +23048,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23152,7 +23152,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23256,7 +23256,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23360,7 +23360,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23464,7 +23464,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23568,7 +23568,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23672,7 +23672,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23776,7 +23776,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23880,7 +23880,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23984,7 +23984,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24088,7 +24088,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24192,7 +24192,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24296,7 +24296,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24400,7 +24400,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24504,7 +24504,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24608,7 +24608,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24712,7 +24712,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24816,7 +24816,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24920,7 +24920,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25024,7 +25024,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25128,7 +25128,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25232,7 +25232,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25336,7 +25336,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25440,7 +25440,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25544,7 +25544,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25648,7 +25648,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25752,7 +25752,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25856,7 +25856,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25960,7 +25960,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26064,7 +26064,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26168,7 +26168,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26272,7 +26272,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26376,7 +26376,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26480,7 +26480,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26584,7 +26584,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26688,7 +26688,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26792,7 +26792,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26896,7 +26896,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27000,7 +27000,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27104,7 +27104,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27208,7 +27208,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27312,7 +27312,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27416,7 +27416,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27520,7 +27520,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27624,7 +27624,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27635,7 +27635,7 @@
         <v>1565</v>
       </c>
       <c r="C109" s="4">
-        <v>22886783</v>
+        <v>14538730</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>1566</v>
@@ -27728,7 +27728,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27832,7 +27832,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27936,7 +27936,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28040,7 +28040,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28144,7 +28144,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28248,7 +28248,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28352,7 +28352,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28456,7 +28456,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28560,7 +28560,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28664,7 +28664,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28768,7 +28768,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28872,7 +28872,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28976,7 +28976,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29080,7 +29080,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29184,7 +29184,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29288,7 +29288,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29392,7 +29392,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29496,7 +29496,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29600,7 +29600,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29704,7 +29704,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29808,7 +29808,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29912,7 +29912,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30016,7 +30016,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30120,7 +30120,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30224,7 +30224,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30328,7 +30328,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30432,7 +30432,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30536,7 +30536,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30640,7 +30640,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30744,7 +30744,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30848,7 +30848,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30952,7 +30952,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31056,7 +31056,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31160,7 +31160,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31264,7 +31264,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31368,7 +31368,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31472,7 +31472,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31576,7 +31576,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31680,7 +31680,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31784,7 +31784,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31888,7 +31888,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -31992,7 +31992,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32096,7 +32096,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32200,7 +32200,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32304,7 +32304,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32408,7 +32408,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32512,7 +32512,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32616,7 +32616,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32720,7 +32720,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32824,7 +32824,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32928,7 +32928,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33032,7 +33032,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33136,7 +33136,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33240,7 +33240,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33344,7 +33344,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33448,7 +33448,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33552,7 +33552,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33656,7 +33656,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33760,7 +33760,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33864,7 +33864,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33968,7 +33968,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34072,7 +34072,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34176,7 +34176,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34280,7 +34280,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34384,7 +34384,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34488,7 +34488,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34592,7 +34592,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34696,7 +34696,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34800,7 +34800,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34904,7 +34904,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35008,7 +35008,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35112,7 +35112,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35216,7 +35216,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35320,7 +35320,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35424,7 +35424,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35528,7 +35528,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35632,7 +35632,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35736,7 +35736,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35840,7 +35840,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35944,7 +35944,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36048,7 +36048,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36152,7 +36152,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36256,7 +36256,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36360,7 +36360,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36371,7 +36371,7 @@
         <v>2582</v>
       </c>
       <c r="C193" s="4">
-        <v>12106908</v>
+        <v>26485235</v>
       </c>
       <c r="D193" s="3" t="s">
         <v>2583</v>
@@ -36464,7 +36464,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36568,7 +36568,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36672,7 +36672,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36776,7 +36776,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36880,7 +36880,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36984,7 +36984,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37088,7 +37088,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37192,7 +37192,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37296,7 +37296,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37400,7 +37400,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37411,7 +37411,7 @@
         <v>2689</v>
       </c>
       <c r="C203" s="4">
-        <v>14654661</v>
+        <v>18360767</v>
       </c>
       <c r="D203" s="3" t="s">
         <v>2690</v>
@@ -37504,7 +37504,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37608,7 +37608,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37712,7 +37712,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37816,7 +37816,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37920,7 +37920,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38024,7 +38024,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38128,7 +38128,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38232,7 +38232,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38336,7 +38336,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38440,7 +38440,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38544,7 +38544,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38648,7 +38648,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38752,7 +38752,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38856,7 +38856,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38867,7 +38867,7 @@
         <v>2868</v>
       </c>
       <c r="C217" s="4">
-        <v>17788092</v>
+        <v>17522721</v>
       </c>
       <c r="D217" s="3" t="s">
         <v>2443</v>
@@ -38960,7 +38960,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39064,7 +39064,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39168,7 +39168,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39272,7 +39272,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39376,7 +39376,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39480,7 +39480,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39584,7 +39584,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39688,7 +39688,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39792,7 +39792,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39896,7 +39896,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40000,7 +40000,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40104,7 +40104,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40208,7 +40208,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40312,7 +40312,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40416,7 +40416,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40520,7 +40520,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40624,7 +40624,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40728,7 +40728,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40832,7 +40832,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40936,7 +40936,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41040,7 +41040,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41144,7 +41144,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41248,7 +41248,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41352,7 +41352,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41456,7 +41456,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41560,7 +41560,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41664,7 +41664,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41768,7 +41768,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41872,7 +41872,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41976,7 +41976,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42080,7 +42080,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42184,7 +42184,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42288,7 +42288,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42392,7 +42392,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42496,7 +42496,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42600,7 +42600,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42704,7 +42704,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42808,7 +42808,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42912,7 +42912,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43016,7 +43016,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43120,7 +43120,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43224,7 +43224,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43328,7 +43328,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43432,7 +43432,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43536,7 +43536,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43640,7 +43640,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43744,7 +43744,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43848,7 +43848,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43952,7 +43952,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44056,7 +44056,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44160,7 +44160,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44264,7 +44264,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44368,7 +44368,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44472,7 +44472,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44576,7 +44576,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44680,7 +44680,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44784,7 +44784,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44888,7 +44888,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -44992,7 +44992,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45096,7 +45096,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45200,7 +45200,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45211,7 +45211,7 @@
         <v>3563</v>
       </c>
       <c r="C278" s="2">
-        <v>8418949</v>
+        <v>26501300</v>
       </c>
       <c r="D278" s="1" t="s">
         <v>3564</v>
@@ -45304,7 +45304,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45408,7 +45408,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45512,7 +45512,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45616,7 +45616,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45720,7 +45720,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45824,7 +45824,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45928,7 +45928,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46032,7 +46032,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46136,7 +46136,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46240,7 +46240,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46344,7 +46344,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46448,7 +46448,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46552,7 +46552,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46656,7 +46656,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46760,7 +46760,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46864,7 +46864,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46968,7 +46968,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47072,7 +47072,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47176,7 +47176,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47280,7 +47280,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47384,7 +47384,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47488,7 +47488,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47592,7 +47592,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47696,7 +47696,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47800,7 +47800,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47904,7 +47904,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48008,7 +48008,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48112,7 +48112,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48216,7 +48216,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48320,7 +48320,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48424,7 +48424,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48528,7 +48528,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48632,7 +48632,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48736,7 +48736,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48840,7 +48840,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48944,7 +48944,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49048,7 +49048,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49152,7 +49152,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49256,7 +49256,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49360,7 +49360,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49464,7 +49464,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49568,7 +49568,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49672,7 +49672,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49776,7 +49776,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49880,7 +49880,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49984,7 +49984,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50088,7 +50088,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50192,7 +50192,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50296,7 +50296,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50400,7 +50400,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50504,7 +50504,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50608,7 +50608,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50712,7 +50712,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50816,7 +50816,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50920,7 +50920,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51024,7 +51024,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51128,7 +51128,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51232,7 +51232,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51336,7 +51336,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51440,7 +51440,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51544,7 +51544,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51648,7 +51648,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51752,7 +51752,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51856,7 +51856,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51960,7 +51960,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52064,7 +52064,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52168,7 +52168,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52272,7 +52272,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52376,7 +52376,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52480,7 +52480,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52584,7 +52584,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52688,7 +52688,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52792,7 +52792,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52896,7 +52896,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53000,7 +53000,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53104,7 +53104,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53208,7 +53208,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53312,7 +53312,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53416,7 +53416,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53520,7 +53520,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53574,7 +53574,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53678,7 +53678,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53782,7 +53782,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53886,7 +53886,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -53990,7 +53990,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54094,7 +54094,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54198,7 +54198,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54302,7 +54302,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54406,7 +54406,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54510,7 +54510,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54614,7 +54614,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54718,7 +54718,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54822,7 +54822,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54926,7 +54926,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55030,7 +55030,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55134,7 +55134,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55238,7 +55238,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55342,7 +55342,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55446,7 +55446,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55550,7 +55550,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55654,7 +55654,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55758,7 +55758,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55862,7 +55862,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55966,7 +55966,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56070,7 +56070,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56174,7 +56174,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56278,7 +56278,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56332,7 +56332,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56436,7 +56436,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56540,7 +56540,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56644,7 +56644,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56748,7 +56748,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56852,7 +56852,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46251.463067129633</v>
+        <v>46251.711817129632</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-20 09:55:29
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16609,7 +16609,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16713,7 +16713,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16817,7 +16817,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16921,7 +16921,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17025,7 +17025,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17129,7 +17129,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17233,7 +17233,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17337,7 +17337,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17441,7 +17441,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17545,7 +17545,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17649,7 +17649,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17753,7 +17753,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17857,7 +17857,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17961,7 +17961,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18065,7 +18065,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18169,7 +18169,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18273,7 +18273,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18377,7 +18377,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18481,7 +18481,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18585,7 +18585,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18689,7 +18689,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18793,7 +18793,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18897,7 +18897,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19001,7 +19001,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19105,7 +19105,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19209,7 +19209,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19313,7 +19313,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19417,7 +19417,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19521,7 +19521,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19625,7 +19625,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19729,7 +19729,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19833,7 +19833,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19937,7 +19937,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20041,7 +20041,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20145,7 +20145,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20249,7 +20249,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20353,7 +20353,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20457,7 +20457,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20561,7 +20561,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20665,7 +20665,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20769,7 +20769,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20873,7 +20873,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20977,7 +20977,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21081,7 +21081,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21185,7 +21185,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21289,7 +21289,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21393,7 +21393,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21497,7 +21497,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21601,7 +21601,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21705,7 +21705,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21809,7 +21809,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21913,7 +21913,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22017,7 +22017,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22121,7 +22121,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22225,7 +22225,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22329,7 +22329,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22433,7 +22433,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22537,7 +22537,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22641,7 +22641,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22745,7 +22745,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22849,7 +22849,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22953,7 +22953,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23057,7 +23057,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23161,7 +23161,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23265,7 +23265,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23369,7 +23369,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23473,7 +23473,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23577,7 +23577,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23681,7 +23681,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23785,7 +23785,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23889,7 +23889,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23993,7 +23993,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24097,7 +24097,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24201,7 +24201,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24305,7 +24305,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24409,7 +24409,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24513,7 +24513,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24617,7 +24617,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24721,7 +24721,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24825,7 +24825,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24929,7 +24929,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25033,7 +25033,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25137,7 +25137,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25241,7 +25241,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25345,7 +25345,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25449,7 +25449,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25553,7 +25553,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25657,7 +25657,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25761,7 +25761,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25865,7 +25865,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25969,7 +25969,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26073,7 +26073,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26177,7 +26177,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26281,7 +26281,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26385,7 +26385,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26489,7 +26489,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26593,7 +26593,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26697,7 +26697,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26801,7 +26801,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26905,7 +26905,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27009,7 +27009,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27113,7 +27113,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27217,7 +27217,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27321,7 +27321,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27425,7 +27425,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27529,7 +27529,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27633,7 +27633,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27737,7 +27737,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27841,7 +27841,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27945,7 +27945,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28049,7 +28049,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28153,7 +28153,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28257,7 +28257,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28361,7 +28361,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28465,7 +28465,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28569,7 +28569,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28673,7 +28673,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28777,7 +28777,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28881,7 +28881,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28985,7 +28985,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29089,7 +29089,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29193,7 +29193,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29297,7 +29297,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29401,7 +29401,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29505,7 +29505,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29609,7 +29609,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29713,7 +29713,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29817,7 +29817,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29921,7 +29921,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30025,7 +30025,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30129,7 +30129,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30233,7 +30233,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30337,7 +30337,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30441,7 +30441,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30545,7 +30545,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30556,7 +30556,7 @@
         <v>1939</v>
       </c>
       <c r="C137" s="4">
-        <v>15830950</v>
+        <v>16419354</v>
       </c>
       <c r="D137" s="3" t="s">
         <v>1940</v>
@@ -30649,7 +30649,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30753,7 +30753,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30857,7 +30857,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30961,7 +30961,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31065,7 +31065,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31169,7 +31169,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31273,7 +31273,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31377,7 +31377,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31481,7 +31481,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31585,7 +31585,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31689,7 +31689,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31793,7 +31793,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31897,7 +31897,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32001,7 +32001,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32105,7 +32105,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32209,7 +32209,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32313,7 +32313,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32417,7 +32417,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32521,7 +32521,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32625,7 +32625,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32729,7 +32729,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32833,7 +32833,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32937,7 +32937,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33041,7 +33041,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33145,7 +33145,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33249,7 +33249,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33353,7 +33353,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33457,7 +33457,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33561,7 +33561,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33665,7 +33665,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33769,7 +33769,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33873,7 +33873,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33977,7 +33977,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34081,7 +34081,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34185,7 +34185,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34289,7 +34289,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34393,7 +34393,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34497,7 +34497,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34601,7 +34601,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34705,7 +34705,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34809,7 +34809,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34820,7 +34820,7 @@
         <v>2402</v>
       </c>
       <c r="C178" s="2">
-        <v>23232923</v>
+        <v>13078195</v>
       </c>
       <c r="D178" s="1" t="s">
         <v>2403</v>
@@ -34913,7 +34913,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35017,7 +35017,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35121,7 +35121,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35225,7 +35225,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35329,7 +35329,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35433,7 +35433,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35537,7 +35537,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35641,7 +35641,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35745,7 +35745,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35849,7 +35849,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35953,7 +35953,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36057,7 +36057,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36161,7 +36161,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36265,7 +36265,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36369,7 +36369,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36473,7 +36473,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36577,7 +36577,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36681,7 +36681,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36785,7 +36785,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36889,7 +36889,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36993,7 +36993,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37097,7 +37097,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37201,7 +37201,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37305,7 +37305,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37409,7 +37409,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37513,7 +37513,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37617,7 +37617,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37721,7 +37721,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37825,7 +37825,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37929,7 +37929,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38033,7 +38033,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38137,7 +38137,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38241,7 +38241,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38345,7 +38345,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38449,7 +38449,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38553,7 +38553,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38657,7 +38657,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38761,7 +38761,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38865,7 +38865,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38969,7 +38969,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39073,7 +39073,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39177,7 +39177,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39281,7 +39281,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39385,7 +39385,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39489,7 +39489,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39593,7 +39593,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39697,7 +39697,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39801,7 +39801,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39905,7 +39905,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40009,7 +40009,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40113,7 +40113,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40217,7 +40217,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40321,7 +40321,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40425,7 +40425,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40529,7 +40529,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40633,7 +40633,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40737,7 +40737,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40841,7 +40841,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40945,7 +40945,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41049,7 +41049,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41153,7 +41153,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41257,7 +41257,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41361,7 +41361,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41465,7 +41465,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41569,7 +41569,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41673,7 +41673,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41777,7 +41777,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41881,7 +41881,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41985,7 +41985,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42089,7 +42089,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42193,7 +42193,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42297,7 +42297,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42401,7 +42401,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42505,7 +42505,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42609,7 +42609,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42713,7 +42713,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42817,7 +42817,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42921,7 +42921,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43025,7 +43025,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43129,7 +43129,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43233,7 +43233,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43337,7 +43337,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43441,7 +43441,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43545,7 +43545,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43649,7 +43649,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43753,7 +43753,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43857,7 +43857,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43961,7 +43961,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44065,7 +44065,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44169,7 +44169,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44273,7 +44273,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44377,7 +44377,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44481,7 +44481,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44585,7 +44585,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44689,7 +44689,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44793,7 +44793,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44897,7 +44897,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45001,7 +45001,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45105,7 +45105,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45209,7 +45209,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45313,7 +45313,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45417,7 +45417,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45521,7 +45521,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45625,7 +45625,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45729,7 +45729,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45833,7 +45833,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45937,7 +45937,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46041,7 +46041,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46145,7 +46145,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46249,7 +46249,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46353,7 +46353,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46457,7 +46457,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46561,7 +46561,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46665,7 +46665,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46769,7 +46769,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46873,7 +46873,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46977,7 +46977,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47081,7 +47081,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47185,7 +47185,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47289,7 +47289,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47393,7 +47393,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47404,7 +47404,7 @@
         <v>3832</v>
       </c>
       <c r="C299" s="4">
-        <v>14255919</v>
+        <v>13078195</v>
       </c>
       <c r="D299" s="3" t="s">
         <v>3050</v>
@@ -47497,7 +47497,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47601,7 +47601,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47705,7 +47705,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47809,7 +47809,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47913,7 +47913,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48017,7 +48017,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48121,7 +48121,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48225,7 +48225,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48329,7 +48329,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48433,7 +48433,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48537,7 +48537,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48641,7 +48641,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48745,7 +48745,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48849,7 +48849,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48953,7 +48953,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49057,7 +49057,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49161,7 +49161,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49265,7 +49265,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49369,7 +49369,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49473,7 +49473,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49577,7 +49577,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49681,7 +49681,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49785,7 +49785,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49889,7 +49889,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49993,7 +49993,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50097,7 +50097,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50201,7 +50201,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50305,7 +50305,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50409,7 +50409,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50513,7 +50513,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50617,7 +50617,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50721,7 +50721,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50825,7 +50825,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50929,7 +50929,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51033,7 +51033,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51137,7 +51137,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51241,7 +51241,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51345,7 +51345,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51449,7 +51449,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51553,7 +51553,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51657,7 +51657,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51761,7 +51761,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51865,7 +51865,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51969,7 +51969,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52073,7 +52073,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52177,7 +52177,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52281,7 +52281,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52385,7 +52385,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52489,7 +52489,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52593,7 +52593,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52697,7 +52697,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52801,7 +52801,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52905,7 +52905,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53009,7 +53009,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53113,7 +53113,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53217,7 +53217,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53321,7 +53321,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53332,7 +53332,7 @@
         <v>4517</v>
       </c>
       <c r="C356" s="2">
-        <v>23232923</v>
+        <v>13078195</v>
       </c>
       <c r="D356" s="1" t="s">
         <v>3050</v>
@@ -53425,7 +53425,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53529,7 +53529,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53583,7 +53583,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53687,7 +53687,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53791,7 +53791,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53895,7 +53895,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -53999,7 +53999,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54103,7 +54103,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54207,7 +54207,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54311,7 +54311,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54415,7 +54415,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54519,7 +54519,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54623,7 +54623,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54727,7 +54727,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54831,7 +54831,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54935,7 +54935,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55039,7 +55039,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55143,7 +55143,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55247,7 +55247,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55351,7 +55351,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55455,7 +55455,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55559,7 +55559,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55663,7 +55663,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55767,7 +55767,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55871,7 +55871,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55975,7 +55975,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56079,7 +56079,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56183,7 +56183,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56287,7 +56287,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56341,7 +56341,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56445,7 +56445,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56549,7 +56549,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56653,7 +56653,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56757,7 +56757,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56861,7 +56861,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46254.387118055558</v>
+        <v>46254.413530092592</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-20 11:33:51
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16609,7 +16609,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16713,7 +16713,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16817,7 +16817,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16921,7 +16921,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17025,7 +17025,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17129,7 +17129,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17233,7 +17233,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17337,7 +17337,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17441,7 +17441,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17545,7 +17545,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17649,7 +17649,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17753,7 +17753,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17857,7 +17857,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17961,7 +17961,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18065,7 +18065,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18169,7 +18169,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18273,7 +18273,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18377,7 +18377,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18481,7 +18481,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18585,7 +18585,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18689,7 +18689,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18793,7 +18793,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18897,7 +18897,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19001,7 +19001,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19105,7 +19105,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19209,7 +19209,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19313,7 +19313,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19417,7 +19417,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19521,7 +19521,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19625,7 +19625,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19729,7 +19729,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19833,7 +19833,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19937,7 +19937,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20041,7 +20041,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20145,7 +20145,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20249,7 +20249,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20353,7 +20353,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20457,7 +20457,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20561,7 +20561,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20665,7 +20665,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20769,7 +20769,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20873,7 +20873,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20977,7 +20977,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21081,7 +21081,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21185,7 +21185,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21289,7 +21289,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21393,7 +21393,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21497,7 +21497,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21601,7 +21601,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21705,7 +21705,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21809,7 +21809,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21913,7 +21913,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22017,7 +22017,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22121,7 +22121,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22225,7 +22225,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22329,7 +22329,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22433,7 +22433,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22537,7 +22537,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22641,7 +22641,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22745,7 +22745,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22849,7 +22849,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22953,7 +22953,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23057,7 +23057,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23161,7 +23161,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23265,7 +23265,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23369,7 +23369,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23473,7 +23473,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23577,7 +23577,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23681,7 +23681,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23785,7 +23785,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23889,7 +23889,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23993,7 +23993,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24097,7 +24097,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24201,7 +24201,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24305,7 +24305,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24409,7 +24409,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24513,7 +24513,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24617,7 +24617,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24721,7 +24721,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24825,7 +24825,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24929,7 +24929,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25033,7 +25033,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25137,7 +25137,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25241,7 +25241,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25345,7 +25345,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25449,7 +25449,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25553,7 +25553,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25657,7 +25657,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25761,7 +25761,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25865,7 +25865,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25969,7 +25969,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26073,7 +26073,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26177,7 +26177,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26281,7 +26281,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26385,7 +26385,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26489,7 +26489,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26593,7 +26593,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26697,7 +26697,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26801,7 +26801,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26905,7 +26905,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27009,7 +27009,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27113,7 +27113,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27217,7 +27217,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27321,7 +27321,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27425,7 +27425,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27529,7 +27529,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27633,7 +27633,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27737,7 +27737,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27841,7 +27841,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27945,7 +27945,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28049,7 +28049,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28153,7 +28153,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28257,7 +28257,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28361,7 +28361,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28465,7 +28465,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28569,7 +28569,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28673,7 +28673,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28777,7 +28777,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28881,7 +28881,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28985,7 +28985,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29089,7 +29089,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29193,7 +29193,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29297,7 +29297,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29401,7 +29401,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29505,7 +29505,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29609,7 +29609,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29713,7 +29713,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29817,7 +29817,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29921,7 +29921,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30025,7 +30025,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30129,7 +30129,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30233,7 +30233,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30337,7 +30337,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30441,7 +30441,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30545,7 +30545,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30649,7 +30649,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30753,7 +30753,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30857,7 +30857,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30961,7 +30961,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31065,7 +31065,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31169,7 +31169,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31273,7 +31273,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31377,7 +31377,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31481,7 +31481,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31585,7 +31585,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31689,7 +31689,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31793,7 +31793,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31897,7 +31897,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32001,7 +32001,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32105,7 +32105,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32209,7 +32209,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32313,7 +32313,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32417,7 +32417,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32521,7 +32521,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32625,7 +32625,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32729,7 +32729,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32833,7 +32833,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32937,7 +32937,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33041,7 +33041,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33145,7 +33145,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33249,7 +33249,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33353,7 +33353,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33457,7 +33457,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33561,7 +33561,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33665,7 +33665,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33769,7 +33769,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33873,7 +33873,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33977,7 +33977,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34081,7 +34081,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34185,7 +34185,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34289,7 +34289,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34393,7 +34393,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34497,7 +34497,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34601,7 +34601,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34705,7 +34705,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34809,7 +34809,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34913,7 +34913,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35017,7 +35017,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35121,7 +35121,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35225,7 +35225,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35329,7 +35329,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35433,7 +35433,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35537,7 +35537,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35641,7 +35641,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35745,7 +35745,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35849,7 +35849,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35953,7 +35953,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36057,7 +36057,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36161,7 +36161,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36265,7 +36265,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36369,7 +36369,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36473,7 +36473,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36577,7 +36577,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36681,7 +36681,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36785,7 +36785,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36889,7 +36889,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36993,7 +36993,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37097,7 +37097,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37201,7 +37201,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37305,7 +37305,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37409,7 +37409,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37513,7 +37513,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37617,7 +37617,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37721,7 +37721,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37825,7 +37825,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37929,7 +37929,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38033,7 +38033,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38137,7 +38137,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38241,7 +38241,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38345,7 +38345,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38449,7 +38449,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38553,7 +38553,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38657,7 +38657,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38761,7 +38761,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38865,7 +38865,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38969,7 +38969,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39073,7 +39073,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39177,7 +39177,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39281,7 +39281,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39385,7 +39385,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39489,7 +39489,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39593,7 +39593,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39697,7 +39697,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39801,7 +39801,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39905,7 +39905,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40009,7 +40009,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40113,7 +40113,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40217,7 +40217,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40321,7 +40321,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40425,7 +40425,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40529,7 +40529,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40633,7 +40633,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40737,7 +40737,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40841,7 +40841,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40945,7 +40945,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41049,7 +41049,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41153,7 +41153,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41257,7 +41257,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41361,7 +41361,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41465,7 +41465,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41569,7 +41569,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41673,7 +41673,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41777,7 +41777,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41881,7 +41881,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41985,7 +41985,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42089,7 +42089,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42193,7 +42193,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42297,7 +42297,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42401,7 +42401,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42505,7 +42505,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42609,7 +42609,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42713,7 +42713,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42817,7 +42817,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42921,7 +42921,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43025,7 +43025,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43129,7 +43129,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43233,7 +43233,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43337,7 +43337,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43441,7 +43441,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43545,7 +43545,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43649,7 +43649,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43753,7 +43753,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43857,7 +43857,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43961,7 +43961,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44065,7 +44065,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44169,7 +44169,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44273,7 +44273,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44377,7 +44377,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44481,7 +44481,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44585,7 +44585,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44689,7 +44689,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44793,7 +44793,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44897,7 +44897,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45001,7 +45001,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45105,7 +45105,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45209,7 +45209,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45313,7 +45313,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45417,7 +45417,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45521,7 +45521,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45625,7 +45625,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45729,7 +45729,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45833,7 +45833,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45937,7 +45937,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46041,7 +46041,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46145,7 +46145,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46249,7 +46249,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46353,7 +46353,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46457,7 +46457,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46561,7 +46561,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46665,7 +46665,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46769,7 +46769,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46873,7 +46873,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46977,7 +46977,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47081,7 +47081,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47185,7 +47185,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47289,7 +47289,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47393,7 +47393,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47497,7 +47497,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47601,7 +47601,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47705,7 +47705,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47809,7 +47809,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47913,7 +47913,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48017,7 +48017,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48121,7 +48121,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48225,7 +48225,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48329,7 +48329,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48433,7 +48433,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48537,7 +48537,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48641,7 +48641,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48745,7 +48745,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48849,7 +48849,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48953,7 +48953,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49057,7 +49057,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49161,7 +49161,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49265,7 +49265,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49369,7 +49369,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49473,7 +49473,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49577,7 +49577,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49681,7 +49681,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49785,7 +49785,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49889,7 +49889,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49993,7 +49993,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50097,7 +50097,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50201,7 +50201,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50305,7 +50305,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50409,7 +50409,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50513,7 +50513,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50617,7 +50617,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50721,7 +50721,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50825,7 +50825,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50929,7 +50929,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51033,7 +51033,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51137,7 +51137,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51241,7 +51241,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51345,7 +51345,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51449,7 +51449,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51553,7 +51553,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51657,7 +51657,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51761,7 +51761,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51865,7 +51865,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51969,7 +51969,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52073,7 +52073,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52177,7 +52177,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52281,7 +52281,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52385,7 +52385,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52489,7 +52489,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52593,7 +52593,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52697,7 +52697,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52801,7 +52801,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52905,7 +52905,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53009,7 +53009,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53113,7 +53113,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53217,7 +53217,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53321,7 +53321,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53425,7 +53425,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53529,7 +53529,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53583,7 +53583,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53687,7 +53687,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53791,7 +53791,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53895,7 +53895,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -53999,7 +53999,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54103,7 +54103,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54207,7 +54207,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54311,7 +54311,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54415,7 +54415,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54519,7 +54519,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54623,7 +54623,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54727,7 +54727,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54831,7 +54831,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54935,7 +54935,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55039,7 +55039,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55143,7 +55143,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55247,7 +55247,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55351,7 +55351,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55455,7 +55455,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55559,7 +55559,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55663,7 +55663,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55767,7 +55767,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55871,7 +55871,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55975,7 +55975,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56079,7 +56079,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56183,7 +56183,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56287,7 +56287,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56341,7 +56341,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56445,7 +56445,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56549,7 +56549,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56653,7 +56653,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56757,7 +56757,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56861,7 +56861,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46254.413530092592</v>
+        <v>46254.481840277775</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-21 08:00:01
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16609,7 +16609,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16713,7 +16713,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16817,7 +16817,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16921,7 +16921,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17025,7 +17025,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17129,7 +17129,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17233,7 +17233,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17337,7 +17337,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17441,7 +17441,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17545,7 +17545,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17649,7 +17649,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17753,7 +17753,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17857,7 +17857,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17961,7 +17961,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18065,7 +18065,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18169,7 +18169,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18273,7 +18273,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18377,7 +18377,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18481,7 +18481,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18585,7 +18585,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18689,7 +18689,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18793,7 +18793,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18897,7 +18897,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19001,7 +19001,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19105,7 +19105,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19209,7 +19209,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19313,7 +19313,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19417,7 +19417,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19521,7 +19521,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19625,7 +19625,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19729,7 +19729,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19833,7 +19833,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19937,7 +19937,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20041,7 +20041,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20145,7 +20145,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20249,7 +20249,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20353,7 +20353,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20457,7 +20457,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20561,7 +20561,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20665,7 +20665,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20769,7 +20769,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20873,7 +20873,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20977,7 +20977,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21081,7 +21081,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21185,7 +21185,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21289,7 +21289,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21393,7 +21393,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21497,7 +21497,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21601,7 +21601,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21705,7 +21705,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21809,7 +21809,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21913,7 +21913,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22017,7 +22017,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22121,7 +22121,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22225,7 +22225,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22329,7 +22329,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22433,7 +22433,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22537,7 +22537,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22641,7 +22641,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22745,7 +22745,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22849,7 +22849,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22953,7 +22953,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23057,7 +23057,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23161,7 +23161,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23265,7 +23265,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23369,7 +23369,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23473,7 +23473,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23577,7 +23577,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23681,7 +23681,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23785,7 +23785,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23889,7 +23889,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23993,7 +23993,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24097,7 +24097,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24201,7 +24201,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24305,7 +24305,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24409,7 +24409,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24513,7 +24513,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24617,7 +24617,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24721,7 +24721,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24825,7 +24825,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24929,7 +24929,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25033,7 +25033,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25137,7 +25137,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25241,7 +25241,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25345,7 +25345,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25449,7 +25449,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25553,7 +25553,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25657,7 +25657,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25761,7 +25761,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25865,7 +25865,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25969,7 +25969,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26073,7 +26073,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26177,7 +26177,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26281,7 +26281,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26385,7 +26385,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26489,7 +26489,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26593,7 +26593,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26697,7 +26697,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26801,7 +26801,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26905,7 +26905,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27009,7 +27009,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27113,7 +27113,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27217,7 +27217,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27321,7 +27321,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27425,7 +27425,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27529,7 +27529,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27633,7 +27633,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27737,7 +27737,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27841,7 +27841,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27945,7 +27945,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28049,7 +28049,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28153,7 +28153,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28257,7 +28257,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28361,7 +28361,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28465,7 +28465,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28569,7 +28569,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28673,7 +28673,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28777,7 +28777,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28881,7 +28881,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28985,7 +28985,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29089,7 +29089,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29193,7 +29193,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29297,7 +29297,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29401,7 +29401,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29505,7 +29505,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29609,7 +29609,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29713,7 +29713,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29817,7 +29817,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29921,7 +29921,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30025,7 +30025,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30129,7 +30129,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30233,7 +30233,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30337,7 +30337,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30441,7 +30441,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30545,7 +30545,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30649,7 +30649,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30753,7 +30753,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30857,7 +30857,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30961,7 +30961,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31065,7 +31065,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31169,7 +31169,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31273,7 +31273,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31377,7 +31377,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31481,7 +31481,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31585,7 +31585,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31689,7 +31689,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31793,7 +31793,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31897,7 +31897,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32001,7 +32001,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32105,7 +32105,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32209,7 +32209,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32313,7 +32313,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32417,7 +32417,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32521,7 +32521,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32625,7 +32625,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32729,7 +32729,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32833,7 +32833,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32937,7 +32937,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33041,7 +33041,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33145,7 +33145,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33249,7 +33249,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33353,7 +33353,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33457,7 +33457,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33561,7 +33561,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33665,7 +33665,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33769,7 +33769,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33873,7 +33873,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33977,7 +33977,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34081,7 +34081,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34185,7 +34185,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34289,7 +34289,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34393,7 +34393,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34497,7 +34497,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34601,7 +34601,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34705,7 +34705,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34809,7 +34809,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34913,7 +34913,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35017,7 +35017,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35121,7 +35121,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35225,7 +35225,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35329,7 +35329,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35433,7 +35433,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35537,7 +35537,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35641,7 +35641,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35745,7 +35745,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35849,7 +35849,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35953,7 +35953,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36057,7 +36057,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36161,7 +36161,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36265,7 +36265,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36369,7 +36369,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36473,7 +36473,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36577,7 +36577,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36681,7 +36681,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36785,7 +36785,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36889,7 +36889,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36993,7 +36993,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37097,7 +37097,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37201,7 +37201,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37305,7 +37305,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37409,7 +37409,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37513,7 +37513,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37617,7 +37617,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37721,7 +37721,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37825,7 +37825,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37929,7 +37929,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38033,7 +38033,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38137,7 +38137,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38241,7 +38241,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38345,7 +38345,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38449,7 +38449,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38553,7 +38553,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38657,7 +38657,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38761,7 +38761,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38865,7 +38865,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38969,7 +38969,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39073,7 +39073,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39177,7 +39177,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39281,7 +39281,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39385,7 +39385,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39489,7 +39489,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39593,7 +39593,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39697,7 +39697,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39801,7 +39801,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39905,7 +39905,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40009,7 +40009,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40113,7 +40113,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40217,7 +40217,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40321,7 +40321,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40425,7 +40425,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40529,7 +40529,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40633,7 +40633,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40737,7 +40737,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40841,7 +40841,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40945,7 +40945,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41049,7 +41049,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41153,7 +41153,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41257,7 +41257,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41361,7 +41361,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41465,7 +41465,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41569,7 +41569,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41673,7 +41673,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41777,7 +41777,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41881,7 +41881,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41985,7 +41985,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42089,7 +42089,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42193,7 +42193,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42297,7 +42297,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42401,7 +42401,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42505,7 +42505,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42609,7 +42609,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42713,7 +42713,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42817,7 +42817,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42921,7 +42921,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43025,7 +43025,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43129,7 +43129,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43233,7 +43233,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43337,7 +43337,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43441,7 +43441,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43545,7 +43545,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43649,7 +43649,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43753,7 +43753,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43857,7 +43857,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43961,7 +43961,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44065,7 +44065,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44169,7 +44169,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44273,7 +44273,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44377,7 +44377,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44481,7 +44481,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44585,7 +44585,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44689,7 +44689,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44793,7 +44793,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44897,7 +44897,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45001,7 +45001,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45105,7 +45105,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45209,7 +45209,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45313,7 +45313,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45417,7 +45417,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45521,7 +45521,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45625,7 +45625,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45729,7 +45729,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45833,7 +45833,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45937,7 +45937,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46041,7 +46041,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46145,7 +46145,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46249,7 +46249,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46353,7 +46353,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46457,7 +46457,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46561,7 +46561,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46665,7 +46665,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46769,7 +46769,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46873,7 +46873,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46977,7 +46977,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47081,7 +47081,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47185,7 +47185,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47289,7 +47289,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47393,7 +47393,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47497,7 +47497,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47601,7 +47601,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47705,7 +47705,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47809,7 +47809,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47913,7 +47913,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48017,7 +48017,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48121,7 +48121,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48225,7 +48225,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48329,7 +48329,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48433,7 +48433,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48537,7 +48537,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48641,7 +48641,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48745,7 +48745,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48849,7 +48849,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48953,7 +48953,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49057,7 +49057,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49161,7 +49161,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49265,7 +49265,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49369,7 +49369,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49473,7 +49473,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49577,7 +49577,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49681,7 +49681,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49785,7 +49785,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49889,7 +49889,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49993,7 +49993,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50097,7 +50097,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50201,7 +50201,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50305,7 +50305,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50409,7 +50409,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50513,7 +50513,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50617,7 +50617,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50721,7 +50721,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50825,7 +50825,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50929,7 +50929,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51033,7 +51033,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51137,7 +51137,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51241,7 +51241,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51345,7 +51345,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51449,7 +51449,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51553,7 +51553,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51657,7 +51657,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51761,7 +51761,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51865,7 +51865,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51969,7 +51969,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52073,7 +52073,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52177,7 +52177,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52281,7 +52281,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52385,7 +52385,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52489,7 +52489,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52593,7 +52593,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52697,7 +52697,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52801,7 +52801,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52905,7 +52905,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53009,7 +53009,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53113,7 +53113,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53217,7 +53217,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53321,7 +53321,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53425,7 +53425,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53529,7 +53529,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53583,7 +53583,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53687,7 +53687,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53791,7 +53791,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53895,7 +53895,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -53999,7 +53999,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54103,7 +54103,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54207,7 +54207,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54311,7 +54311,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54415,7 +54415,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54519,7 +54519,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54623,7 +54623,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54727,7 +54727,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54831,7 +54831,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54935,7 +54935,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55039,7 +55039,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55143,7 +55143,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55247,7 +55247,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55351,7 +55351,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55455,7 +55455,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55559,7 +55559,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55663,7 +55663,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55767,7 +55767,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55871,7 +55871,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55975,7 +55975,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56079,7 +56079,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56183,7 +56183,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56287,7 +56287,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56341,7 +56341,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56445,7 +56445,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56549,7 +56549,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56653,7 +56653,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56757,7 +56757,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56861,7 +56861,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46254.481840277775</v>
+        <v>46255.333344907405</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-23 08:00:05
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16615,7 +16615,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16719,7 +16719,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16823,7 +16823,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16927,7 +16927,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17031,7 +17031,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17135,7 +17135,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17239,7 +17239,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17343,7 +17343,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17447,7 +17447,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17551,7 +17551,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17655,7 +17655,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17759,7 +17759,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17863,7 +17863,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17967,7 +17967,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18071,7 +18071,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18175,7 +18175,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18279,7 +18279,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18383,7 +18383,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18487,7 +18487,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18591,7 +18591,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18695,7 +18695,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18799,7 +18799,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18903,7 +18903,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19007,7 +19007,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19111,7 +19111,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19215,7 +19215,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19319,7 +19319,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19423,7 +19423,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19527,7 +19527,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19631,7 +19631,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19735,7 +19735,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19839,7 +19839,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19943,7 +19943,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20047,7 +20047,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20151,7 +20151,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20255,7 +20255,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20359,7 +20359,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20463,7 +20463,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20567,7 +20567,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20671,7 +20671,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20775,7 +20775,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20879,7 +20879,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20983,7 +20983,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21087,7 +21087,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21191,7 +21191,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21295,7 +21295,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21399,7 +21399,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21503,7 +21503,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21607,7 +21607,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21711,7 +21711,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21815,7 +21815,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21919,7 +21919,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22023,7 +22023,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22127,7 +22127,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22231,7 +22231,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22335,7 +22335,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22439,7 +22439,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22543,7 +22543,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22647,7 +22647,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22751,7 +22751,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22855,7 +22855,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22959,7 +22959,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23063,7 +23063,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23167,7 +23167,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23271,7 +23271,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23375,7 +23375,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23479,7 +23479,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23583,7 +23583,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23687,7 +23687,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23791,7 +23791,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23895,7 +23895,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23999,7 +23999,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24103,7 +24103,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24207,7 +24207,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24311,7 +24311,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24415,7 +24415,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24519,7 +24519,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24623,7 +24623,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24727,7 +24727,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24831,7 +24831,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24935,7 +24935,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25039,7 +25039,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25143,7 +25143,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25247,7 +25247,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25351,7 +25351,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25455,7 +25455,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25559,7 +25559,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25663,7 +25663,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25767,7 +25767,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25871,7 +25871,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25975,7 +25975,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26079,7 +26079,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26183,7 +26183,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26287,7 +26287,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26391,7 +26391,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26495,7 +26495,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26599,7 +26599,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26703,7 +26703,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26807,7 +26807,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26911,7 +26911,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27015,7 +27015,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27119,7 +27119,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27223,7 +27223,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27327,7 +27327,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27431,7 +27431,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27535,7 +27535,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27639,7 +27639,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27743,7 +27743,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27847,7 +27847,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27951,7 +27951,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28055,7 +28055,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28159,7 +28159,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28263,7 +28263,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28367,7 +28367,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28471,7 +28471,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28575,7 +28575,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28679,7 +28679,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28783,7 +28783,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28887,7 +28887,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28991,7 +28991,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29095,7 +29095,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29199,7 +29199,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29303,7 +29303,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29407,7 +29407,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29511,7 +29511,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29615,7 +29615,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29719,7 +29719,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29823,7 +29823,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29927,7 +29927,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30031,7 +30031,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30135,7 +30135,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30239,7 +30239,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30343,7 +30343,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30447,7 +30447,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30551,7 +30551,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30655,7 +30655,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30759,7 +30759,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30863,7 +30863,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30967,7 +30967,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31071,7 +31071,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31175,7 +31175,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31279,7 +31279,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31383,7 +31383,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31487,7 +31487,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31591,7 +31591,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31695,7 +31695,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31799,7 +31799,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31903,7 +31903,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32007,7 +32007,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32111,7 +32111,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32215,7 +32215,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32319,7 +32319,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32423,7 +32423,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32527,7 +32527,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32631,7 +32631,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32735,7 +32735,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32839,7 +32839,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32943,7 +32943,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33047,7 +33047,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33151,7 +33151,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33255,7 +33255,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33359,7 +33359,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33463,7 +33463,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33567,7 +33567,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33671,7 +33671,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33775,7 +33775,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33879,7 +33879,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33983,7 +33983,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34087,7 +34087,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34191,7 +34191,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34295,7 +34295,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34399,7 +34399,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34503,7 +34503,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34607,7 +34607,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34711,7 +34711,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34815,7 +34815,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34919,7 +34919,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35023,7 +35023,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35127,7 +35127,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35231,7 +35231,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35335,7 +35335,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35439,7 +35439,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35543,7 +35543,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35647,7 +35647,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35751,7 +35751,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35855,7 +35855,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35959,7 +35959,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36063,7 +36063,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36167,7 +36167,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36271,7 +36271,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36375,7 +36375,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36479,7 +36479,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36583,7 +36583,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36687,7 +36687,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36791,7 +36791,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36895,7 +36895,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36999,7 +36999,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37103,7 +37103,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37207,7 +37207,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37311,7 +37311,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37415,7 +37415,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37519,7 +37519,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37623,7 +37623,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37727,7 +37727,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37831,7 +37831,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37935,7 +37935,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38039,7 +38039,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38143,7 +38143,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38247,7 +38247,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38351,7 +38351,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38455,7 +38455,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38559,7 +38559,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38663,7 +38663,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38767,7 +38767,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38871,7 +38871,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38975,7 +38975,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39079,7 +39079,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39183,7 +39183,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39287,7 +39287,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39391,7 +39391,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39495,7 +39495,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39599,7 +39599,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39703,7 +39703,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39807,7 +39807,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39911,7 +39911,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40015,7 +40015,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40119,7 +40119,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40223,7 +40223,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40327,7 +40327,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40431,7 +40431,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40535,7 +40535,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40639,7 +40639,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40743,7 +40743,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40847,7 +40847,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40951,7 +40951,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41055,7 +41055,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41159,7 +41159,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41263,7 +41263,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41367,7 +41367,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41471,7 +41471,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41575,7 +41575,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41679,7 +41679,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41783,7 +41783,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41887,7 +41887,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41991,7 +41991,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42095,7 +42095,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42199,7 +42199,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42303,7 +42303,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42407,7 +42407,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42511,7 +42511,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42615,7 +42615,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42719,7 +42719,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42823,7 +42823,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42927,7 +42927,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43031,7 +43031,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43135,7 +43135,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43239,7 +43239,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43343,7 +43343,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43447,7 +43447,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43551,7 +43551,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43655,7 +43655,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43759,7 +43759,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43863,7 +43863,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43967,7 +43967,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44071,7 +44071,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44175,7 +44175,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44279,7 +44279,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44383,7 +44383,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44487,7 +44487,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44591,7 +44591,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44695,7 +44695,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44799,7 +44799,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44903,7 +44903,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45007,7 +45007,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45111,7 +45111,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45215,7 +45215,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45319,7 +45319,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45423,7 +45423,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45527,7 +45527,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45631,7 +45631,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45735,7 +45735,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45839,7 +45839,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45943,7 +45943,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46047,7 +46047,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46151,7 +46151,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46255,7 +46255,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46359,7 +46359,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46463,7 +46463,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46567,7 +46567,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46671,7 +46671,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46775,7 +46775,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46879,7 +46879,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46983,7 +46983,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47087,7 +47087,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47191,7 +47191,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47295,7 +47295,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47399,7 +47399,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47503,7 +47503,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47607,7 +47607,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47711,7 +47711,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47815,7 +47815,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47919,7 +47919,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48023,7 +48023,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48127,7 +48127,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48231,7 +48231,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48335,7 +48335,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48439,7 +48439,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48543,7 +48543,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48647,7 +48647,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48751,7 +48751,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48855,7 +48855,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48959,7 +48959,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49063,7 +49063,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49167,7 +49167,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49271,7 +49271,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49375,7 +49375,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49479,7 +49479,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49583,7 +49583,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49687,7 +49687,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49791,7 +49791,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49895,7 +49895,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49999,7 +49999,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50103,7 +50103,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50207,7 +50207,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50311,7 +50311,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50415,7 +50415,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50519,7 +50519,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50623,7 +50623,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50727,7 +50727,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50831,7 +50831,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50935,7 +50935,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51039,7 +51039,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51143,7 +51143,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51247,7 +51247,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51351,7 +51351,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51455,7 +51455,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51559,7 +51559,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51663,7 +51663,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51767,7 +51767,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51871,7 +51871,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51975,7 +51975,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52079,7 +52079,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52183,7 +52183,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52287,7 +52287,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52391,7 +52391,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52495,7 +52495,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52599,7 +52599,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52703,7 +52703,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52807,7 +52807,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52911,7 +52911,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53015,7 +53015,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53119,7 +53119,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53223,7 +53223,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53327,7 +53327,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53431,7 +53431,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53535,7 +53535,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53589,7 +53589,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53693,7 +53693,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53797,7 +53797,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53901,7 +53901,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -54005,7 +54005,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54109,7 +54109,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54213,7 +54213,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54317,7 +54317,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54421,7 +54421,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54525,7 +54525,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54629,7 +54629,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54733,7 +54733,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54837,7 +54837,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54941,7 +54941,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55045,7 +55045,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55149,7 +55149,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55253,7 +55253,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55357,7 +55357,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55461,7 +55461,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55565,7 +55565,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55669,7 +55669,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55773,7 +55773,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55877,7 +55877,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55981,7 +55981,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56085,7 +56085,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56189,7 +56189,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56293,7 +56293,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56347,7 +56347,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56451,7 +56451,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56555,7 +56555,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56659,7 +56659,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56763,7 +56763,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56867,7 +56867,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46256.333356481482</v>
+        <v>46257.333391203705</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-25 08:00:01
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16612,7 +16612,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16716,7 +16716,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16820,7 +16820,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16924,7 +16924,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17028,7 +17028,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17132,7 +17132,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17236,7 +17236,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17340,7 +17340,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17444,7 +17444,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17548,7 +17548,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17652,7 +17652,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17756,7 +17756,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17860,7 +17860,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17964,7 +17964,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18068,7 +18068,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18172,7 +18172,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18276,7 +18276,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18380,7 +18380,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18484,7 +18484,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18588,7 +18588,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18692,7 +18692,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18796,7 +18796,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18900,7 +18900,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19004,7 +19004,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19108,7 +19108,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19212,7 +19212,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19316,7 +19316,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19420,7 +19420,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19524,7 +19524,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19628,7 +19628,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19732,7 +19732,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19836,7 +19836,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19940,7 +19940,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20044,7 +20044,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20148,7 +20148,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20252,7 +20252,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20356,7 +20356,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20460,7 +20460,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20564,7 +20564,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20668,7 +20668,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20772,7 +20772,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20876,7 +20876,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20980,7 +20980,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21084,7 +21084,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21188,7 +21188,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21292,7 +21292,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21396,7 +21396,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21500,7 +21500,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21604,7 +21604,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21708,7 +21708,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21812,7 +21812,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21916,7 +21916,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22020,7 +22020,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22124,7 +22124,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22228,7 +22228,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22332,7 +22332,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22436,7 +22436,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22540,7 +22540,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22644,7 +22644,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22748,7 +22748,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22852,7 +22852,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22956,7 +22956,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23060,7 +23060,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23164,7 +23164,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23268,7 +23268,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23372,7 +23372,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23476,7 +23476,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23580,7 +23580,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23684,7 +23684,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23788,7 +23788,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23892,7 +23892,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23996,7 +23996,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24100,7 +24100,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24204,7 +24204,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24308,7 +24308,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24412,7 +24412,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24516,7 +24516,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24620,7 +24620,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24724,7 +24724,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24828,7 +24828,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24932,7 +24932,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25036,7 +25036,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25140,7 +25140,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25244,7 +25244,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25348,7 +25348,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25452,7 +25452,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25556,7 +25556,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25660,7 +25660,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25764,7 +25764,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25868,7 +25868,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25972,7 +25972,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26076,7 +26076,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26180,7 +26180,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26284,7 +26284,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26388,7 +26388,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26492,7 +26492,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26596,7 +26596,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26700,7 +26700,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26804,7 +26804,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26908,7 +26908,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27012,7 +27012,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27116,7 +27116,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27220,7 +27220,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27324,7 +27324,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27428,7 +27428,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27532,7 +27532,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27636,7 +27636,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27740,7 +27740,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27844,7 +27844,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27948,7 +27948,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28052,7 +28052,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28156,7 +28156,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28260,7 +28260,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28364,7 +28364,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28468,7 +28468,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28572,7 +28572,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28676,7 +28676,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28780,7 +28780,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28884,7 +28884,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28988,7 +28988,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29092,7 +29092,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29196,7 +29196,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29300,7 +29300,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29404,7 +29404,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29508,7 +29508,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29612,7 +29612,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29716,7 +29716,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29820,7 +29820,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29924,7 +29924,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30028,7 +30028,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30132,7 +30132,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30236,7 +30236,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30340,7 +30340,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30444,7 +30444,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30548,7 +30548,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30652,7 +30652,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30756,7 +30756,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30860,7 +30860,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30964,7 +30964,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31068,7 +31068,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31172,7 +31172,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31276,7 +31276,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31380,7 +31380,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31484,7 +31484,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31588,7 +31588,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31692,7 +31692,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31796,7 +31796,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31900,7 +31900,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32004,7 +32004,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32108,7 +32108,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32212,7 +32212,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32316,7 +32316,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32420,7 +32420,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32524,7 +32524,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32628,7 +32628,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32732,7 +32732,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32836,7 +32836,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32940,7 +32940,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33044,7 +33044,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33148,7 +33148,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33252,7 +33252,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33356,7 +33356,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33460,7 +33460,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33564,7 +33564,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33668,7 +33668,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33772,7 +33772,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33876,7 +33876,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33980,7 +33980,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34084,7 +34084,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34188,7 +34188,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34292,7 +34292,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34396,7 +34396,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34500,7 +34500,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34604,7 +34604,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34708,7 +34708,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34812,7 +34812,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34916,7 +34916,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35020,7 +35020,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35124,7 +35124,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35228,7 +35228,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35332,7 +35332,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35436,7 +35436,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35540,7 +35540,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35644,7 +35644,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35748,7 +35748,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35852,7 +35852,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35956,7 +35956,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36060,7 +36060,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36164,7 +36164,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36268,7 +36268,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36372,7 +36372,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36476,7 +36476,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36580,7 +36580,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36684,7 +36684,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36788,7 +36788,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36892,7 +36892,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36996,7 +36996,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37100,7 +37100,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37204,7 +37204,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37308,7 +37308,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37412,7 +37412,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37516,7 +37516,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37620,7 +37620,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37724,7 +37724,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37828,7 +37828,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37932,7 +37932,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38036,7 +38036,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38140,7 +38140,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38244,7 +38244,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38348,7 +38348,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38452,7 +38452,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38556,7 +38556,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38660,7 +38660,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38764,7 +38764,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38868,7 +38868,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38972,7 +38972,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39076,7 +39076,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39180,7 +39180,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39284,7 +39284,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39388,7 +39388,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39492,7 +39492,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39596,7 +39596,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39700,7 +39700,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39804,7 +39804,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39908,7 +39908,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40012,7 +40012,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40116,7 +40116,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40220,7 +40220,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40324,7 +40324,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40428,7 +40428,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40532,7 +40532,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40636,7 +40636,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40740,7 +40740,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40844,7 +40844,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40948,7 +40948,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41052,7 +41052,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41156,7 +41156,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41260,7 +41260,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41364,7 +41364,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41468,7 +41468,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41572,7 +41572,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41676,7 +41676,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41780,7 +41780,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41884,7 +41884,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41988,7 +41988,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42092,7 +42092,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42196,7 +42196,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42300,7 +42300,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42404,7 +42404,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42508,7 +42508,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42612,7 +42612,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42716,7 +42716,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42820,7 +42820,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42924,7 +42924,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43028,7 +43028,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43132,7 +43132,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43236,7 +43236,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43340,7 +43340,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43444,7 +43444,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43548,7 +43548,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43652,7 +43652,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43756,7 +43756,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43860,7 +43860,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43964,7 +43964,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44068,7 +44068,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44172,7 +44172,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44276,7 +44276,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44380,7 +44380,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44484,7 +44484,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44588,7 +44588,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44692,7 +44692,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44796,7 +44796,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44900,7 +44900,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45004,7 +45004,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45108,7 +45108,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45212,7 +45212,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45316,7 +45316,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45420,7 +45420,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45524,7 +45524,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45628,7 +45628,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45732,7 +45732,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45836,7 +45836,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45940,7 +45940,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46044,7 +46044,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46148,7 +46148,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46252,7 +46252,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46356,7 +46356,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46460,7 +46460,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46564,7 +46564,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46668,7 +46668,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46772,7 +46772,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46876,7 +46876,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46980,7 +46980,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47084,7 +47084,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47188,7 +47188,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47292,7 +47292,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47396,7 +47396,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47500,7 +47500,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47604,7 +47604,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47708,7 +47708,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47812,7 +47812,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47916,7 +47916,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48020,7 +48020,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48124,7 +48124,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48228,7 +48228,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48332,7 +48332,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48436,7 +48436,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48540,7 +48540,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48644,7 +48644,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48748,7 +48748,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48852,7 +48852,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48956,7 +48956,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49060,7 +49060,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49164,7 +49164,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49268,7 +49268,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49372,7 +49372,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49476,7 +49476,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49580,7 +49580,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49684,7 +49684,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49788,7 +49788,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49892,7 +49892,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49996,7 +49996,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50100,7 +50100,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50204,7 +50204,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50308,7 +50308,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50412,7 +50412,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50516,7 +50516,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50620,7 +50620,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50724,7 +50724,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50828,7 +50828,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50932,7 +50932,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51036,7 +51036,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51140,7 +51140,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51244,7 +51244,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51348,7 +51348,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51452,7 +51452,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51556,7 +51556,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51660,7 +51660,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51764,7 +51764,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51868,7 +51868,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51972,7 +51972,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52076,7 +52076,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52180,7 +52180,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52284,7 +52284,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52388,7 +52388,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52492,7 +52492,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52596,7 +52596,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52700,7 +52700,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52804,7 +52804,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52908,7 +52908,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53012,7 +53012,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53116,7 +53116,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53220,7 +53220,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53324,7 +53324,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53428,7 +53428,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53532,7 +53532,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53586,7 +53586,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53690,7 +53690,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53794,7 +53794,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53898,7 +53898,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -54002,7 +54002,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54106,7 +54106,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54210,7 +54210,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54314,7 +54314,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54418,7 +54418,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54522,7 +54522,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54626,7 +54626,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54730,7 +54730,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54834,7 +54834,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54938,7 +54938,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55042,7 +55042,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55146,7 +55146,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55250,7 +55250,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55354,7 +55354,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55458,7 +55458,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55562,7 +55562,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55666,7 +55666,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55770,7 +55770,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55874,7 +55874,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55978,7 +55978,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56082,7 +56082,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56186,7 +56186,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56290,7 +56290,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56344,7 +56344,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56448,7 +56448,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56552,7 +56552,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56656,7 +56656,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56760,7 +56760,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56864,7 +56864,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46258.715555555558</v>
+        <v>46259.333344907405</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-26 08:00:01
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16624,7 +16624,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16728,7 +16728,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16832,7 +16832,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16936,7 +16936,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17040,7 +17040,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17144,7 +17144,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17248,7 +17248,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17352,7 +17352,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17456,7 +17456,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17560,7 +17560,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17664,7 +17664,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17768,7 +17768,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17872,7 +17872,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17976,7 +17976,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18080,7 +18080,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18184,7 +18184,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18288,7 +18288,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18392,7 +18392,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18496,7 +18496,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18600,7 +18600,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18704,7 +18704,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18808,7 +18808,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18912,7 +18912,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19016,7 +19016,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19120,7 +19120,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19224,7 +19224,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19328,7 +19328,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19432,7 +19432,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19536,7 +19536,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19640,7 +19640,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19744,7 +19744,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19848,7 +19848,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19952,7 +19952,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20056,7 +20056,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20160,7 +20160,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20264,7 +20264,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20368,7 +20368,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20472,7 +20472,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20576,7 +20576,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20680,7 +20680,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20784,7 +20784,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20888,7 +20888,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20992,7 +20992,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21096,7 +21096,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21200,7 +21200,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21304,7 +21304,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21408,7 +21408,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21512,7 +21512,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21616,7 +21616,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21720,7 +21720,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21824,7 +21824,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21928,7 +21928,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22032,7 +22032,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22136,7 +22136,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22240,7 +22240,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22344,7 +22344,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22448,7 +22448,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22552,7 +22552,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22656,7 +22656,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22760,7 +22760,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22864,7 +22864,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22968,7 +22968,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23072,7 +23072,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23176,7 +23176,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23280,7 +23280,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23384,7 +23384,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23488,7 +23488,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23592,7 +23592,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23696,7 +23696,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23800,7 +23800,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23904,7 +23904,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -24008,7 +24008,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24112,7 +24112,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24216,7 +24216,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24320,7 +24320,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24424,7 +24424,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24528,7 +24528,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24632,7 +24632,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24736,7 +24736,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24840,7 +24840,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24944,7 +24944,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25048,7 +25048,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25152,7 +25152,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25256,7 +25256,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25360,7 +25360,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25464,7 +25464,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25568,7 +25568,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25672,7 +25672,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25776,7 +25776,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25880,7 +25880,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25984,7 +25984,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26088,7 +26088,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26192,7 +26192,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26296,7 +26296,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26400,7 +26400,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26504,7 +26504,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26608,7 +26608,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26712,7 +26712,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26816,7 +26816,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26920,7 +26920,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27024,7 +27024,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27128,7 +27128,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27232,7 +27232,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27336,7 +27336,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27440,7 +27440,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27544,7 +27544,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27648,7 +27648,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27752,7 +27752,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27856,7 +27856,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27960,7 +27960,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28064,7 +28064,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28168,7 +28168,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28272,7 +28272,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28376,7 +28376,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28480,7 +28480,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28584,7 +28584,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28688,7 +28688,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28792,7 +28792,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28896,7 +28896,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -29000,7 +29000,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29104,7 +29104,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29208,7 +29208,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29312,7 +29312,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29416,7 +29416,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29520,7 +29520,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29624,7 +29624,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29728,7 +29728,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29832,7 +29832,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29936,7 +29936,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30040,7 +30040,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30144,7 +30144,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30248,7 +30248,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30352,7 +30352,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30456,7 +30456,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30560,7 +30560,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30664,7 +30664,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30768,7 +30768,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30872,7 +30872,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30976,7 +30976,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31080,7 +31080,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31184,7 +31184,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31288,7 +31288,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31392,7 +31392,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31496,7 +31496,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31600,7 +31600,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31704,7 +31704,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31808,7 +31808,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31912,7 +31912,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32016,7 +32016,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32120,7 +32120,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32224,7 +32224,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32328,7 +32328,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32432,7 +32432,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32536,7 +32536,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32640,7 +32640,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32744,7 +32744,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32848,7 +32848,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32952,7 +32952,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33056,7 +33056,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33160,7 +33160,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33264,7 +33264,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33368,7 +33368,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33472,7 +33472,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33576,7 +33576,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33680,7 +33680,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33784,7 +33784,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33888,7 +33888,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33992,7 +33992,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34096,7 +34096,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34200,7 +34200,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34304,7 +34304,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34408,7 +34408,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34512,7 +34512,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34616,7 +34616,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34720,7 +34720,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34824,7 +34824,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34928,7 +34928,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35032,7 +35032,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35136,7 +35136,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35240,7 +35240,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35344,7 +35344,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35448,7 +35448,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35552,7 +35552,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35656,7 +35656,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35760,7 +35760,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35864,7 +35864,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35968,7 +35968,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36072,7 +36072,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36176,7 +36176,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36280,7 +36280,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36384,7 +36384,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36488,7 +36488,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36592,7 +36592,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36696,7 +36696,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36800,7 +36800,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36904,7 +36904,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -37008,7 +37008,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37112,7 +37112,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37216,7 +37216,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37320,7 +37320,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37424,7 +37424,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37528,7 +37528,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37632,7 +37632,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37736,7 +37736,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37840,7 +37840,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37944,7 +37944,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38048,7 +38048,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38152,7 +38152,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38256,7 +38256,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38360,7 +38360,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38464,7 +38464,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38568,7 +38568,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38672,7 +38672,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38776,7 +38776,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38880,7 +38880,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38984,7 +38984,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -38995,7 +38995,7 @@
         <v>2878</v>
       </c>
       <c r="C218" s="2">
-        <v>13886663</v>
+        <v>15541014</v>
       </c>
       <c r="D218" s="1" t="s">
         <v>871</v>
@@ -39088,7 +39088,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39192,7 +39192,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39296,7 +39296,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39400,7 +39400,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39504,7 +39504,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39608,7 +39608,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39712,7 +39712,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39816,7 +39816,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39920,7 +39920,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40024,7 +40024,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40128,7 +40128,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40232,7 +40232,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40336,7 +40336,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40440,7 +40440,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40544,7 +40544,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40648,7 +40648,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40752,7 +40752,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40856,7 +40856,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40960,7 +40960,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41064,7 +41064,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41168,7 +41168,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41272,7 +41272,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41376,7 +41376,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41480,7 +41480,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41584,7 +41584,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41688,7 +41688,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41792,7 +41792,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41896,7 +41896,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -42000,7 +42000,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42104,7 +42104,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42208,7 +42208,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42312,7 +42312,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42416,7 +42416,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42520,7 +42520,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42624,7 +42624,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42728,7 +42728,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42832,7 +42832,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42936,7 +42936,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43040,7 +43040,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43144,7 +43144,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43248,7 +43248,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43352,7 +43352,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43456,7 +43456,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43560,7 +43560,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43664,7 +43664,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43768,7 +43768,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43872,7 +43872,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43976,7 +43976,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44080,7 +44080,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44184,7 +44184,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44288,7 +44288,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44392,7 +44392,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44496,7 +44496,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44600,7 +44600,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44704,7 +44704,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44808,7 +44808,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44912,7 +44912,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45016,7 +45016,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45120,7 +45120,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45224,7 +45224,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45328,7 +45328,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45432,7 +45432,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45536,7 +45536,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45640,7 +45640,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45744,7 +45744,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45848,7 +45848,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45952,7 +45952,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46056,7 +46056,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46160,7 +46160,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46264,7 +46264,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46368,7 +46368,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46472,7 +46472,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46576,7 +46576,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46680,7 +46680,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46784,7 +46784,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46888,7 +46888,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46992,7 +46992,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47096,7 +47096,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47200,7 +47200,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47304,7 +47304,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47408,7 +47408,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47512,7 +47512,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47616,7 +47616,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47720,7 +47720,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47824,7 +47824,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47928,7 +47928,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48032,7 +48032,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48136,7 +48136,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48240,7 +48240,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48344,7 +48344,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48448,7 +48448,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48552,7 +48552,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48656,7 +48656,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48760,7 +48760,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48864,7 +48864,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48968,7 +48968,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49072,7 +49072,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49176,7 +49176,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49280,7 +49280,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49384,7 +49384,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49488,7 +49488,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49592,7 +49592,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49696,7 +49696,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49800,7 +49800,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49904,7 +49904,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -50008,7 +50008,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50112,7 +50112,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50216,7 +50216,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50320,7 +50320,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50424,7 +50424,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50528,7 +50528,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50632,7 +50632,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50736,7 +50736,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50840,7 +50840,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50944,7 +50944,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51048,7 +51048,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51152,7 +51152,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51256,7 +51256,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51360,7 +51360,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51464,7 +51464,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51568,7 +51568,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51672,7 +51672,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51776,7 +51776,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51880,7 +51880,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51984,7 +51984,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52088,7 +52088,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52192,7 +52192,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52296,7 +52296,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52400,7 +52400,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52504,7 +52504,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52608,7 +52608,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52712,7 +52712,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52816,7 +52816,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52920,7 +52920,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53024,7 +53024,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53128,7 +53128,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53232,7 +53232,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53336,7 +53336,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53440,7 +53440,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53544,7 +53544,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53598,7 +53598,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53702,7 +53702,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53806,7 +53806,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53910,7 +53910,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -54014,7 +54014,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54118,7 +54118,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54222,7 +54222,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54326,7 +54326,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54430,7 +54430,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54534,7 +54534,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54638,7 +54638,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54742,7 +54742,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54846,7 +54846,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54950,7 +54950,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55054,7 +55054,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55158,7 +55158,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55262,7 +55262,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55366,7 +55366,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55470,7 +55470,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55574,7 +55574,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55678,7 +55678,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55782,7 +55782,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55886,7 +55886,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55990,7 +55990,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56094,7 +56094,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56198,7 +56198,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56302,7 +56302,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56356,7 +56356,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56460,7 +56460,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56564,7 +56564,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56668,7 +56668,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56772,7 +56772,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56876,7 +56876,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46259.602824074071</v>
+        <v>46260.333344907405</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-26 09:01:39
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16624,7 +16624,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16728,7 +16728,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16832,7 +16832,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16936,7 +16936,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17040,7 +17040,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17144,7 +17144,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17248,7 +17248,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17352,7 +17352,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17456,7 +17456,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17560,7 +17560,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17664,7 +17664,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17768,7 +17768,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17872,7 +17872,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17976,7 +17976,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18080,7 +18080,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18184,7 +18184,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18288,7 +18288,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18392,7 +18392,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18496,7 +18496,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18600,7 +18600,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18704,7 +18704,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18808,7 +18808,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18912,7 +18912,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19016,7 +19016,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19120,7 +19120,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19224,7 +19224,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19328,7 +19328,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19432,7 +19432,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19536,7 +19536,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19640,7 +19640,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19744,7 +19744,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19848,7 +19848,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19952,7 +19952,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20056,7 +20056,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20160,7 +20160,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20264,7 +20264,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20368,7 +20368,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20472,7 +20472,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20576,7 +20576,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20680,7 +20680,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20784,7 +20784,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20888,7 +20888,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20992,7 +20992,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21096,7 +21096,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21200,7 +21200,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21304,7 +21304,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21408,7 +21408,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21512,7 +21512,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21616,7 +21616,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21720,7 +21720,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21824,7 +21824,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21928,7 +21928,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22032,7 +22032,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22136,7 +22136,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22240,7 +22240,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22344,7 +22344,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22448,7 +22448,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22552,7 +22552,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22656,7 +22656,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22760,7 +22760,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22864,7 +22864,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22968,7 +22968,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23072,7 +23072,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23176,7 +23176,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23280,7 +23280,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23384,7 +23384,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23488,7 +23488,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23592,7 +23592,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23696,7 +23696,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23800,7 +23800,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23904,7 +23904,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -24008,7 +24008,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24112,7 +24112,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24216,7 +24216,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24320,7 +24320,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24424,7 +24424,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24528,7 +24528,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24632,7 +24632,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24736,7 +24736,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24840,7 +24840,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24944,7 +24944,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25048,7 +25048,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25152,7 +25152,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25256,7 +25256,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25360,7 +25360,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25464,7 +25464,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25568,7 +25568,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25672,7 +25672,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25776,7 +25776,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25880,7 +25880,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25984,7 +25984,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26088,7 +26088,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26192,7 +26192,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26296,7 +26296,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26400,7 +26400,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26504,7 +26504,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26608,7 +26608,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26712,7 +26712,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26816,7 +26816,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26920,7 +26920,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27024,7 +27024,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27128,7 +27128,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27232,7 +27232,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27336,7 +27336,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27440,7 +27440,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27544,7 +27544,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27648,7 +27648,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27752,7 +27752,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27856,7 +27856,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27960,7 +27960,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28064,7 +28064,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28168,7 +28168,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28272,7 +28272,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28376,7 +28376,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28480,7 +28480,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28584,7 +28584,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28688,7 +28688,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28792,7 +28792,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28896,7 +28896,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -29000,7 +29000,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29104,7 +29104,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29208,7 +29208,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29312,7 +29312,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29416,7 +29416,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29520,7 +29520,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29624,7 +29624,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29728,7 +29728,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29832,7 +29832,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29936,7 +29936,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30040,7 +30040,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30144,7 +30144,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30248,7 +30248,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30352,7 +30352,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30456,7 +30456,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30560,7 +30560,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30664,7 +30664,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30768,7 +30768,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30872,7 +30872,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30976,7 +30976,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31080,7 +31080,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31184,7 +31184,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31288,7 +31288,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31392,7 +31392,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31496,7 +31496,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31600,7 +31600,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31704,7 +31704,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31808,7 +31808,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31912,7 +31912,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32016,7 +32016,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32120,7 +32120,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32224,7 +32224,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32328,7 +32328,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32432,7 +32432,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32536,7 +32536,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32640,7 +32640,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32744,7 +32744,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32848,7 +32848,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32952,7 +32952,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33056,7 +33056,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33160,7 +33160,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33264,7 +33264,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33368,7 +33368,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33472,7 +33472,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33576,7 +33576,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33680,7 +33680,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33784,7 +33784,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33888,7 +33888,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33992,7 +33992,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34096,7 +34096,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34200,7 +34200,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34304,7 +34304,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34408,7 +34408,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34512,7 +34512,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34616,7 +34616,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34720,7 +34720,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34824,7 +34824,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34928,7 +34928,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35032,7 +35032,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35136,7 +35136,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35240,7 +35240,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35344,7 +35344,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35448,7 +35448,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35552,7 +35552,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35656,7 +35656,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35760,7 +35760,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35864,7 +35864,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35968,7 +35968,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36072,7 +36072,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36176,7 +36176,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36280,7 +36280,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36384,7 +36384,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36488,7 +36488,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36592,7 +36592,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36696,7 +36696,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36800,7 +36800,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36904,7 +36904,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -37008,7 +37008,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37112,7 +37112,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37216,7 +37216,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37320,7 +37320,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37424,7 +37424,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37528,7 +37528,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37632,7 +37632,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37736,7 +37736,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37840,7 +37840,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37944,7 +37944,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38048,7 +38048,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38152,7 +38152,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38256,7 +38256,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38360,7 +38360,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38464,7 +38464,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38568,7 +38568,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38672,7 +38672,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38776,7 +38776,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38880,7 +38880,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38984,7 +38984,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39088,7 +39088,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39192,7 +39192,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39296,7 +39296,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39400,7 +39400,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39504,7 +39504,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39608,7 +39608,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39712,7 +39712,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39816,7 +39816,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39920,7 +39920,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40024,7 +40024,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40128,7 +40128,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40232,7 +40232,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40336,7 +40336,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40440,7 +40440,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40544,7 +40544,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40648,7 +40648,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40752,7 +40752,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40856,7 +40856,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40960,7 +40960,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41064,7 +41064,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41168,7 +41168,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41272,7 +41272,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41376,7 +41376,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41480,7 +41480,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41584,7 +41584,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41688,7 +41688,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41792,7 +41792,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41896,7 +41896,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -42000,7 +42000,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42104,7 +42104,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42208,7 +42208,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42312,7 +42312,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42416,7 +42416,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42520,7 +42520,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42624,7 +42624,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42728,7 +42728,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42832,7 +42832,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42936,7 +42936,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43040,7 +43040,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43144,7 +43144,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43248,7 +43248,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43352,7 +43352,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43456,7 +43456,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43560,7 +43560,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43664,7 +43664,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43768,7 +43768,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43872,7 +43872,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43976,7 +43976,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44080,7 +44080,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44184,7 +44184,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44288,7 +44288,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44392,7 +44392,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44496,7 +44496,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44600,7 +44600,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44704,7 +44704,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44808,7 +44808,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44912,7 +44912,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45016,7 +45016,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45120,7 +45120,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45224,7 +45224,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45328,7 +45328,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45432,7 +45432,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45536,7 +45536,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45640,7 +45640,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45744,7 +45744,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45848,7 +45848,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45952,7 +45952,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46056,7 +46056,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46160,7 +46160,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46264,7 +46264,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46368,7 +46368,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46472,7 +46472,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46576,7 +46576,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46680,7 +46680,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46784,7 +46784,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46888,7 +46888,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46992,7 +46992,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47096,7 +47096,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47200,7 +47200,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47304,7 +47304,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47408,7 +47408,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47512,7 +47512,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47616,7 +47616,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47720,7 +47720,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47824,7 +47824,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47928,7 +47928,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48032,7 +48032,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48136,7 +48136,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48240,7 +48240,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48344,7 +48344,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48448,7 +48448,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48552,7 +48552,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48656,7 +48656,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48760,7 +48760,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48864,7 +48864,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48968,7 +48968,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49072,7 +49072,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49176,7 +49176,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49280,7 +49280,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49384,7 +49384,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49488,7 +49488,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49592,7 +49592,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49696,7 +49696,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49800,7 +49800,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49904,7 +49904,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -50008,7 +50008,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50112,7 +50112,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50216,7 +50216,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50320,7 +50320,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50424,7 +50424,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50528,7 +50528,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50632,7 +50632,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50736,7 +50736,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50840,7 +50840,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50944,7 +50944,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51048,7 +51048,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51152,7 +51152,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51256,7 +51256,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51360,7 +51360,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51464,7 +51464,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51568,7 +51568,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51672,7 +51672,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51776,7 +51776,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51880,7 +51880,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51984,7 +51984,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52088,7 +52088,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52192,7 +52192,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52296,7 +52296,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52400,7 +52400,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52504,7 +52504,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52608,7 +52608,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52712,7 +52712,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52816,7 +52816,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52920,7 +52920,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53024,7 +53024,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53128,7 +53128,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53232,7 +53232,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53336,7 +53336,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53440,7 +53440,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53544,7 +53544,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53598,7 +53598,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53702,7 +53702,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53806,7 +53806,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53910,7 +53910,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -54014,7 +54014,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54118,7 +54118,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54222,7 +54222,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54326,7 +54326,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54430,7 +54430,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54534,7 +54534,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54638,7 +54638,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54742,7 +54742,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54846,7 +54846,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54950,7 +54950,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55054,7 +55054,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55158,7 +55158,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55262,7 +55262,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55366,7 +55366,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55470,7 +55470,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55574,7 +55574,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55678,7 +55678,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55782,7 +55782,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55886,7 +55886,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55990,7 +55990,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56094,7 +56094,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56198,7 +56198,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56302,7 +56302,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56356,7 +56356,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56460,7 +56460,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56564,7 +56564,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56668,7 +56668,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56772,7 +56772,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56876,7 +56876,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46260.333344907405</v>
+        <v>46260.376145833332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-26 09:54:04
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16624,7 +16624,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16728,7 +16728,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16832,7 +16832,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16936,7 +16936,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17040,7 +17040,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17144,7 +17144,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17248,7 +17248,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17352,7 +17352,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17456,7 +17456,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17560,7 +17560,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17664,7 +17664,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17768,7 +17768,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17872,7 +17872,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17976,7 +17976,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18080,7 +18080,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18184,7 +18184,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18288,7 +18288,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18392,7 +18392,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18496,7 +18496,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18600,7 +18600,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18704,7 +18704,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18808,7 +18808,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18912,7 +18912,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19016,7 +19016,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19120,7 +19120,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19224,7 +19224,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19328,7 +19328,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19432,7 +19432,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19536,7 +19536,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19640,7 +19640,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19744,7 +19744,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19848,7 +19848,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19952,7 +19952,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20056,7 +20056,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20160,7 +20160,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20264,7 +20264,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20368,7 +20368,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20472,7 +20472,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20576,7 +20576,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20680,7 +20680,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20784,7 +20784,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20888,7 +20888,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20992,7 +20992,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21096,7 +21096,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21200,7 +21200,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21304,7 +21304,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21408,7 +21408,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21512,7 +21512,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21616,7 +21616,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21720,7 +21720,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21824,7 +21824,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21928,7 +21928,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22032,7 +22032,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22136,7 +22136,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22240,7 +22240,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22344,7 +22344,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22448,7 +22448,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22552,7 +22552,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22656,7 +22656,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22760,7 +22760,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22864,7 +22864,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22968,7 +22968,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23072,7 +23072,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23176,7 +23176,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23280,7 +23280,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23384,7 +23384,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23488,7 +23488,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23592,7 +23592,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23696,7 +23696,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23800,7 +23800,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23904,7 +23904,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -24008,7 +24008,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24112,7 +24112,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24216,7 +24216,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24320,7 +24320,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24424,7 +24424,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24528,7 +24528,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24632,7 +24632,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24736,7 +24736,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24840,7 +24840,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24944,7 +24944,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25048,7 +25048,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25152,7 +25152,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25256,7 +25256,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25360,7 +25360,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25464,7 +25464,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25568,7 +25568,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25672,7 +25672,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25776,7 +25776,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25880,7 +25880,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25984,7 +25984,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26088,7 +26088,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26192,7 +26192,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26296,7 +26296,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26400,7 +26400,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26504,7 +26504,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26608,7 +26608,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26712,7 +26712,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26816,7 +26816,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26920,7 +26920,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27024,7 +27024,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27128,7 +27128,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27232,7 +27232,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27336,7 +27336,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27440,7 +27440,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27544,7 +27544,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27648,7 +27648,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27752,7 +27752,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27856,7 +27856,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27960,7 +27960,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28064,7 +28064,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28168,7 +28168,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28272,7 +28272,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28376,7 +28376,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28480,7 +28480,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28584,7 +28584,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28688,7 +28688,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28792,7 +28792,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28896,7 +28896,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -29000,7 +29000,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29104,7 +29104,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29208,7 +29208,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29312,7 +29312,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29416,7 +29416,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29520,7 +29520,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29624,7 +29624,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29728,7 +29728,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29832,7 +29832,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29936,7 +29936,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30040,7 +30040,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30144,7 +30144,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30248,7 +30248,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30352,7 +30352,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30456,7 +30456,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30560,7 +30560,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30664,7 +30664,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30768,7 +30768,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30872,7 +30872,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30976,7 +30976,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31080,7 +31080,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31184,7 +31184,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31288,7 +31288,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31392,7 +31392,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31496,7 +31496,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31600,7 +31600,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31704,7 +31704,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31808,7 +31808,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31912,7 +31912,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32016,7 +32016,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32120,7 +32120,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32224,7 +32224,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32328,7 +32328,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32432,7 +32432,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32536,7 +32536,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32640,7 +32640,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32744,7 +32744,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32848,7 +32848,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32952,7 +32952,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33056,7 +33056,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33160,7 +33160,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33264,7 +33264,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33368,7 +33368,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33472,7 +33472,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33576,7 +33576,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33680,7 +33680,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33784,7 +33784,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33888,7 +33888,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33992,7 +33992,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34096,7 +34096,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34200,7 +34200,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34304,7 +34304,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34408,7 +34408,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34512,7 +34512,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34616,7 +34616,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34720,7 +34720,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34824,7 +34824,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34928,7 +34928,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35032,7 +35032,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35136,7 +35136,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35240,7 +35240,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35344,7 +35344,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35448,7 +35448,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35552,7 +35552,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35656,7 +35656,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35760,7 +35760,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35864,7 +35864,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35968,7 +35968,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36072,7 +36072,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36176,7 +36176,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36280,7 +36280,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36384,7 +36384,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36488,7 +36488,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36592,7 +36592,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36696,7 +36696,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36800,7 +36800,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36904,7 +36904,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -37008,7 +37008,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37112,7 +37112,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37216,7 +37216,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37320,7 +37320,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37424,7 +37424,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37528,7 +37528,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37632,7 +37632,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37736,7 +37736,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37840,7 +37840,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37944,7 +37944,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38048,7 +38048,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38152,7 +38152,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38256,7 +38256,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38360,7 +38360,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38464,7 +38464,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38568,7 +38568,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38672,7 +38672,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38776,7 +38776,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38880,7 +38880,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38984,7 +38984,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39088,7 +39088,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39192,7 +39192,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39296,7 +39296,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39400,7 +39400,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39504,7 +39504,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39608,7 +39608,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39712,7 +39712,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39816,7 +39816,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39920,7 +39920,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40024,7 +40024,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40128,7 +40128,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40232,7 +40232,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40336,7 +40336,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40440,7 +40440,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40544,7 +40544,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40648,7 +40648,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40752,7 +40752,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40856,7 +40856,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40960,7 +40960,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41064,7 +41064,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41168,7 +41168,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41272,7 +41272,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41376,7 +41376,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41480,7 +41480,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41584,7 +41584,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41688,7 +41688,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41792,7 +41792,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41896,7 +41896,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -42000,7 +42000,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42104,7 +42104,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42208,7 +42208,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42312,7 +42312,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42416,7 +42416,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42520,7 +42520,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42624,7 +42624,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42728,7 +42728,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42832,7 +42832,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42936,7 +42936,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43040,7 +43040,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43144,7 +43144,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43248,7 +43248,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43352,7 +43352,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43456,7 +43456,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43560,7 +43560,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43664,7 +43664,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43768,7 +43768,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43872,7 +43872,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43976,7 +43976,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44080,7 +44080,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44184,7 +44184,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44288,7 +44288,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44392,7 +44392,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44496,7 +44496,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44600,7 +44600,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44704,7 +44704,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44808,7 +44808,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44912,7 +44912,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45016,7 +45016,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45120,7 +45120,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45224,7 +45224,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45328,7 +45328,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45432,7 +45432,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45536,7 +45536,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45640,7 +45640,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45744,7 +45744,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45848,7 +45848,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45952,7 +45952,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46056,7 +46056,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46160,7 +46160,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46264,7 +46264,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46368,7 +46368,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46472,7 +46472,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46576,7 +46576,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46680,7 +46680,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46784,7 +46784,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46888,7 +46888,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46992,7 +46992,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47096,7 +47096,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47200,7 +47200,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47304,7 +47304,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47408,7 +47408,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47512,7 +47512,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47616,7 +47616,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47720,7 +47720,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47824,7 +47824,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47928,7 +47928,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48032,7 +48032,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48136,7 +48136,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48240,7 +48240,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48344,7 +48344,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48448,7 +48448,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48552,7 +48552,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48656,7 +48656,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48760,7 +48760,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48864,7 +48864,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48968,7 +48968,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49072,7 +49072,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49176,7 +49176,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49280,7 +49280,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49384,7 +49384,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49488,7 +49488,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49592,7 +49592,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49696,7 +49696,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49800,7 +49800,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49904,7 +49904,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -50008,7 +50008,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50112,7 +50112,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50216,7 +50216,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50320,7 +50320,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50424,7 +50424,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50528,7 +50528,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50632,7 +50632,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50736,7 +50736,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50840,7 +50840,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50944,7 +50944,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51048,7 +51048,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51152,7 +51152,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51256,7 +51256,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51360,7 +51360,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51464,7 +51464,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51568,7 +51568,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51672,7 +51672,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51776,7 +51776,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51880,7 +51880,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51984,7 +51984,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52088,7 +52088,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52192,7 +52192,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52296,7 +52296,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52400,7 +52400,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52504,7 +52504,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52608,7 +52608,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52712,7 +52712,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52816,7 +52816,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52920,7 +52920,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53024,7 +53024,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53128,7 +53128,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53232,7 +53232,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53336,7 +53336,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53440,7 +53440,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53544,7 +53544,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53598,7 +53598,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53702,7 +53702,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53806,7 +53806,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53910,7 +53910,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -54014,7 +54014,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54118,7 +54118,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54222,7 +54222,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54326,7 +54326,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54430,7 +54430,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54534,7 +54534,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54638,7 +54638,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54742,7 +54742,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54846,7 +54846,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54950,7 +54950,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55054,7 +55054,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55158,7 +55158,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55262,7 +55262,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55366,7 +55366,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55470,7 +55470,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55574,7 +55574,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55678,7 +55678,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55782,7 +55782,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55886,7 +55886,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55990,7 +55990,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56094,7 +56094,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56198,7 +56198,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56302,7 +56302,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56356,7 +56356,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56460,7 +56460,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56564,7 +56564,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56668,7 +56668,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56772,7 +56772,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56876,7 +56876,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46260.376145833332</v>
+        <v>46260.412546296298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-26 10:26:23
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16624,7 +16624,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16728,7 +16728,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16832,7 +16832,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16936,7 +16936,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17040,7 +17040,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17144,7 +17144,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17248,7 +17248,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17352,7 +17352,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17456,7 +17456,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17560,7 +17560,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17664,7 +17664,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17768,7 +17768,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17872,7 +17872,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17976,7 +17976,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18080,7 +18080,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18184,7 +18184,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18288,7 +18288,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18392,7 +18392,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18496,7 +18496,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18600,7 +18600,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18704,7 +18704,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18808,7 +18808,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18912,7 +18912,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19016,7 +19016,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19120,7 +19120,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19224,7 +19224,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19328,7 +19328,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19432,7 +19432,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19536,7 +19536,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19640,7 +19640,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19744,7 +19744,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19848,7 +19848,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19952,7 +19952,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20056,7 +20056,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20160,7 +20160,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20264,7 +20264,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20368,7 +20368,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20472,7 +20472,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20576,7 +20576,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20680,7 +20680,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20784,7 +20784,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20888,7 +20888,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20992,7 +20992,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21096,7 +21096,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21200,7 +21200,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21304,7 +21304,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21408,7 +21408,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21512,7 +21512,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21616,7 +21616,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21720,7 +21720,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21824,7 +21824,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21928,7 +21928,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22032,7 +22032,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22136,7 +22136,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22240,7 +22240,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22344,7 +22344,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22448,7 +22448,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22552,7 +22552,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22656,7 +22656,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22760,7 +22760,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22864,7 +22864,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22968,7 +22968,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23072,7 +23072,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23176,7 +23176,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23280,7 +23280,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23384,7 +23384,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23488,7 +23488,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23592,7 +23592,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23696,7 +23696,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23800,7 +23800,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23904,7 +23904,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -24008,7 +24008,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24112,7 +24112,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24216,7 +24216,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24320,7 +24320,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24424,7 +24424,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24528,7 +24528,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24632,7 +24632,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24736,7 +24736,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24840,7 +24840,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24944,7 +24944,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25048,7 +25048,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25152,7 +25152,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25256,7 +25256,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25360,7 +25360,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25464,7 +25464,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25568,7 +25568,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25672,7 +25672,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25776,7 +25776,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25880,7 +25880,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25984,7 +25984,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26088,7 +26088,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26192,7 +26192,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26296,7 +26296,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26400,7 +26400,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26504,7 +26504,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26608,7 +26608,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26712,7 +26712,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26816,7 +26816,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26920,7 +26920,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27024,7 +27024,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27128,7 +27128,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27232,7 +27232,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27336,7 +27336,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27440,7 +27440,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27544,7 +27544,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27648,7 +27648,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27752,7 +27752,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27856,7 +27856,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27960,7 +27960,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28064,7 +28064,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28168,7 +28168,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28272,7 +28272,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28376,7 +28376,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28480,7 +28480,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28584,7 +28584,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28688,7 +28688,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28792,7 +28792,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28896,7 +28896,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -29000,7 +29000,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29104,7 +29104,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29208,7 +29208,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29312,7 +29312,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29416,7 +29416,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29520,7 +29520,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29624,7 +29624,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29728,7 +29728,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29832,7 +29832,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29936,7 +29936,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30040,7 +30040,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30144,7 +30144,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30248,7 +30248,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30352,7 +30352,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30456,7 +30456,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30560,7 +30560,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30664,7 +30664,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30768,7 +30768,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30872,7 +30872,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30976,7 +30976,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31080,7 +31080,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31184,7 +31184,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31288,7 +31288,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31392,7 +31392,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31496,7 +31496,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31600,7 +31600,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31704,7 +31704,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31808,7 +31808,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31912,7 +31912,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32016,7 +32016,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32120,7 +32120,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32224,7 +32224,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32328,7 +32328,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32432,7 +32432,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32536,7 +32536,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32640,7 +32640,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32744,7 +32744,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32848,7 +32848,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32952,7 +32952,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33056,7 +33056,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33160,7 +33160,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33264,7 +33264,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33368,7 +33368,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33472,7 +33472,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33576,7 +33576,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33680,7 +33680,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33784,7 +33784,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33888,7 +33888,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33992,7 +33992,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34096,7 +34096,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34200,7 +34200,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34304,7 +34304,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34408,7 +34408,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34512,7 +34512,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34616,7 +34616,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34720,7 +34720,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34824,7 +34824,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34928,7 +34928,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35032,7 +35032,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35136,7 +35136,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35240,7 +35240,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35344,7 +35344,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35448,7 +35448,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35552,7 +35552,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35656,7 +35656,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35760,7 +35760,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35864,7 +35864,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35968,7 +35968,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36072,7 +36072,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36176,7 +36176,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36280,7 +36280,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36384,7 +36384,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36488,7 +36488,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36592,7 +36592,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36696,7 +36696,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36800,7 +36800,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36904,7 +36904,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -37008,7 +37008,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37112,7 +37112,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37216,7 +37216,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37320,7 +37320,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37424,7 +37424,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37528,7 +37528,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37632,7 +37632,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37736,7 +37736,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37840,7 +37840,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37944,7 +37944,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38048,7 +38048,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38152,7 +38152,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38256,7 +38256,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38360,7 +38360,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38464,7 +38464,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38568,7 +38568,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38672,7 +38672,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38776,7 +38776,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38880,7 +38880,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38984,7 +38984,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39088,7 +39088,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39192,7 +39192,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39296,7 +39296,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39400,7 +39400,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39504,7 +39504,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39608,7 +39608,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39712,7 +39712,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39816,7 +39816,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39920,7 +39920,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40024,7 +40024,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40128,7 +40128,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40232,7 +40232,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40336,7 +40336,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40440,7 +40440,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40544,7 +40544,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40648,7 +40648,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40752,7 +40752,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40856,7 +40856,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40960,7 +40960,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41064,7 +41064,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41168,7 +41168,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41272,7 +41272,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41376,7 +41376,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41480,7 +41480,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41584,7 +41584,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41688,7 +41688,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41792,7 +41792,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41896,7 +41896,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -42000,7 +42000,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42104,7 +42104,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42208,7 +42208,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42312,7 +42312,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42416,7 +42416,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42520,7 +42520,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42624,7 +42624,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42728,7 +42728,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42832,7 +42832,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42936,7 +42936,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43040,7 +43040,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43144,7 +43144,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43248,7 +43248,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43352,7 +43352,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43456,7 +43456,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43560,7 +43560,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43664,7 +43664,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43768,7 +43768,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43872,7 +43872,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43976,7 +43976,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44080,7 +44080,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44184,7 +44184,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44288,7 +44288,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44392,7 +44392,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44496,7 +44496,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44600,7 +44600,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44704,7 +44704,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44808,7 +44808,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44912,7 +44912,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45016,7 +45016,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45120,7 +45120,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45224,7 +45224,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45328,7 +45328,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45432,7 +45432,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45536,7 +45536,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45640,7 +45640,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45744,7 +45744,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45848,7 +45848,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45952,7 +45952,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46056,7 +46056,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46160,7 +46160,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46264,7 +46264,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46368,7 +46368,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46472,7 +46472,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46576,7 +46576,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46680,7 +46680,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46784,7 +46784,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46888,7 +46888,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46992,7 +46992,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47096,7 +47096,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47200,7 +47200,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47304,7 +47304,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47408,7 +47408,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47512,7 +47512,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47616,7 +47616,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47720,7 +47720,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47824,7 +47824,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47928,7 +47928,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48032,7 +48032,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48136,7 +48136,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48240,7 +48240,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48344,7 +48344,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48448,7 +48448,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48552,7 +48552,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48656,7 +48656,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48760,7 +48760,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48864,7 +48864,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48968,7 +48968,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49072,7 +49072,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49176,7 +49176,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49280,7 +49280,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49384,7 +49384,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49488,7 +49488,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49592,7 +49592,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49696,7 +49696,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49800,7 +49800,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49904,7 +49904,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -50008,7 +50008,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50112,7 +50112,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50216,7 +50216,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50320,7 +50320,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50424,7 +50424,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50528,7 +50528,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50632,7 +50632,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50736,7 +50736,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50840,7 +50840,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50944,7 +50944,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51048,7 +51048,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51152,7 +51152,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51256,7 +51256,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51360,7 +51360,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51464,7 +51464,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51568,7 +51568,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51672,7 +51672,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51776,7 +51776,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51880,7 +51880,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51984,7 +51984,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52088,7 +52088,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52192,7 +52192,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52296,7 +52296,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52400,7 +52400,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52504,7 +52504,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52608,7 +52608,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52712,7 +52712,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52816,7 +52816,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52920,7 +52920,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53024,7 +53024,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53128,7 +53128,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53232,7 +53232,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53336,7 +53336,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53440,7 +53440,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53544,7 +53544,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53598,7 +53598,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53702,7 +53702,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53806,7 +53806,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53910,7 +53910,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -54014,7 +54014,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54118,7 +54118,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54222,7 +54222,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54326,7 +54326,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54430,7 +54430,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54534,7 +54534,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54638,7 +54638,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54742,7 +54742,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54846,7 +54846,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54950,7 +54950,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55054,7 +55054,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55158,7 +55158,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55262,7 +55262,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55366,7 +55366,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55470,7 +55470,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55574,7 +55574,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55678,7 +55678,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55782,7 +55782,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55886,7 +55886,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55990,7 +55990,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56094,7 +56094,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56198,7 +56198,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56302,7 +56302,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56356,7 +56356,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56460,7 +56460,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56564,7 +56564,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56668,7 +56668,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56772,7 +56772,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56876,7 +56876,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46260.412546296298</v>
+        <v>46260.434988425928</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-28 08:00:01
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16609,7 +16609,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16713,7 +16713,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16817,7 +16817,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16921,7 +16921,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17025,7 +17025,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17129,7 +17129,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17233,7 +17233,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17337,7 +17337,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17441,7 +17441,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17545,7 +17545,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17649,7 +17649,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17753,7 +17753,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17857,7 +17857,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17961,7 +17961,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18065,7 +18065,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18169,7 +18169,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18273,7 +18273,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18377,7 +18377,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18481,7 +18481,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18585,7 +18585,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18689,7 +18689,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18793,7 +18793,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18897,7 +18897,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19001,7 +19001,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19105,7 +19105,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19209,7 +19209,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19313,7 +19313,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19417,7 +19417,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19521,7 +19521,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19625,7 +19625,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19729,7 +19729,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19833,7 +19833,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19937,7 +19937,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20041,7 +20041,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20145,7 +20145,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20249,7 +20249,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20353,7 +20353,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20457,7 +20457,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20561,7 +20561,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20665,7 +20665,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20769,7 +20769,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20873,7 +20873,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20977,7 +20977,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21081,7 +21081,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21185,7 +21185,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21289,7 +21289,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21393,7 +21393,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21497,7 +21497,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21601,7 +21601,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21705,7 +21705,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21809,7 +21809,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21913,7 +21913,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22017,7 +22017,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22121,7 +22121,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22225,7 +22225,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22329,7 +22329,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22433,7 +22433,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22537,7 +22537,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22641,7 +22641,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22745,7 +22745,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22849,7 +22849,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22953,7 +22953,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23057,7 +23057,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23161,7 +23161,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23265,7 +23265,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23369,7 +23369,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23473,7 +23473,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23577,7 +23577,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23681,7 +23681,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23785,7 +23785,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23889,7 +23889,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23993,7 +23993,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24097,7 +24097,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24201,7 +24201,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24305,7 +24305,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24409,7 +24409,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24513,7 +24513,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24617,7 +24617,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24721,7 +24721,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24825,7 +24825,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24929,7 +24929,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25033,7 +25033,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25137,7 +25137,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25241,7 +25241,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25345,7 +25345,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25449,7 +25449,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25553,7 +25553,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25657,7 +25657,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25761,7 +25761,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25865,7 +25865,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25969,7 +25969,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26073,7 +26073,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26177,7 +26177,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26281,7 +26281,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26385,7 +26385,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26489,7 +26489,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26593,7 +26593,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26697,7 +26697,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26801,7 +26801,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26905,7 +26905,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27009,7 +27009,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27113,7 +27113,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27217,7 +27217,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27321,7 +27321,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27425,7 +27425,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27529,7 +27529,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27633,7 +27633,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27737,7 +27737,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27841,7 +27841,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27945,7 +27945,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28049,7 +28049,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28153,7 +28153,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28257,7 +28257,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28361,7 +28361,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28465,7 +28465,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28569,7 +28569,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28673,7 +28673,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28777,7 +28777,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28881,7 +28881,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28985,7 +28985,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29089,7 +29089,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29193,7 +29193,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29297,7 +29297,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29401,7 +29401,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29505,7 +29505,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29609,7 +29609,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29713,7 +29713,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29817,7 +29817,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29921,7 +29921,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30025,7 +30025,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30129,7 +30129,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30233,7 +30233,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30337,7 +30337,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30441,7 +30441,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30545,7 +30545,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30649,7 +30649,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30753,7 +30753,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30857,7 +30857,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30961,7 +30961,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31065,7 +31065,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31169,7 +31169,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31273,7 +31273,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31377,7 +31377,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31481,7 +31481,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31585,7 +31585,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31689,7 +31689,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31793,7 +31793,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31897,7 +31897,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32001,7 +32001,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32105,7 +32105,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32209,7 +32209,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32313,7 +32313,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32417,7 +32417,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32521,7 +32521,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32625,7 +32625,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32729,7 +32729,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32833,7 +32833,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32937,7 +32937,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33041,7 +33041,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33145,7 +33145,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33249,7 +33249,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33353,7 +33353,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33457,7 +33457,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33561,7 +33561,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33665,7 +33665,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33769,7 +33769,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33873,7 +33873,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33977,7 +33977,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34081,7 +34081,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34185,7 +34185,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34289,7 +34289,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34393,7 +34393,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34497,7 +34497,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34601,7 +34601,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34705,7 +34705,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34809,7 +34809,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34913,7 +34913,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35017,7 +35017,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35121,7 +35121,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35225,7 +35225,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35329,7 +35329,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35433,7 +35433,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35537,7 +35537,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35641,7 +35641,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35745,7 +35745,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35849,7 +35849,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35953,7 +35953,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36057,7 +36057,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36161,7 +36161,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36265,7 +36265,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36369,7 +36369,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36473,7 +36473,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36577,7 +36577,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36681,7 +36681,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36785,7 +36785,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36889,7 +36889,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36993,7 +36993,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37097,7 +37097,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37201,7 +37201,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37305,7 +37305,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37409,7 +37409,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37513,7 +37513,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37617,7 +37617,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37721,7 +37721,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37825,7 +37825,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37929,7 +37929,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38033,7 +38033,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38137,7 +38137,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38241,7 +38241,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38345,7 +38345,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38449,7 +38449,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38553,7 +38553,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38657,7 +38657,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38761,7 +38761,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38865,7 +38865,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38969,7 +38969,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39073,7 +39073,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39177,7 +39177,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39281,7 +39281,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39385,7 +39385,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39489,7 +39489,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39593,7 +39593,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39697,7 +39697,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39801,7 +39801,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39905,7 +39905,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40009,7 +40009,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40113,7 +40113,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40217,7 +40217,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40321,7 +40321,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40425,7 +40425,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40529,7 +40529,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40633,7 +40633,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40737,7 +40737,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40841,7 +40841,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40945,7 +40945,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41049,7 +41049,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41153,7 +41153,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41257,7 +41257,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41361,7 +41361,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41465,7 +41465,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41569,7 +41569,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41673,7 +41673,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41777,7 +41777,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41881,7 +41881,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41985,7 +41985,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42089,7 +42089,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42193,7 +42193,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42297,7 +42297,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42401,7 +42401,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42505,7 +42505,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42609,7 +42609,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42713,7 +42713,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42817,7 +42817,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42921,7 +42921,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43025,7 +43025,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43129,7 +43129,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43233,7 +43233,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43337,7 +43337,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43441,7 +43441,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43545,7 +43545,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43649,7 +43649,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43753,7 +43753,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43857,7 +43857,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43961,7 +43961,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44065,7 +44065,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44169,7 +44169,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44273,7 +44273,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44377,7 +44377,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44481,7 +44481,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44585,7 +44585,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44689,7 +44689,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44793,7 +44793,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44897,7 +44897,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45001,7 +45001,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45105,7 +45105,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45209,7 +45209,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45313,7 +45313,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45417,7 +45417,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45521,7 +45521,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45625,7 +45625,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45729,7 +45729,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45833,7 +45833,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45937,7 +45937,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46041,7 +46041,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46145,7 +46145,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46249,7 +46249,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46353,7 +46353,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46457,7 +46457,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46561,7 +46561,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46665,7 +46665,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46769,7 +46769,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46873,7 +46873,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46977,7 +46977,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47081,7 +47081,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47185,7 +47185,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47289,7 +47289,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47393,7 +47393,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47497,7 +47497,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47601,7 +47601,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47705,7 +47705,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47809,7 +47809,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47913,7 +47913,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48017,7 +48017,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48121,7 +48121,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48225,7 +48225,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48329,7 +48329,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48433,7 +48433,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48537,7 +48537,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48641,7 +48641,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48745,7 +48745,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48849,7 +48849,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48953,7 +48953,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49057,7 +49057,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49161,7 +49161,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49265,7 +49265,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49369,7 +49369,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49473,7 +49473,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49577,7 +49577,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49681,7 +49681,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49785,7 +49785,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49889,7 +49889,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49993,7 +49993,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50097,7 +50097,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50201,7 +50201,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50305,7 +50305,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50409,7 +50409,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50513,7 +50513,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50617,7 +50617,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50721,7 +50721,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50825,7 +50825,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50929,7 +50929,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51033,7 +51033,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51137,7 +51137,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51241,7 +51241,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51345,7 +51345,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51449,7 +51449,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51553,7 +51553,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51657,7 +51657,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51761,7 +51761,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51865,7 +51865,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51969,7 +51969,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52073,7 +52073,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52177,7 +52177,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52281,7 +52281,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52385,7 +52385,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52489,7 +52489,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52593,7 +52593,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52697,7 +52697,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52801,7 +52801,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52905,7 +52905,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53009,7 +53009,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53113,7 +53113,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53217,7 +53217,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53321,7 +53321,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53425,7 +53425,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53529,7 +53529,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53583,7 +53583,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53687,7 +53687,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53791,7 +53791,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53895,7 +53895,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -53999,7 +53999,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54103,7 +54103,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54207,7 +54207,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54311,7 +54311,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54415,7 +54415,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54519,7 +54519,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54623,7 +54623,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54727,7 +54727,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54831,7 +54831,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54935,7 +54935,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55039,7 +55039,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55143,7 +55143,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55247,7 +55247,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55351,7 +55351,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55455,7 +55455,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55559,7 +55559,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55663,7 +55663,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55767,7 +55767,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55871,7 +55871,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55975,7 +55975,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56079,7 +56079,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56183,7 +56183,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56287,7 +56287,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56341,7 +56341,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56445,7 +56445,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56549,7 +56549,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56653,7 +56653,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56757,7 +56757,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56861,7 +56861,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46261.686562499999</v>
+        <v>46262.333344907405</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-29 08:00:01
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16609,7 +16609,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16713,7 +16713,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16817,7 +16817,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16921,7 +16921,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17025,7 +17025,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17129,7 +17129,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17233,7 +17233,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17337,7 +17337,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17441,7 +17441,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17545,7 +17545,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17649,7 +17649,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17753,7 +17753,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17857,7 +17857,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17961,7 +17961,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18065,7 +18065,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18169,7 +18169,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18273,7 +18273,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18377,7 +18377,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18481,7 +18481,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18585,7 +18585,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18689,7 +18689,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18793,7 +18793,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18897,7 +18897,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19001,7 +19001,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19105,7 +19105,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19209,7 +19209,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19313,7 +19313,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19417,7 +19417,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19521,7 +19521,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19625,7 +19625,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19729,7 +19729,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19833,7 +19833,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19937,7 +19937,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20041,7 +20041,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20145,7 +20145,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20249,7 +20249,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20353,7 +20353,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20457,7 +20457,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20561,7 +20561,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20665,7 +20665,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20769,7 +20769,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20873,7 +20873,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20977,7 +20977,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21081,7 +21081,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21185,7 +21185,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21289,7 +21289,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21393,7 +21393,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21497,7 +21497,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21601,7 +21601,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21705,7 +21705,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21809,7 +21809,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21913,7 +21913,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22017,7 +22017,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22121,7 +22121,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22225,7 +22225,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22329,7 +22329,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22433,7 +22433,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22537,7 +22537,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22641,7 +22641,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22745,7 +22745,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22849,7 +22849,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22953,7 +22953,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23057,7 +23057,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23161,7 +23161,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23265,7 +23265,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23369,7 +23369,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23473,7 +23473,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23577,7 +23577,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23681,7 +23681,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23692,7 +23692,7 @@
         <v>1094</v>
       </c>
       <c r="C71" s="4">
-        <v>11243330</v>
+        <v>15931356</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>531</v>
@@ -23785,7 +23785,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23889,7 +23889,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23993,7 +23993,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24097,7 +24097,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24201,7 +24201,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24305,7 +24305,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24409,7 +24409,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24513,7 +24513,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24617,7 +24617,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24721,7 +24721,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24825,7 +24825,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24929,7 +24929,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25033,7 +25033,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25137,7 +25137,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25241,7 +25241,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25345,7 +25345,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25449,7 +25449,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25553,7 +25553,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25657,7 +25657,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25761,7 +25761,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25865,7 +25865,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25969,7 +25969,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26073,7 +26073,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26177,7 +26177,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26281,7 +26281,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26385,7 +26385,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26489,7 +26489,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26593,7 +26593,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26697,7 +26697,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26801,7 +26801,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26905,7 +26905,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27009,7 +27009,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27113,7 +27113,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27217,7 +27217,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27321,7 +27321,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27425,7 +27425,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27529,7 +27529,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27633,7 +27633,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27737,7 +27737,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27841,7 +27841,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27945,7 +27945,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28049,7 +28049,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28153,7 +28153,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28257,7 +28257,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28361,7 +28361,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28465,7 +28465,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28569,7 +28569,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28673,7 +28673,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28777,7 +28777,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28881,7 +28881,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28985,7 +28985,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29089,7 +29089,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29193,7 +29193,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29297,7 +29297,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29401,7 +29401,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29505,7 +29505,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29609,7 +29609,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29713,7 +29713,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29817,7 +29817,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29921,7 +29921,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30025,7 +30025,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30129,7 +30129,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30233,7 +30233,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30337,7 +30337,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30441,7 +30441,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30545,7 +30545,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30649,7 +30649,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30753,7 +30753,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30857,7 +30857,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30961,7 +30961,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31065,7 +31065,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31169,7 +31169,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31273,7 +31273,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31377,7 +31377,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31481,7 +31481,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31585,7 +31585,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31689,7 +31689,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31793,7 +31793,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31897,7 +31897,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32001,7 +32001,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32105,7 +32105,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32209,7 +32209,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32313,7 +32313,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32417,7 +32417,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32521,7 +32521,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32625,7 +32625,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32729,7 +32729,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32833,7 +32833,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32937,7 +32937,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33041,7 +33041,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33145,7 +33145,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33249,7 +33249,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33353,7 +33353,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33457,7 +33457,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33561,7 +33561,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33665,7 +33665,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33769,7 +33769,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33873,7 +33873,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33977,7 +33977,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34081,7 +34081,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34185,7 +34185,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34289,7 +34289,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34393,7 +34393,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34497,7 +34497,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34601,7 +34601,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34705,7 +34705,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34809,7 +34809,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34913,7 +34913,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35017,7 +35017,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35121,7 +35121,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35225,7 +35225,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35329,7 +35329,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35433,7 +35433,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35537,7 +35537,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35641,7 +35641,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35745,7 +35745,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35849,7 +35849,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35953,7 +35953,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36057,7 +36057,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36161,7 +36161,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36265,7 +36265,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36369,7 +36369,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36473,7 +36473,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36577,7 +36577,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36681,7 +36681,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36785,7 +36785,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36889,7 +36889,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36993,7 +36993,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37097,7 +37097,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37201,7 +37201,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37212,7 +37212,7 @@
         <v>2674</v>
       </c>
       <c r="C201" s="4">
-        <v>16656783</v>
+        <v>17705745</v>
       </c>
       <c r="D201" s="3" t="s">
         <v>2675</v>
@@ -37305,7 +37305,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37409,7 +37409,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37513,7 +37513,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37617,7 +37617,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37721,7 +37721,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37825,7 +37825,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37929,7 +37929,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38033,7 +38033,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38137,7 +38137,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38241,7 +38241,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38345,7 +38345,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38449,7 +38449,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38553,7 +38553,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38657,7 +38657,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38761,7 +38761,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38865,7 +38865,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38969,7 +38969,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39073,7 +39073,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39177,7 +39177,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39281,7 +39281,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39385,7 +39385,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39489,7 +39489,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39593,7 +39593,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39697,7 +39697,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39801,7 +39801,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39905,7 +39905,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40009,7 +40009,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40113,7 +40113,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40217,7 +40217,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40321,7 +40321,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40425,7 +40425,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40529,7 +40529,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40633,7 +40633,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40737,7 +40737,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40841,7 +40841,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40945,7 +40945,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41049,7 +41049,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41153,7 +41153,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41257,7 +41257,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41361,7 +41361,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41465,7 +41465,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41569,7 +41569,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41673,7 +41673,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41777,7 +41777,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41881,7 +41881,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41985,7 +41985,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42089,7 +42089,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42193,7 +42193,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42297,7 +42297,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42401,7 +42401,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42505,7 +42505,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42609,7 +42609,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42713,7 +42713,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42817,7 +42817,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42921,7 +42921,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43025,7 +43025,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43129,7 +43129,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43233,7 +43233,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43337,7 +43337,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43441,7 +43441,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43545,7 +43545,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43649,7 +43649,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43753,7 +43753,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43857,7 +43857,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43961,7 +43961,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44065,7 +44065,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44169,7 +44169,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44273,7 +44273,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44377,7 +44377,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44481,7 +44481,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44585,7 +44585,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44689,7 +44689,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44793,7 +44793,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44897,7 +44897,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45001,7 +45001,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45105,7 +45105,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45209,7 +45209,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45313,7 +45313,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45417,7 +45417,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45521,7 +45521,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45625,7 +45625,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45729,7 +45729,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45833,7 +45833,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45937,7 +45937,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46041,7 +46041,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46145,7 +46145,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46249,7 +46249,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46353,7 +46353,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46457,7 +46457,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46561,7 +46561,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46665,7 +46665,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46769,7 +46769,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46873,7 +46873,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46977,7 +46977,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47081,7 +47081,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47185,7 +47185,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47289,7 +47289,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47393,7 +47393,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47497,7 +47497,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47601,7 +47601,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47705,7 +47705,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47809,7 +47809,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47913,7 +47913,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48017,7 +48017,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48121,7 +48121,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48225,7 +48225,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48329,7 +48329,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48433,7 +48433,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48537,7 +48537,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48641,7 +48641,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48745,7 +48745,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48849,7 +48849,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48953,7 +48953,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49057,7 +49057,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49161,7 +49161,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49265,7 +49265,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49369,7 +49369,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49473,7 +49473,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49577,7 +49577,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49588,7 +49588,7 @@
         <v>4105</v>
       </c>
       <c r="C320" s="2">
-        <v>14130699</v>
+        <v>12910405</v>
       </c>
       <c r="D320" s="1" t="s">
         <v>4106</v>
@@ -49681,7 +49681,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49785,7 +49785,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49889,7 +49889,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49993,7 +49993,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50097,7 +50097,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50201,7 +50201,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50305,7 +50305,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50409,7 +50409,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50513,7 +50513,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50617,7 +50617,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50721,7 +50721,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50825,7 +50825,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50929,7 +50929,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51033,7 +51033,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51137,7 +51137,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51241,7 +51241,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51345,7 +51345,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51449,7 +51449,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51553,7 +51553,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51657,7 +51657,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51668,7 +51668,7 @@
         <v>4338</v>
       </c>
       <c r="C340" s="2">
-        <v>17118023</v>
+        <v>10857800</v>
       </c>
       <c r="D340" s="1" t="s">
         <v>3167</v>
@@ -51761,7 +51761,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51865,7 +51865,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51969,7 +51969,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52073,7 +52073,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52177,7 +52177,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52281,7 +52281,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52385,7 +52385,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52489,7 +52489,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52593,7 +52593,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52697,7 +52697,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52801,7 +52801,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52905,7 +52905,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53009,7 +53009,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53113,7 +53113,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53217,7 +53217,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53321,7 +53321,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53425,7 +53425,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53529,7 +53529,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53583,7 +53583,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53687,7 +53687,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53791,7 +53791,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53895,7 +53895,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -53999,7 +53999,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54103,7 +54103,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54207,7 +54207,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54218,7 +54218,7 @@
         <v>4614</v>
       </c>
       <c r="C365" s="4">
-        <v>15757310</v>
+        <v>25495805</v>
       </c>
       <c r="D365" s="3" t="s">
         <v>4615</v>
@@ -54311,7 +54311,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54415,7 +54415,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54519,7 +54519,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54623,7 +54623,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54727,7 +54727,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54831,7 +54831,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54935,7 +54935,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55039,7 +55039,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55143,7 +55143,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55247,7 +55247,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55351,7 +55351,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55455,7 +55455,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55559,7 +55559,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55663,7 +55663,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55767,7 +55767,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55871,7 +55871,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55975,7 +55975,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56079,7 +56079,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56183,7 +56183,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56287,7 +56287,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56341,7 +56341,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56445,7 +56445,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56549,7 +56549,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56653,7 +56653,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56757,7 +56757,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56861,7 +56861,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46262.333344907405</v>
+        <v>46263.333344907405</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-30 08:00:01
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16609,7 +16609,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16713,7 +16713,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16817,7 +16817,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16921,7 +16921,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17025,7 +17025,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17129,7 +17129,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17233,7 +17233,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17337,7 +17337,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17441,7 +17441,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17545,7 +17545,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17649,7 +17649,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17753,7 +17753,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17857,7 +17857,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17961,7 +17961,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18065,7 +18065,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18169,7 +18169,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18273,7 +18273,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18377,7 +18377,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18481,7 +18481,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18585,7 +18585,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18689,7 +18689,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18793,7 +18793,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18897,7 +18897,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19001,7 +19001,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19105,7 +19105,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19209,7 +19209,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19313,7 +19313,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19417,7 +19417,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19521,7 +19521,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19625,7 +19625,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19729,7 +19729,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19833,7 +19833,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19937,7 +19937,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20041,7 +20041,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20145,7 +20145,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20249,7 +20249,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20353,7 +20353,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20457,7 +20457,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20561,7 +20561,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20665,7 +20665,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20769,7 +20769,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20873,7 +20873,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20977,7 +20977,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21081,7 +21081,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21185,7 +21185,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21289,7 +21289,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21393,7 +21393,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21497,7 +21497,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21601,7 +21601,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21705,7 +21705,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21809,7 +21809,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21913,7 +21913,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22017,7 +22017,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22121,7 +22121,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22225,7 +22225,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22329,7 +22329,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22433,7 +22433,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22537,7 +22537,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22641,7 +22641,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22745,7 +22745,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22849,7 +22849,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22953,7 +22953,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23057,7 +23057,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23161,7 +23161,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23265,7 +23265,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23369,7 +23369,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23473,7 +23473,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23577,7 +23577,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23681,7 +23681,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23785,7 +23785,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23889,7 +23889,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23993,7 +23993,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24097,7 +24097,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24201,7 +24201,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24305,7 +24305,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24409,7 +24409,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24513,7 +24513,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24617,7 +24617,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24721,7 +24721,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24825,7 +24825,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24929,7 +24929,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25033,7 +25033,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25137,7 +25137,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25241,7 +25241,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25345,7 +25345,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25449,7 +25449,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25553,7 +25553,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25657,7 +25657,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25761,7 +25761,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25865,7 +25865,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25969,7 +25969,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26073,7 +26073,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26177,7 +26177,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26281,7 +26281,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26385,7 +26385,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26489,7 +26489,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26593,7 +26593,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26697,7 +26697,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26801,7 +26801,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26905,7 +26905,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27009,7 +27009,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27113,7 +27113,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27217,7 +27217,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27321,7 +27321,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27425,7 +27425,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27529,7 +27529,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27633,7 +27633,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27737,7 +27737,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27841,7 +27841,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27945,7 +27945,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28049,7 +28049,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28153,7 +28153,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28257,7 +28257,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28361,7 +28361,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28465,7 +28465,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28569,7 +28569,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28673,7 +28673,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28777,7 +28777,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28881,7 +28881,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28985,7 +28985,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29089,7 +29089,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29193,7 +29193,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29297,7 +29297,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29401,7 +29401,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29505,7 +29505,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29609,7 +29609,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29713,7 +29713,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29817,7 +29817,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29921,7 +29921,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30025,7 +30025,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30129,7 +30129,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30233,7 +30233,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30337,7 +30337,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30441,7 +30441,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30545,7 +30545,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30649,7 +30649,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30753,7 +30753,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30857,7 +30857,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30961,7 +30961,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31065,7 +31065,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31169,7 +31169,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31273,7 +31273,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31377,7 +31377,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31481,7 +31481,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31585,7 +31585,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31689,7 +31689,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31793,7 +31793,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31897,7 +31897,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32001,7 +32001,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32105,7 +32105,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32209,7 +32209,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32313,7 +32313,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32417,7 +32417,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32521,7 +32521,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32625,7 +32625,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32729,7 +32729,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32833,7 +32833,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32937,7 +32937,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33041,7 +33041,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33145,7 +33145,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33249,7 +33249,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33353,7 +33353,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33457,7 +33457,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33561,7 +33561,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33665,7 +33665,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33769,7 +33769,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33873,7 +33873,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33977,7 +33977,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34081,7 +34081,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34185,7 +34185,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34289,7 +34289,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34393,7 +34393,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34497,7 +34497,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34601,7 +34601,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34705,7 +34705,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34809,7 +34809,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34913,7 +34913,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35017,7 +35017,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35121,7 +35121,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35225,7 +35225,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35329,7 +35329,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35433,7 +35433,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35537,7 +35537,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35641,7 +35641,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35745,7 +35745,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35849,7 +35849,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35953,7 +35953,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36057,7 +36057,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36161,7 +36161,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36265,7 +36265,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36369,7 +36369,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36473,7 +36473,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36577,7 +36577,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36681,7 +36681,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36785,7 +36785,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36889,7 +36889,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36993,7 +36993,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37097,7 +37097,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37201,7 +37201,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37305,7 +37305,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37409,7 +37409,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37513,7 +37513,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37617,7 +37617,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37721,7 +37721,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37825,7 +37825,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37929,7 +37929,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38033,7 +38033,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38137,7 +38137,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38241,7 +38241,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38345,7 +38345,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38449,7 +38449,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38553,7 +38553,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38657,7 +38657,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38761,7 +38761,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38865,7 +38865,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38969,7 +38969,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39073,7 +39073,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39177,7 +39177,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39281,7 +39281,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39385,7 +39385,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39489,7 +39489,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39593,7 +39593,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39697,7 +39697,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39801,7 +39801,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39905,7 +39905,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40009,7 +40009,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40113,7 +40113,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40217,7 +40217,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40321,7 +40321,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40425,7 +40425,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40529,7 +40529,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40633,7 +40633,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40737,7 +40737,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40841,7 +40841,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40945,7 +40945,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41049,7 +41049,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41153,7 +41153,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41257,7 +41257,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41361,7 +41361,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41465,7 +41465,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41569,7 +41569,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41673,7 +41673,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41777,7 +41777,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41881,7 +41881,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41985,7 +41985,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42089,7 +42089,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42193,7 +42193,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42297,7 +42297,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42401,7 +42401,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42505,7 +42505,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42609,7 +42609,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42713,7 +42713,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42817,7 +42817,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42921,7 +42921,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43025,7 +43025,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43129,7 +43129,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43233,7 +43233,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43337,7 +43337,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43441,7 +43441,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43545,7 +43545,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43649,7 +43649,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43753,7 +43753,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43857,7 +43857,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43961,7 +43961,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44065,7 +44065,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44169,7 +44169,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44273,7 +44273,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44377,7 +44377,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44481,7 +44481,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44585,7 +44585,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44689,7 +44689,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44793,7 +44793,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44897,7 +44897,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45001,7 +45001,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45105,7 +45105,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45209,7 +45209,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="278" spans="1:34" x14ac:dyDescent="0.25">
@@ -45313,7 +45313,7 @@
         <v>13</v>
       </c>
       <c r="AH278" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="279" spans="1:34" x14ac:dyDescent="0.25">
@@ -45417,7 +45417,7 @@
         <v>13</v>
       </c>
       <c r="AH279" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="280" spans="1:34" x14ac:dyDescent="0.25">
@@ -45521,7 +45521,7 @@
         <v>13</v>
       </c>
       <c r="AH280" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="281" spans="1:34" x14ac:dyDescent="0.25">
@@ -45625,7 +45625,7 @@
         <v>13</v>
       </c>
       <c r="AH281" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="282" spans="1:34" x14ac:dyDescent="0.25">
@@ -45729,7 +45729,7 @@
         <v>13</v>
       </c>
       <c r="AH282" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="283" spans="1:34" x14ac:dyDescent="0.25">
@@ -45833,7 +45833,7 @@
         <v>5</v>
       </c>
       <c r="AH283" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="284" spans="1:34" x14ac:dyDescent="0.25">
@@ -45937,7 +45937,7 @@
         <v>13</v>
       </c>
       <c r="AH284" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="285" spans="1:34" x14ac:dyDescent="0.25">
@@ -46041,7 +46041,7 @@
         <v>13</v>
       </c>
       <c r="AH285" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="286" spans="1:34" x14ac:dyDescent="0.25">
@@ -46145,7 +46145,7 @@
         <v>13</v>
       </c>
       <c r="AH286" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="287" spans="1:34" x14ac:dyDescent="0.25">
@@ -46249,7 +46249,7 @@
         <v>13</v>
       </c>
       <c r="AH287" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="288" spans="1:34" x14ac:dyDescent="0.25">
@@ -46353,7 +46353,7 @@
         <v>13</v>
       </c>
       <c r="AH288" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="289" spans="1:34" x14ac:dyDescent="0.25">
@@ -46457,7 +46457,7 @@
         <v>13</v>
       </c>
       <c r="AH289" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="290" spans="1:34" x14ac:dyDescent="0.25">
@@ -46561,7 +46561,7 @@
         <v>13</v>
       </c>
       <c r="AH290" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="291" spans="1:34" x14ac:dyDescent="0.25">
@@ -46665,7 +46665,7 @@
         <v>13</v>
       </c>
       <c r="AH291" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="292" spans="1:34" x14ac:dyDescent="0.25">
@@ -46769,7 +46769,7 @@
         <v>13</v>
       </c>
       <c r="AH292" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="293" spans="1:34" x14ac:dyDescent="0.25">
@@ -46873,7 +46873,7 @@
         <v>13</v>
       </c>
       <c r="AH293" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="294" spans="1:34" x14ac:dyDescent="0.25">
@@ -46977,7 +46977,7 @@
         <v>13</v>
       </c>
       <c r="AH294" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="295" spans="1:34" x14ac:dyDescent="0.25">
@@ -47081,7 +47081,7 @@
         <v>13</v>
       </c>
       <c r="AH295" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="296" spans="1:34" x14ac:dyDescent="0.25">
@@ -47185,7 +47185,7 @@
         <v>13</v>
       </c>
       <c r="AH296" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="297" spans="1:34" x14ac:dyDescent="0.25">
@@ -47289,7 +47289,7 @@
         <v>13</v>
       </c>
       <c r="AH297" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="298" spans="1:34" x14ac:dyDescent="0.25">
@@ -47393,7 +47393,7 @@
         <v>13</v>
       </c>
       <c r="AH298" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="299" spans="1:34" x14ac:dyDescent="0.25">
@@ -47497,7 +47497,7 @@
         <v>13</v>
       </c>
       <c r="AH299" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="300" spans="1:34" x14ac:dyDescent="0.25">
@@ -47601,7 +47601,7 @@
         <v>13</v>
       </c>
       <c r="AH300" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="301" spans="1:34" x14ac:dyDescent="0.25">
@@ -47705,7 +47705,7 @@
         <v>13</v>
       </c>
       <c r="AH301" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="302" spans="1:34" x14ac:dyDescent="0.25">
@@ -47809,7 +47809,7 @@
         <v>13</v>
       </c>
       <c r="AH302" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="303" spans="1:34" x14ac:dyDescent="0.25">
@@ -47913,7 +47913,7 @@
         <v>13</v>
       </c>
       <c r="AH303" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="304" spans="1:34" x14ac:dyDescent="0.25">
@@ -48017,7 +48017,7 @@
         <v>13</v>
       </c>
       <c r="AH304" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="305" spans="1:34" x14ac:dyDescent="0.25">
@@ -48121,7 +48121,7 @@
         <v>13</v>
       </c>
       <c r="AH305" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="306" spans="1:34" x14ac:dyDescent="0.25">
@@ -48225,7 +48225,7 @@
         <v>13</v>
       </c>
       <c r="AH306" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="307" spans="1:34" x14ac:dyDescent="0.25">
@@ -48329,7 +48329,7 @@
         <v>13</v>
       </c>
       <c r="AH307" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="308" spans="1:34" x14ac:dyDescent="0.25">
@@ -48433,7 +48433,7 @@
         <v>13</v>
       </c>
       <c r="AH308" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="309" spans="1:34" x14ac:dyDescent="0.25">
@@ -48537,7 +48537,7 @@
         <v>13</v>
       </c>
       <c r="AH309" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="310" spans="1:34" x14ac:dyDescent="0.25">
@@ -48641,7 +48641,7 @@
         <v>13</v>
       </c>
       <c r="AH310" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="311" spans="1:34" x14ac:dyDescent="0.25">
@@ -48745,7 +48745,7 @@
         <v>13</v>
       </c>
       <c r="AH311" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="312" spans="1:34" x14ac:dyDescent="0.25">
@@ -48849,7 +48849,7 @@
         <v>13</v>
       </c>
       <c r="AH312" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="313" spans="1:34" x14ac:dyDescent="0.25">
@@ -48953,7 +48953,7 @@
         <v>13</v>
       </c>
       <c r="AH313" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="314" spans="1:34" x14ac:dyDescent="0.25">
@@ -49057,7 +49057,7 @@
         <v>13</v>
       </c>
       <c r="AH314" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="315" spans="1:34" x14ac:dyDescent="0.25">
@@ -49161,7 +49161,7 @@
         <v>13</v>
       </c>
       <c r="AH315" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="316" spans="1:34" x14ac:dyDescent="0.25">
@@ -49265,7 +49265,7 @@
         <v>13</v>
       </c>
       <c r="AH316" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="317" spans="1:34" x14ac:dyDescent="0.25">
@@ -49369,7 +49369,7 @@
         <v>8</v>
       </c>
       <c r="AH317" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="318" spans="1:34" x14ac:dyDescent="0.25">
@@ -49473,7 +49473,7 @@
         <v>13</v>
       </c>
       <c r="AH318" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="319" spans="1:34" x14ac:dyDescent="0.25">
@@ -49577,7 +49577,7 @@
         <v>13</v>
       </c>
       <c r="AH319" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="320" spans="1:34" x14ac:dyDescent="0.25">
@@ -49681,7 +49681,7 @@
         <v>13</v>
       </c>
       <c r="AH320" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="321" spans="1:34" x14ac:dyDescent="0.25">
@@ -49785,7 +49785,7 @@
         <v>13</v>
       </c>
       <c r="AH321" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="322" spans="1:34" x14ac:dyDescent="0.25">
@@ -49889,7 +49889,7 @@
         <v>8</v>
       </c>
       <c r="AH322" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="323" spans="1:34" x14ac:dyDescent="0.25">
@@ -49993,7 +49993,7 @@
         <v>13</v>
       </c>
       <c r="AH323" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="324" spans="1:34" x14ac:dyDescent="0.25">
@@ -50097,7 +50097,7 @@
         <v>5</v>
       </c>
       <c r="AH324" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="325" spans="1:34" x14ac:dyDescent="0.25">
@@ -50201,7 +50201,7 @@
         <v>13</v>
       </c>
       <c r="AH325" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="326" spans="1:34" x14ac:dyDescent="0.25">
@@ -50305,7 +50305,7 @@
         <v>13</v>
       </c>
       <c r="AH326" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="327" spans="1:34" x14ac:dyDescent="0.25">
@@ -50409,7 +50409,7 @@
         <v>13</v>
       </c>
       <c r="AH327" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="328" spans="1:34" x14ac:dyDescent="0.25">
@@ -50513,7 +50513,7 @@
         <v>13</v>
       </c>
       <c r="AH328" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="329" spans="1:34" x14ac:dyDescent="0.25">
@@ -50617,7 +50617,7 @@
         <v>13</v>
       </c>
       <c r="AH329" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="330" spans="1:34" x14ac:dyDescent="0.25">
@@ -50721,7 +50721,7 @@
         <v>13</v>
       </c>
       <c r="AH330" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="331" spans="1:34" x14ac:dyDescent="0.25">
@@ -50825,7 +50825,7 @@
         <v>13</v>
       </c>
       <c r="AH331" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="332" spans="1:34" x14ac:dyDescent="0.25">
@@ -50929,7 +50929,7 @@
         <v>13</v>
       </c>
       <c r="AH332" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="333" spans="1:34" x14ac:dyDescent="0.25">
@@ -51033,7 +51033,7 @@
         <v>13</v>
       </c>
       <c r="AH333" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="334" spans="1:34" x14ac:dyDescent="0.25">
@@ -51137,7 +51137,7 @@
         <v>13</v>
       </c>
       <c r="AH334" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="335" spans="1:34" x14ac:dyDescent="0.25">
@@ -51241,7 +51241,7 @@
         <v>13</v>
       </c>
       <c r="AH335" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="336" spans="1:34" x14ac:dyDescent="0.25">
@@ -51345,7 +51345,7 @@
         <v>10</v>
       </c>
       <c r="AH336" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="337" spans="1:34" x14ac:dyDescent="0.25">
@@ -51449,7 +51449,7 @@
         <v>13</v>
       </c>
       <c r="AH337" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="338" spans="1:34" x14ac:dyDescent="0.25">
@@ -51553,7 +51553,7 @@
         <v>13</v>
       </c>
       <c r="AH338" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="339" spans="1:34" x14ac:dyDescent="0.25">
@@ -51657,7 +51657,7 @@
         <v>13</v>
       </c>
       <c r="AH339" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="340" spans="1:34" x14ac:dyDescent="0.25">
@@ -51761,7 +51761,7 @@
         <v>5</v>
       </c>
       <c r="AH340" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="341" spans="1:34" x14ac:dyDescent="0.25">
@@ -51865,7 +51865,7 @@
         <v>13</v>
       </c>
       <c r="AH341" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="342" spans="1:34" x14ac:dyDescent="0.25">
@@ -51969,7 +51969,7 @@
         <v>13</v>
       </c>
       <c r="AH342" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="343" spans="1:34" x14ac:dyDescent="0.25">
@@ -52073,7 +52073,7 @@
         <v>13</v>
       </c>
       <c r="AH343" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="344" spans="1:34" x14ac:dyDescent="0.25">
@@ -52177,7 +52177,7 @@
         <v>13</v>
       </c>
       <c r="AH344" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="345" spans="1:34" x14ac:dyDescent="0.25">
@@ -52281,7 +52281,7 @@
         <v>13</v>
       </c>
       <c r="AH345" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="346" spans="1:34" x14ac:dyDescent="0.25">
@@ -52385,7 +52385,7 @@
         <v>13</v>
       </c>
       <c r="AH346" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="347" spans="1:34" x14ac:dyDescent="0.25">
@@ -52489,7 +52489,7 @@
         <v>13</v>
       </c>
       <c r="AH347" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="348" spans="1:34" x14ac:dyDescent="0.25">
@@ -52593,7 +52593,7 @@
         <v>13</v>
       </c>
       <c r="AH348" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="349" spans="1:34" x14ac:dyDescent="0.25">
@@ -52697,7 +52697,7 @@
         <v>13</v>
       </c>
       <c r="AH349" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="350" spans="1:34" x14ac:dyDescent="0.25">
@@ -52801,7 +52801,7 @@
         <v>13</v>
       </c>
       <c r="AH350" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="351" spans="1:34" x14ac:dyDescent="0.25">
@@ -52905,7 +52905,7 @@
         <v>13</v>
       </c>
       <c r="AH351" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="352" spans="1:34" x14ac:dyDescent="0.25">
@@ -53009,7 +53009,7 @@
         <v>13</v>
       </c>
       <c r="AH352" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="353" spans="1:34" x14ac:dyDescent="0.25">
@@ -53113,7 +53113,7 @@
         <v>13</v>
       </c>
       <c r="AH353" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="354" spans="1:34" x14ac:dyDescent="0.25">
@@ -53217,7 +53217,7 @@
         <v>13</v>
       </c>
       <c r="AH354" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="355" spans="1:34" x14ac:dyDescent="0.25">
@@ -53321,7 +53321,7 @@
         <v>13</v>
       </c>
       <c r="AH355" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="356" spans="1:34" x14ac:dyDescent="0.25">
@@ -53425,7 +53425,7 @@
         <v>13</v>
       </c>
       <c r="AH356" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="357" spans="1:34" x14ac:dyDescent="0.25">
@@ -53529,7 +53529,7 @@
         <v>13</v>
       </c>
       <c r="AH357" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="358" spans="1:34" x14ac:dyDescent="0.25">
@@ -53583,7 +53583,7 @@
         <v>13</v>
       </c>
       <c r="AH358" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="359" spans="1:34" x14ac:dyDescent="0.25">
@@ -53687,7 +53687,7 @@
         <v>13</v>
       </c>
       <c r="AH359" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="360" spans="1:34" x14ac:dyDescent="0.25">
@@ -53791,7 +53791,7 @@
         <v>13</v>
       </c>
       <c r="AH360" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="361" spans="1:34" x14ac:dyDescent="0.25">
@@ -53895,7 +53895,7 @@
         <v>13</v>
       </c>
       <c r="AH361" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="362" spans="1:34" x14ac:dyDescent="0.25">
@@ -53999,7 +53999,7 @@
         <v>13</v>
       </c>
       <c r="AH362" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="363" spans="1:34" x14ac:dyDescent="0.25">
@@ -54103,7 +54103,7 @@
         <v>13</v>
       </c>
       <c r="AH363" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="364" spans="1:34" x14ac:dyDescent="0.25">
@@ -54207,7 +54207,7 @@
         <v>13</v>
       </c>
       <c r="AH364" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="365" spans="1:34" x14ac:dyDescent="0.25">
@@ -54311,7 +54311,7 @@
         <v>13</v>
       </c>
       <c r="AH365" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="366" spans="1:34" x14ac:dyDescent="0.25">
@@ -54415,7 +54415,7 @@
         <v>13</v>
       </c>
       <c r="AH366" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="367" spans="1:34" x14ac:dyDescent="0.25">
@@ -54519,7 +54519,7 @@
         <v>13</v>
       </c>
       <c r="AH367" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="368" spans="1:34" x14ac:dyDescent="0.25">
@@ -54623,7 +54623,7 @@
         <v>13</v>
       </c>
       <c r="AH368" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="369" spans="1:34" x14ac:dyDescent="0.25">
@@ -54727,7 +54727,7 @@
         <v>13</v>
       </c>
       <c r="AH369" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="370" spans="1:34" x14ac:dyDescent="0.25">
@@ -54831,7 +54831,7 @@
         <v>13</v>
       </c>
       <c r="AH370" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="371" spans="1:34" x14ac:dyDescent="0.25">
@@ -54935,7 +54935,7 @@
         <v>5</v>
       </c>
       <c r="AH371" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="372" spans="1:34" x14ac:dyDescent="0.25">
@@ -55039,7 +55039,7 @@
         <v>13</v>
       </c>
       <c r="AH372" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="373" spans="1:34" x14ac:dyDescent="0.25">
@@ -55143,7 +55143,7 @@
         <v>13</v>
       </c>
       <c r="AH373" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="374" spans="1:34" x14ac:dyDescent="0.25">
@@ -55247,7 +55247,7 @@
         <v>13</v>
       </c>
       <c r="AH374" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="375" spans="1:34" x14ac:dyDescent="0.25">
@@ -55351,7 +55351,7 @@
         <v>13</v>
       </c>
       <c r="AH375" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="376" spans="1:34" x14ac:dyDescent="0.25">
@@ -55455,7 +55455,7 @@
         <v>13</v>
       </c>
       <c r="AH376" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="377" spans="1:34" x14ac:dyDescent="0.25">
@@ -55559,7 +55559,7 @@
         <v>13</v>
       </c>
       <c r="AH377" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="378" spans="1:34" x14ac:dyDescent="0.25">
@@ -55663,7 +55663,7 @@
         <v>13</v>
       </c>
       <c r="AH378" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="379" spans="1:34" x14ac:dyDescent="0.25">
@@ -55767,7 +55767,7 @@
         <v>5</v>
       </c>
       <c r="AH379" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="380" spans="1:34" x14ac:dyDescent="0.25">
@@ -55871,7 +55871,7 @@
         <v>13</v>
       </c>
       <c r="AH380" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="381" spans="1:34" x14ac:dyDescent="0.25">
@@ -55975,7 +55975,7 @@
         <v>13</v>
       </c>
       <c r="AH381" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="382" spans="1:34" x14ac:dyDescent="0.25">
@@ -56079,7 +56079,7 @@
         <v>13</v>
       </c>
       <c r="AH382" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="383" spans="1:34" x14ac:dyDescent="0.25">
@@ -56183,7 +56183,7 @@
         <v>13</v>
       </c>
       <c r="AH383" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="384" spans="1:34" x14ac:dyDescent="0.25">
@@ -56287,7 +56287,7 @@
         <v>13</v>
       </c>
       <c r="AH384" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="385" spans="1:34" x14ac:dyDescent="0.25">
@@ -56341,7 +56341,7 @@
         <v>13</v>
       </c>
       <c r="AH385" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="386" spans="1:34" x14ac:dyDescent="0.25">
@@ -56445,7 +56445,7 @@
         <v>13</v>
       </c>
       <c r="AH386" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="387" spans="1:34" x14ac:dyDescent="0.25">
@@ -56549,7 +56549,7 @@
         <v>13</v>
       </c>
       <c r="AH387" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="388" spans="1:34" x14ac:dyDescent="0.25">
@@ -56653,7 +56653,7 @@
         <v>13</v>
       </c>
       <c r="AH388" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="389" spans="1:34" x14ac:dyDescent="0.25">
@@ -56757,7 +56757,7 @@
         <v>13</v>
       </c>
       <c r="AH389" s="6">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
     <row r="390" spans="1:34" x14ac:dyDescent="0.25">
@@ -56861,7 +56861,7 @@
         <v>13</v>
       </c>
       <c r="AH390" s="5">
-        <v>46263.333344907405</v>
+        <v>46264.333344907405</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática (Datos Provedores.xlsx): 2026-08-31 09:09:37
</commit_message>
<xml_diff>
--- a/Excels Entregable Farmacia/Datos Provedores.xlsx
+++ b/Excels Entregable Farmacia/Datos Provedores.xlsx
@@ -16609,7 +16609,7 @@
         <v>13</v>
       </c>
       <c r="AH2" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -16713,7 +16713,7 @@
         <v>13</v>
       </c>
       <c r="AH3" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -16817,7 +16817,7 @@
         <v>13</v>
       </c>
       <c r="AH4" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -16921,7 +16921,7 @@
         <v>13</v>
       </c>
       <c r="AH5" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -17025,7 +17025,7 @@
         <v>13</v>
       </c>
       <c r="AH6" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -17129,7 +17129,7 @@
         <v>13</v>
       </c>
       <c r="AH7" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -17233,7 +17233,7 @@
         <v>13</v>
       </c>
       <c r="AH8" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -17337,7 +17337,7 @@
         <v>13</v>
       </c>
       <c r="AH9" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -17441,7 +17441,7 @@
         <v>13</v>
       </c>
       <c r="AH10" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -17545,7 +17545,7 @@
         <v>13</v>
       </c>
       <c r="AH11" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
@@ -17649,7 +17649,7 @@
         <v>13</v>
       </c>
       <c r="AH12" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -17753,7 +17753,7 @@
         <v>13</v>
       </c>
       <c r="AH13" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -17857,7 +17857,7 @@
         <v>13</v>
       </c>
       <c r="AH14" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -17961,7 +17961,7 @@
         <v>13</v>
       </c>
       <c r="AH15" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -18065,7 +18065,7 @@
         <v>13</v>
       </c>
       <c r="AH16" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
@@ -18169,7 +18169,7 @@
         <v>13</v>
       </c>
       <c r="AH17" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
@@ -18273,7 +18273,7 @@
         <v>13</v>
       </c>
       <c r="AH18" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
@@ -18377,7 +18377,7 @@
         <v>13</v>
       </c>
       <c r="AH19" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
@@ -18481,7 +18481,7 @@
         <v>13</v>
       </c>
       <c r="AH20" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -18585,7 +18585,7 @@
         <v>13</v>
       </c>
       <c r="AH21" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
@@ -18689,7 +18689,7 @@
         <v>13</v>
       </c>
       <c r="AH22" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
@@ -18793,7 +18793,7 @@
         <v>13</v>
       </c>
       <c r="AH23" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
@@ -18897,7 +18897,7 @@
         <v>13</v>
       </c>
       <c r="AH24" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
@@ -19001,7 +19001,7 @@
         <v>13</v>
       </c>
       <c r="AH25" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
@@ -19105,7 +19105,7 @@
         <v>13</v>
       </c>
       <c r="AH26" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
@@ -19209,7 +19209,7 @@
         <v>13</v>
       </c>
       <c r="AH27" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
@@ -19313,7 +19313,7 @@
         <v>13</v>
       </c>
       <c r="AH28" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
@@ -19417,7 +19417,7 @@
         <v>5</v>
       </c>
       <c r="AH29" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
@@ -19521,7 +19521,7 @@
         <v>13</v>
       </c>
       <c r="AH30" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
@@ -19625,7 +19625,7 @@
         <v>13</v>
       </c>
       <c r="AH31" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
@@ -19729,7 +19729,7 @@
         <v>13</v>
       </c>
       <c r="AH32" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -19833,7 +19833,7 @@
         <v>13</v>
       </c>
       <c r="AH33" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -19937,7 +19937,7 @@
         <v>13</v>
       </c>
       <c r="AH34" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -20041,7 +20041,7 @@
         <v>13</v>
       </c>
       <c r="AH35" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -20145,7 +20145,7 @@
         <v>13</v>
       </c>
       <c r="AH36" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
@@ -20249,7 +20249,7 @@
         <v>13</v>
       </c>
       <c r="AH37" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
@@ -20353,7 +20353,7 @@
         <v>13</v>
       </c>
       <c r="AH38" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
@@ -20457,7 +20457,7 @@
         <v>13</v>
       </c>
       <c r="AH39" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
@@ -20561,7 +20561,7 @@
         <v>13</v>
       </c>
       <c r="AH40" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
@@ -20665,7 +20665,7 @@
         <v>13</v>
       </c>
       <c r="AH41" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
@@ -20769,7 +20769,7 @@
         <v>13</v>
       </c>
       <c r="AH42" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
@@ -20873,7 +20873,7 @@
         <v>13</v>
       </c>
       <c r="AH43" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
@@ -20977,7 +20977,7 @@
         <v>13</v>
       </c>
       <c r="AH44" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
@@ -21081,7 +21081,7 @@
         <v>13</v>
       </c>
       <c r="AH45" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
@@ -21185,7 +21185,7 @@
         <v>13</v>
       </c>
       <c r="AH46" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
@@ -21289,7 +21289,7 @@
         <v>13</v>
       </c>
       <c r="AH47" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
@@ -21393,7 +21393,7 @@
         <v>13</v>
       </c>
       <c r="AH48" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -21497,7 +21497,7 @@
         <v>13</v>
       </c>
       <c r="AH49" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
@@ -21601,7 +21601,7 @@
         <v>13</v>
       </c>
       <c r="AH50" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -21705,7 +21705,7 @@
         <v>6</v>
       </c>
       <c r="AH51" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
@@ -21809,7 +21809,7 @@
         <v>13</v>
       </c>
       <c r="AH52" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
@@ -21913,7 +21913,7 @@
         <v>13</v>
       </c>
       <c r="AH53" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -22017,7 +22017,7 @@
         <v>13</v>
       </c>
       <c r="AH54" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
@@ -22121,7 +22121,7 @@
         <v>13</v>
       </c>
       <c r="AH55" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
@@ -22225,7 +22225,7 @@
         <v>5</v>
       </c>
       <c r="AH56" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
@@ -22329,7 +22329,7 @@
         <v>13</v>
       </c>
       <c r="AH57" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
@@ -22433,7 +22433,7 @@
         <v>13</v>
       </c>
       <c r="AH58" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
@@ -22537,7 +22537,7 @@
         <v>13</v>
       </c>
       <c r="AH59" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
@@ -22641,7 +22641,7 @@
         <v>13</v>
       </c>
       <c r="AH60" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
@@ -22745,7 +22745,7 @@
         <v>13</v>
       </c>
       <c r="AH61" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
@@ -22849,7 +22849,7 @@
         <v>13</v>
       </c>
       <c r="AH62" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
@@ -22953,7 +22953,7 @@
         <v>13</v>
       </c>
       <c r="AH63" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
@@ -23057,7 +23057,7 @@
         <v>13</v>
       </c>
       <c r="AH64" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
@@ -23161,7 +23161,7 @@
         <v>13</v>
       </c>
       <c r="AH65" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
@@ -23265,7 +23265,7 @@
         <v>13</v>
       </c>
       <c r="AH66" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
@@ -23369,7 +23369,7 @@
         <v>13</v>
       </c>
       <c r="AH67" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
@@ -23473,7 +23473,7 @@
         <v>13</v>
       </c>
       <c r="AH68" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
@@ -23577,7 +23577,7 @@
         <v>13</v>
       </c>
       <c r="AH69" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
@@ -23681,7 +23681,7 @@
         <v>13</v>
       </c>
       <c r="AH70" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
@@ -23785,7 +23785,7 @@
         <v>13</v>
       </c>
       <c r="AH71" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
@@ -23889,7 +23889,7 @@
         <v>8</v>
       </c>
       <c r="AH72" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
@@ -23993,7 +23993,7 @@
         <v>5</v>
       </c>
       <c r="AH73" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
@@ -24097,7 +24097,7 @@
         <v>13</v>
       </c>
       <c r="AH74" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
@@ -24201,7 +24201,7 @@
         <v>5</v>
       </c>
       <c r="AH75" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
@@ -24305,7 +24305,7 @@
         <v>13</v>
       </c>
       <c r="AH76" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
@@ -24409,7 +24409,7 @@
         <v>13</v>
       </c>
       <c r="AH77" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="78" spans="1:34" x14ac:dyDescent="0.25">
@@ -24513,7 +24513,7 @@
         <v>9</v>
       </c>
       <c r="AH78" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="79" spans="1:34" x14ac:dyDescent="0.25">
@@ -24617,7 +24617,7 @@
         <v>13</v>
       </c>
       <c r="AH79" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="80" spans="1:34" x14ac:dyDescent="0.25">
@@ -24721,7 +24721,7 @@
         <v>13</v>
       </c>
       <c r="AH80" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
@@ -24825,7 +24825,7 @@
         <v>13</v>
       </c>
       <c r="AH81" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
@@ -24929,7 +24929,7 @@
         <v>13</v>
       </c>
       <c r="AH82" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
@@ -25033,7 +25033,7 @@
         <v>13</v>
       </c>
       <c r="AH83" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
@@ -25137,7 +25137,7 @@
         <v>13</v>
       </c>
       <c r="AH84" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
@@ -25241,7 +25241,7 @@
         <v>13</v>
       </c>
       <c r="AH85" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="86" spans="1:34" x14ac:dyDescent="0.25">
@@ -25345,7 +25345,7 @@
         <v>13</v>
       </c>
       <c r="AH86" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="87" spans="1:34" x14ac:dyDescent="0.25">
@@ -25449,7 +25449,7 @@
         <v>13</v>
       </c>
       <c r="AH87" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="88" spans="1:34" x14ac:dyDescent="0.25">
@@ -25553,7 +25553,7 @@
         <v>13</v>
       </c>
       <c r="AH88" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="89" spans="1:34" x14ac:dyDescent="0.25">
@@ -25657,7 +25657,7 @@
         <v>13</v>
       </c>
       <c r="AH89" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="90" spans="1:34" x14ac:dyDescent="0.25">
@@ -25761,7 +25761,7 @@
         <v>13</v>
       </c>
       <c r="AH90" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="91" spans="1:34" x14ac:dyDescent="0.25">
@@ -25865,7 +25865,7 @@
         <v>13</v>
       </c>
       <c r="AH91" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="92" spans="1:34" x14ac:dyDescent="0.25">
@@ -25969,7 +25969,7 @@
         <v>13</v>
       </c>
       <c r="AH92" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="93" spans="1:34" x14ac:dyDescent="0.25">
@@ -26073,7 +26073,7 @@
         <v>13</v>
       </c>
       <c r="AH93" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="94" spans="1:34" x14ac:dyDescent="0.25">
@@ -26177,7 +26177,7 @@
         <v>13</v>
       </c>
       <c r="AH94" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="95" spans="1:34" x14ac:dyDescent="0.25">
@@ -26281,7 +26281,7 @@
         <v>13</v>
       </c>
       <c r="AH95" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="96" spans="1:34" x14ac:dyDescent="0.25">
@@ -26385,7 +26385,7 @@
         <v>13</v>
       </c>
       <c r="AH96" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
@@ -26489,7 +26489,7 @@
         <v>13</v>
       </c>
       <c r="AH97" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="98" spans="1:34" x14ac:dyDescent="0.25">
@@ -26593,7 +26593,7 @@
         <v>13</v>
       </c>
       <c r="AH98" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="99" spans="1:34" x14ac:dyDescent="0.25">
@@ -26697,7 +26697,7 @@
         <v>13</v>
       </c>
       <c r="AH99" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="100" spans="1:34" x14ac:dyDescent="0.25">
@@ -26801,7 +26801,7 @@
         <v>13</v>
       </c>
       <c r="AH100" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="101" spans="1:34" x14ac:dyDescent="0.25">
@@ -26905,7 +26905,7 @@
         <v>13</v>
       </c>
       <c r="AH101" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="102" spans="1:34" x14ac:dyDescent="0.25">
@@ -27009,7 +27009,7 @@
         <v>13</v>
       </c>
       <c r="AH102" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="103" spans="1:34" x14ac:dyDescent="0.25">
@@ -27113,7 +27113,7 @@
         <v>13</v>
       </c>
       <c r="AH103" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="104" spans="1:34" x14ac:dyDescent="0.25">
@@ -27217,7 +27217,7 @@
         <v>13</v>
       </c>
       <c r="AH104" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="105" spans="1:34" x14ac:dyDescent="0.25">
@@ -27321,7 +27321,7 @@
         <v>13</v>
       </c>
       <c r="AH105" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="106" spans="1:34" x14ac:dyDescent="0.25">
@@ -27425,7 +27425,7 @@
         <v>13</v>
       </c>
       <c r="AH106" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="107" spans="1:34" x14ac:dyDescent="0.25">
@@ -27529,7 +27529,7 @@
         <v>13</v>
       </c>
       <c r="AH107" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="108" spans="1:34" x14ac:dyDescent="0.25">
@@ -27633,7 +27633,7 @@
         <v>13</v>
       </c>
       <c r="AH108" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="109" spans="1:34" x14ac:dyDescent="0.25">
@@ -27737,7 +27737,7 @@
         <v>13</v>
       </c>
       <c r="AH109" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="110" spans="1:34" x14ac:dyDescent="0.25">
@@ -27841,7 +27841,7 @@
         <v>13</v>
       </c>
       <c r="AH110" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="111" spans="1:34" x14ac:dyDescent="0.25">
@@ -27945,7 +27945,7 @@
         <v>13</v>
       </c>
       <c r="AH111" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="112" spans="1:34" x14ac:dyDescent="0.25">
@@ -28049,7 +28049,7 @@
         <v>13</v>
       </c>
       <c r="AH112" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="113" spans="1:34" x14ac:dyDescent="0.25">
@@ -28153,7 +28153,7 @@
         <v>13</v>
       </c>
       <c r="AH113" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="114" spans="1:34" x14ac:dyDescent="0.25">
@@ -28257,7 +28257,7 @@
         <v>13</v>
       </c>
       <c r="AH114" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="115" spans="1:34" x14ac:dyDescent="0.25">
@@ -28361,7 +28361,7 @@
         <v>13</v>
       </c>
       <c r="AH115" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="116" spans="1:34" x14ac:dyDescent="0.25">
@@ -28465,7 +28465,7 @@
         <v>13</v>
       </c>
       <c r="AH116" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="117" spans="1:34" x14ac:dyDescent="0.25">
@@ -28569,7 +28569,7 @@
         <v>5</v>
       </c>
       <c r="AH117" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="118" spans="1:34" x14ac:dyDescent="0.25">
@@ -28673,7 +28673,7 @@
         <v>13</v>
       </c>
       <c r="AH118" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="119" spans="1:34" x14ac:dyDescent="0.25">
@@ -28777,7 +28777,7 @@
         <v>13</v>
       </c>
       <c r="AH119" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="120" spans="1:34" x14ac:dyDescent="0.25">
@@ -28881,7 +28881,7 @@
         <v>13</v>
       </c>
       <c r="AH120" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="121" spans="1:34" x14ac:dyDescent="0.25">
@@ -28985,7 +28985,7 @@
         <v>13</v>
       </c>
       <c r="AH121" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="122" spans="1:34" x14ac:dyDescent="0.25">
@@ -29089,7 +29089,7 @@
         <v>13</v>
       </c>
       <c r="AH122" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="123" spans="1:34" x14ac:dyDescent="0.25">
@@ -29193,7 +29193,7 @@
         <v>13</v>
       </c>
       <c r="AH123" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="124" spans="1:34" x14ac:dyDescent="0.25">
@@ -29297,7 +29297,7 @@
         <v>13</v>
       </c>
       <c r="AH124" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="125" spans="1:34" x14ac:dyDescent="0.25">
@@ -29401,7 +29401,7 @@
         <v>13</v>
       </c>
       <c r="AH125" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="126" spans="1:34" x14ac:dyDescent="0.25">
@@ -29505,7 +29505,7 @@
         <v>13</v>
       </c>
       <c r="AH126" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="127" spans="1:34" x14ac:dyDescent="0.25">
@@ -29609,7 +29609,7 @@
         <v>13</v>
       </c>
       <c r="AH127" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="128" spans="1:34" x14ac:dyDescent="0.25">
@@ -29713,7 +29713,7 @@
         <v>13</v>
       </c>
       <c r="AH128" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="129" spans="1:34" x14ac:dyDescent="0.25">
@@ -29817,7 +29817,7 @@
         <v>13</v>
       </c>
       <c r="AH129" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="130" spans="1:34" x14ac:dyDescent="0.25">
@@ -29921,7 +29921,7 @@
         <v>13</v>
       </c>
       <c r="AH130" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="131" spans="1:34" x14ac:dyDescent="0.25">
@@ -30025,7 +30025,7 @@
         <v>5</v>
       </c>
       <c r="AH131" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="132" spans="1:34" x14ac:dyDescent="0.25">
@@ -30129,7 +30129,7 @@
         <v>5</v>
       </c>
       <c r="AH132" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="133" spans="1:34" x14ac:dyDescent="0.25">
@@ -30233,7 +30233,7 @@
         <v>13</v>
       </c>
       <c r="AH133" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="134" spans="1:34" x14ac:dyDescent="0.25">
@@ -30337,7 +30337,7 @@
         <v>13</v>
       </c>
       <c r="AH134" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="135" spans="1:34" x14ac:dyDescent="0.25">
@@ -30441,7 +30441,7 @@
         <v>13</v>
       </c>
       <c r="AH135" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.25">
@@ -30545,7 +30545,7 @@
         <v>13</v>
       </c>
       <c r="AH136" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="137" spans="1:34" x14ac:dyDescent="0.25">
@@ -30649,7 +30649,7 @@
         <v>13</v>
       </c>
       <c r="AH137" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="138" spans="1:34" x14ac:dyDescent="0.25">
@@ -30753,7 +30753,7 @@
         <v>13</v>
       </c>
       <c r="AH138" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="139" spans="1:34" x14ac:dyDescent="0.25">
@@ -30857,7 +30857,7 @@
         <v>13</v>
       </c>
       <c r="AH139" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="140" spans="1:34" x14ac:dyDescent="0.25">
@@ -30961,7 +30961,7 @@
         <v>13</v>
       </c>
       <c r="AH140" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="141" spans="1:34" x14ac:dyDescent="0.25">
@@ -31065,7 +31065,7 @@
         <v>13</v>
       </c>
       <c r="AH141" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="142" spans="1:34" x14ac:dyDescent="0.25">
@@ -31169,7 +31169,7 @@
         <v>13</v>
       </c>
       <c r="AH142" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="143" spans="1:34" x14ac:dyDescent="0.25">
@@ -31273,7 +31273,7 @@
         <v>13</v>
       </c>
       <c r="AH143" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="144" spans="1:34" x14ac:dyDescent="0.25">
@@ -31377,7 +31377,7 @@
         <v>13</v>
       </c>
       <c r="AH144" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="145" spans="1:34" x14ac:dyDescent="0.25">
@@ -31481,7 +31481,7 @@
         <v>13</v>
       </c>
       <c r="AH145" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="146" spans="1:34" x14ac:dyDescent="0.25">
@@ -31585,7 +31585,7 @@
         <v>13</v>
       </c>
       <c r="AH146" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="147" spans="1:34" x14ac:dyDescent="0.25">
@@ -31689,7 +31689,7 @@
         <v>13</v>
       </c>
       <c r="AH147" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="148" spans="1:34" x14ac:dyDescent="0.25">
@@ -31793,7 +31793,7 @@
         <v>13</v>
       </c>
       <c r="AH148" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="149" spans="1:34" x14ac:dyDescent="0.25">
@@ -31897,7 +31897,7 @@
         <v>13</v>
       </c>
       <c r="AH149" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="150" spans="1:34" x14ac:dyDescent="0.25">
@@ -32001,7 +32001,7 @@
         <v>13</v>
       </c>
       <c r="AH150" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="151" spans="1:34" x14ac:dyDescent="0.25">
@@ -32105,7 +32105,7 @@
         <v>5</v>
       </c>
       <c r="AH151" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="152" spans="1:34" x14ac:dyDescent="0.25">
@@ -32209,7 +32209,7 @@
         <v>13</v>
       </c>
       <c r="AH152" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="153" spans="1:34" x14ac:dyDescent="0.25">
@@ -32313,7 +32313,7 @@
         <v>13</v>
       </c>
       <c r="AH153" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="154" spans="1:34" x14ac:dyDescent="0.25">
@@ -32417,7 +32417,7 @@
         <v>13</v>
       </c>
       <c r="AH154" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="155" spans="1:34" x14ac:dyDescent="0.25">
@@ -32521,7 +32521,7 @@
         <v>13</v>
       </c>
       <c r="AH155" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="156" spans="1:34" x14ac:dyDescent="0.25">
@@ -32625,7 +32625,7 @@
         <v>13</v>
       </c>
       <c r="AH156" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="157" spans="1:34" x14ac:dyDescent="0.25">
@@ -32729,7 +32729,7 @@
         <v>13</v>
       </c>
       <c r="AH157" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="158" spans="1:34" x14ac:dyDescent="0.25">
@@ -32833,7 +32833,7 @@
         <v>13</v>
       </c>
       <c r="AH158" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="159" spans="1:34" x14ac:dyDescent="0.25">
@@ -32937,7 +32937,7 @@
         <v>13</v>
       </c>
       <c r="AH159" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="160" spans="1:34" x14ac:dyDescent="0.25">
@@ -33041,7 +33041,7 @@
         <v>13</v>
       </c>
       <c r="AH160" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="161" spans="1:34" x14ac:dyDescent="0.25">
@@ -33145,7 +33145,7 @@
         <v>13</v>
       </c>
       <c r="AH161" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="162" spans="1:34" x14ac:dyDescent="0.25">
@@ -33249,7 +33249,7 @@
         <v>13</v>
       </c>
       <c r="AH162" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="163" spans="1:34" x14ac:dyDescent="0.25">
@@ -33353,7 +33353,7 @@
         <v>5</v>
       </c>
       <c r="AH163" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="164" spans="1:34" x14ac:dyDescent="0.25">
@@ -33457,7 +33457,7 @@
         <v>13</v>
       </c>
       <c r="AH164" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="165" spans="1:34" x14ac:dyDescent="0.25">
@@ -33561,7 +33561,7 @@
         <v>13</v>
       </c>
       <c r="AH165" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="166" spans="1:34" x14ac:dyDescent="0.25">
@@ -33665,7 +33665,7 @@
         <v>13</v>
       </c>
       <c r="AH166" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="167" spans="1:34" x14ac:dyDescent="0.25">
@@ -33769,7 +33769,7 @@
         <v>13</v>
       </c>
       <c r="AH167" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="168" spans="1:34" x14ac:dyDescent="0.25">
@@ -33873,7 +33873,7 @@
         <v>13</v>
       </c>
       <c r="AH168" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="169" spans="1:34" x14ac:dyDescent="0.25">
@@ -33977,7 +33977,7 @@
         <v>13</v>
       </c>
       <c r="AH169" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="170" spans="1:34" x14ac:dyDescent="0.25">
@@ -34081,7 +34081,7 @@
         <v>13</v>
       </c>
       <c r="AH170" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="171" spans="1:34" x14ac:dyDescent="0.25">
@@ -34185,7 +34185,7 @@
         <v>13</v>
       </c>
       <c r="AH171" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="172" spans="1:34" x14ac:dyDescent="0.25">
@@ -34289,7 +34289,7 @@
         <v>13</v>
       </c>
       <c r="AH172" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="173" spans="1:34" x14ac:dyDescent="0.25">
@@ -34393,7 +34393,7 @@
         <v>13</v>
       </c>
       <c r="AH173" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="174" spans="1:34" x14ac:dyDescent="0.25">
@@ -34497,7 +34497,7 @@
         <v>13</v>
       </c>
       <c r="AH174" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="175" spans="1:34" x14ac:dyDescent="0.25">
@@ -34601,7 +34601,7 @@
         <v>13</v>
       </c>
       <c r="AH175" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="176" spans="1:34" x14ac:dyDescent="0.25">
@@ -34705,7 +34705,7 @@
         <v>13</v>
       </c>
       <c r="AH176" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="177" spans="1:34" x14ac:dyDescent="0.25">
@@ -34809,7 +34809,7 @@
         <v>13</v>
       </c>
       <c r="AH177" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="178" spans="1:34" x14ac:dyDescent="0.25">
@@ -34913,7 +34913,7 @@
         <v>13</v>
       </c>
       <c r="AH178" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="179" spans="1:34" x14ac:dyDescent="0.25">
@@ -35017,7 +35017,7 @@
         <v>13</v>
       </c>
       <c r="AH179" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="180" spans="1:34" x14ac:dyDescent="0.25">
@@ -35121,7 +35121,7 @@
         <v>13</v>
       </c>
       <c r="AH180" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="181" spans="1:34" x14ac:dyDescent="0.25">
@@ -35225,7 +35225,7 @@
         <v>13</v>
       </c>
       <c r="AH181" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="182" spans="1:34" x14ac:dyDescent="0.25">
@@ -35329,7 +35329,7 @@
         <v>6</v>
       </c>
       <c r="AH182" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="183" spans="1:34" x14ac:dyDescent="0.25">
@@ -35433,7 +35433,7 @@
         <v>13</v>
       </c>
       <c r="AH183" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="184" spans="1:34" x14ac:dyDescent="0.25">
@@ -35537,7 +35537,7 @@
         <v>13</v>
       </c>
       <c r="AH184" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="185" spans="1:34" x14ac:dyDescent="0.25">
@@ -35641,7 +35641,7 @@
         <v>13</v>
       </c>
       <c r="AH185" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="186" spans="1:34" x14ac:dyDescent="0.25">
@@ -35745,7 +35745,7 @@
         <v>13</v>
       </c>
       <c r="AH186" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="187" spans="1:34" x14ac:dyDescent="0.25">
@@ -35849,7 +35849,7 @@
         <v>13</v>
       </c>
       <c r="AH187" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="188" spans="1:34" x14ac:dyDescent="0.25">
@@ -35953,7 +35953,7 @@
         <v>5</v>
       </c>
       <c r="AH188" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="189" spans="1:34" x14ac:dyDescent="0.25">
@@ -36057,7 +36057,7 @@
         <v>13</v>
       </c>
       <c r="AH189" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="190" spans="1:34" x14ac:dyDescent="0.25">
@@ -36161,7 +36161,7 @@
         <v>13</v>
       </c>
       <c r="AH190" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="191" spans="1:34" x14ac:dyDescent="0.25">
@@ -36265,7 +36265,7 @@
         <v>13</v>
       </c>
       <c r="AH191" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="192" spans="1:34" x14ac:dyDescent="0.25">
@@ -36369,7 +36369,7 @@
         <v>7</v>
       </c>
       <c r="AH192" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="193" spans="1:34" x14ac:dyDescent="0.25">
@@ -36473,7 +36473,7 @@
         <v>13</v>
       </c>
       <c r="AH193" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="194" spans="1:34" x14ac:dyDescent="0.25">
@@ -36577,7 +36577,7 @@
         <v>13</v>
       </c>
       <c r="AH194" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="195" spans="1:34" x14ac:dyDescent="0.25">
@@ -36681,7 +36681,7 @@
         <v>13</v>
       </c>
       <c r="AH195" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="196" spans="1:34" x14ac:dyDescent="0.25">
@@ -36785,7 +36785,7 @@
         <v>13</v>
       </c>
       <c r="AH196" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="197" spans="1:34" x14ac:dyDescent="0.25">
@@ -36889,7 +36889,7 @@
         <v>13</v>
       </c>
       <c r="AH197" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="198" spans="1:34" x14ac:dyDescent="0.25">
@@ -36993,7 +36993,7 @@
         <v>13</v>
       </c>
       <c r="AH198" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="199" spans="1:34" x14ac:dyDescent="0.25">
@@ -37097,7 +37097,7 @@
         <v>13</v>
       </c>
       <c r="AH199" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="200" spans="1:34" x14ac:dyDescent="0.25">
@@ -37201,7 +37201,7 @@
         <v>13</v>
       </c>
       <c r="AH200" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="201" spans="1:34" x14ac:dyDescent="0.25">
@@ -37305,7 +37305,7 @@
         <v>13</v>
       </c>
       <c r="AH201" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="202" spans="1:34" x14ac:dyDescent="0.25">
@@ -37409,7 +37409,7 @@
         <v>5</v>
       </c>
       <c r="AH202" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="203" spans="1:34" x14ac:dyDescent="0.25">
@@ -37513,7 +37513,7 @@
         <v>13</v>
       </c>
       <c r="AH203" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="204" spans="1:34" x14ac:dyDescent="0.25">
@@ -37617,7 +37617,7 @@
         <v>13</v>
       </c>
       <c r="AH204" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="205" spans="1:34" x14ac:dyDescent="0.25">
@@ -37721,7 +37721,7 @@
         <v>13</v>
       </c>
       <c r="AH205" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="206" spans="1:34" x14ac:dyDescent="0.25">
@@ -37825,7 +37825,7 @@
         <v>13</v>
       </c>
       <c r="AH206" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="207" spans="1:34" x14ac:dyDescent="0.25">
@@ -37929,7 +37929,7 @@
         <v>13</v>
       </c>
       <c r="AH207" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="208" spans="1:34" x14ac:dyDescent="0.25">
@@ -38033,7 +38033,7 @@
         <v>13</v>
       </c>
       <c r="AH208" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="209" spans="1:34" x14ac:dyDescent="0.25">
@@ -38137,7 +38137,7 @@
         <v>13</v>
       </c>
       <c r="AH209" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="210" spans="1:34" x14ac:dyDescent="0.25">
@@ -38241,7 +38241,7 @@
         <v>10</v>
       </c>
       <c r="AH210" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="211" spans="1:34" x14ac:dyDescent="0.25">
@@ -38345,7 +38345,7 @@
         <v>5</v>
       </c>
       <c r="AH211" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="212" spans="1:34" x14ac:dyDescent="0.25">
@@ -38449,7 +38449,7 @@
         <v>13</v>
       </c>
       <c r="AH212" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="213" spans="1:34" x14ac:dyDescent="0.25">
@@ -38553,7 +38553,7 @@
         <v>13</v>
       </c>
       <c r="AH213" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="214" spans="1:34" x14ac:dyDescent="0.25">
@@ -38657,7 +38657,7 @@
         <v>13</v>
       </c>
       <c r="AH214" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="215" spans="1:34" x14ac:dyDescent="0.25">
@@ -38761,7 +38761,7 @@
         <v>13</v>
       </c>
       <c r="AH215" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="216" spans="1:34" x14ac:dyDescent="0.25">
@@ -38865,7 +38865,7 @@
         <v>13</v>
       </c>
       <c r="AH216" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="217" spans="1:34" x14ac:dyDescent="0.25">
@@ -38969,7 +38969,7 @@
         <v>6</v>
       </c>
       <c r="AH217" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="218" spans="1:34" x14ac:dyDescent="0.25">
@@ -39073,7 +39073,7 @@
         <v>13</v>
       </c>
       <c r="AH218" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="219" spans="1:34" x14ac:dyDescent="0.25">
@@ -39177,7 +39177,7 @@
         <v>13</v>
       </c>
       <c r="AH219" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="220" spans="1:34" x14ac:dyDescent="0.25">
@@ -39281,7 +39281,7 @@
         <v>5</v>
       </c>
       <c r="AH220" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="221" spans="1:34" x14ac:dyDescent="0.25">
@@ -39385,7 +39385,7 @@
         <v>13</v>
       </c>
       <c r="AH221" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="222" spans="1:34" x14ac:dyDescent="0.25">
@@ -39489,7 +39489,7 @@
         <v>13</v>
       </c>
       <c r="AH222" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="223" spans="1:34" x14ac:dyDescent="0.25">
@@ -39593,7 +39593,7 @@
         <v>13</v>
       </c>
       <c r="AH223" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="224" spans="1:34" x14ac:dyDescent="0.25">
@@ -39697,7 +39697,7 @@
         <v>13</v>
       </c>
       <c r="AH224" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="225" spans="1:34" x14ac:dyDescent="0.25">
@@ -39801,7 +39801,7 @@
         <v>13</v>
       </c>
       <c r="AH225" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="226" spans="1:34" x14ac:dyDescent="0.25">
@@ -39905,7 +39905,7 @@
         <v>13</v>
       </c>
       <c r="AH226" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="227" spans="1:34" x14ac:dyDescent="0.25">
@@ -40009,7 +40009,7 @@
         <v>13</v>
       </c>
       <c r="AH227" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="228" spans="1:34" x14ac:dyDescent="0.25">
@@ -40113,7 +40113,7 @@
         <v>13</v>
       </c>
       <c r="AH228" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="229" spans="1:34" x14ac:dyDescent="0.25">
@@ -40217,7 +40217,7 @@
         <v>13</v>
       </c>
       <c r="AH229" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="230" spans="1:34" x14ac:dyDescent="0.25">
@@ -40321,7 +40321,7 @@
         <v>13</v>
       </c>
       <c r="AH230" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="231" spans="1:34" x14ac:dyDescent="0.25">
@@ -40425,7 +40425,7 @@
         <v>13</v>
       </c>
       <c r="AH231" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="232" spans="1:34" x14ac:dyDescent="0.25">
@@ -40529,7 +40529,7 @@
         <v>13</v>
       </c>
       <c r="AH232" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="233" spans="1:34" x14ac:dyDescent="0.25">
@@ -40633,7 +40633,7 @@
         <v>13</v>
       </c>
       <c r="AH233" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="234" spans="1:34" x14ac:dyDescent="0.25">
@@ -40737,7 +40737,7 @@
         <v>13</v>
       </c>
       <c r="AH234" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="235" spans="1:34" x14ac:dyDescent="0.25">
@@ -40841,7 +40841,7 @@
         <v>13</v>
       </c>
       <c r="AH235" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="236" spans="1:34" x14ac:dyDescent="0.25">
@@ -40945,7 +40945,7 @@
         <v>13</v>
       </c>
       <c r="AH236" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="237" spans="1:34" x14ac:dyDescent="0.25">
@@ -41049,7 +41049,7 @@
         <v>13</v>
       </c>
       <c r="AH237" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="238" spans="1:34" x14ac:dyDescent="0.25">
@@ -41153,7 +41153,7 @@
         <v>13</v>
       </c>
       <c r="AH238" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="239" spans="1:34" x14ac:dyDescent="0.25">
@@ -41257,7 +41257,7 @@
         <v>13</v>
       </c>
       <c r="AH239" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="240" spans="1:34" x14ac:dyDescent="0.25">
@@ -41361,7 +41361,7 @@
         <v>13</v>
       </c>
       <c r="AH240" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="241" spans="1:34" x14ac:dyDescent="0.25">
@@ -41465,7 +41465,7 @@
         <v>13</v>
       </c>
       <c r="AH241" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="242" spans="1:34" x14ac:dyDescent="0.25">
@@ -41569,7 +41569,7 @@
         <v>5</v>
       </c>
       <c r="AH242" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="243" spans="1:34" x14ac:dyDescent="0.25">
@@ -41673,7 +41673,7 @@
         <v>13</v>
       </c>
       <c r="AH243" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="244" spans="1:34" x14ac:dyDescent="0.25">
@@ -41777,7 +41777,7 @@
         <v>13</v>
       </c>
       <c r="AH244" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="245" spans="1:34" x14ac:dyDescent="0.25">
@@ -41881,7 +41881,7 @@
         <v>13</v>
       </c>
       <c r="AH245" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="246" spans="1:34" x14ac:dyDescent="0.25">
@@ -41985,7 +41985,7 @@
         <v>13</v>
       </c>
       <c r="AH246" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="247" spans="1:34" x14ac:dyDescent="0.25">
@@ -42089,7 +42089,7 @@
         <v>13</v>
       </c>
       <c r="AH247" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="248" spans="1:34" x14ac:dyDescent="0.25">
@@ -42193,7 +42193,7 @@
         <v>13</v>
       </c>
       <c r="AH248" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="249" spans="1:34" x14ac:dyDescent="0.25">
@@ -42297,7 +42297,7 @@
         <v>13</v>
       </c>
       <c r="AH249" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="250" spans="1:34" x14ac:dyDescent="0.25">
@@ -42401,7 +42401,7 @@
         <v>13</v>
       </c>
       <c r="AH250" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="251" spans="1:34" x14ac:dyDescent="0.25">
@@ -42505,7 +42505,7 @@
         <v>13</v>
       </c>
       <c r="AH251" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="252" spans="1:34" x14ac:dyDescent="0.25">
@@ -42609,7 +42609,7 @@
         <v>13</v>
       </c>
       <c r="AH252" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="253" spans="1:34" x14ac:dyDescent="0.25">
@@ -42713,7 +42713,7 @@
         <v>13</v>
       </c>
       <c r="AH253" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="254" spans="1:34" x14ac:dyDescent="0.25">
@@ -42817,7 +42817,7 @@
         <v>13</v>
       </c>
       <c r="AH254" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="255" spans="1:34" x14ac:dyDescent="0.25">
@@ -42921,7 +42921,7 @@
         <v>13</v>
       </c>
       <c r="AH255" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="256" spans="1:34" x14ac:dyDescent="0.25">
@@ -43025,7 +43025,7 @@
         <v>13</v>
       </c>
       <c r="AH256" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="257" spans="1:34" x14ac:dyDescent="0.25">
@@ -43129,7 +43129,7 @@
         <v>13</v>
       </c>
       <c r="AH257" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="258" spans="1:34" x14ac:dyDescent="0.25">
@@ -43233,7 +43233,7 @@
         <v>13</v>
       </c>
       <c r="AH258" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="259" spans="1:34" x14ac:dyDescent="0.25">
@@ -43337,7 +43337,7 @@
         <v>13</v>
       </c>
       <c r="AH259" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="260" spans="1:34" x14ac:dyDescent="0.25">
@@ -43441,7 +43441,7 @@
         <v>13</v>
       </c>
       <c r="AH260" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="261" spans="1:34" x14ac:dyDescent="0.25">
@@ -43545,7 +43545,7 @@
         <v>13</v>
       </c>
       <c r="AH261" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="262" spans="1:34" x14ac:dyDescent="0.25">
@@ -43649,7 +43649,7 @@
         <v>13</v>
       </c>
       <c r="AH262" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="263" spans="1:34" x14ac:dyDescent="0.25">
@@ -43753,7 +43753,7 @@
         <v>13</v>
       </c>
       <c r="AH263" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="264" spans="1:34" x14ac:dyDescent="0.25">
@@ -43857,7 +43857,7 @@
         <v>13</v>
       </c>
       <c r="AH264" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="265" spans="1:34" x14ac:dyDescent="0.25">
@@ -43961,7 +43961,7 @@
         <v>13</v>
       </c>
       <c r="AH265" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="266" spans="1:34" x14ac:dyDescent="0.25">
@@ -44065,7 +44065,7 @@
         <v>13</v>
       </c>
       <c r="AH266" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="267" spans="1:34" x14ac:dyDescent="0.25">
@@ -44169,7 +44169,7 @@
         <v>13</v>
       </c>
       <c r="AH267" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="268" spans="1:34" x14ac:dyDescent="0.25">
@@ -44273,7 +44273,7 @@
         <v>13</v>
       </c>
       <c r="AH268" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="269" spans="1:34" x14ac:dyDescent="0.25">
@@ -44377,7 +44377,7 @@
         <v>13</v>
       </c>
       <c r="AH269" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="270" spans="1:34" x14ac:dyDescent="0.25">
@@ -44481,7 +44481,7 @@
         <v>13</v>
       </c>
       <c r="AH270" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="271" spans="1:34" x14ac:dyDescent="0.25">
@@ -44585,7 +44585,7 @@
         <v>13</v>
       </c>
       <c r="AH271" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="272" spans="1:34" x14ac:dyDescent="0.25">
@@ -44596,7 +44596,7 @@
         <v>3496</v>
       </c>
       <c r="C272" s="2">
-        <v>15931356</v>
+        <v>11243330</v>
       </c>
       <c r="D272" s="1" t="s">
         <v>531</v>
@@ -44689,7 +44689,7 @@
         <v>13</v>
       </c>
       <c r="AH272" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="273" spans="1:34" x14ac:dyDescent="0.25">
@@ -44793,7 +44793,7 @@
         <v>13</v>
       </c>
       <c r="AH273" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="274" spans="1:34" x14ac:dyDescent="0.25">
@@ -44897,7 +44897,7 @@
         <v>13</v>
       </c>
       <c r="AH274" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="275" spans="1:34" x14ac:dyDescent="0.25">
@@ -45001,7 +45001,7 @@
         <v>13</v>
       </c>
       <c r="AH275" s="6">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="276" spans="1:34" x14ac:dyDescent="0.25">
@@ -45105,7 +45105,7 @@
         <v>13</v>
       </c>
       <c r="AH276" s="5">
-        <v>46264.333344907405</v>
+        <v>46265.381678240738</v>
       </c>
     </row>
     <row r="277" spans="1:34" x14ac:dyDescent="0.25">
@@ -45209,7 +45209,7 @@
         <v>13</v>
       </c>
       <c r="AH277" s="6">
-        <v>46264.333344907405</v>
+      